<commit_message>
Harden employee portal for Monday assessment readiness.
Add EIR/NDS tests, assessment-only lock, optional camera/fullscreen, 5-strike proctoring, video naming/reset cleanup, idle-logout disable on live tests, and admin UX fixes.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Resource_Question_Mapping.xlsx
+++ b/Resource_Question_Mapping.xlsx
@@ -754,7 +754,6 @@
           <t>[HSS Troubleshooting] The healthCheck.log shows isRtpReadinessOK: False. Which command should be used next to check RTP-based process status?</t>
         </is>
       </c>
-      <c r="AH2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -922,7 +921,6 @@
           <t>[HSS Troubleshooting] An operator runs kubectl get pod -n hss and notices one pod shows 2/3 Running in the Ready column. What does this indicate?</t>
         </is>
       </c>
-      <c r="AH3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1090,7 +1088,6 @@
           <t>[HSS Deployment] After deploying Nokia HSS CNF through NCOM, the engineer must confirm whether all pods are running in the target namespace. Which command should be used?</t>
         </is>
       </c>
-      <c r="AH4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1258,7 +1255,6 @@
           <t>[UDM Planning] Planning for LLB failover requires historical CFR statistics on each connection to influence PG server selection. What is this called?</t>
         </is>
       </c>
-      <c r="AH5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1426,7 +1422,6 @@
           <t>[Deployment &amp; Troubleshooting] If all HTTP/2 LB Pods run into Http/2 egress connection failure simultaneously, what happens at the NRF level?</t>
         </is>
       </c>
-      <c r="AH6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1594,7 +1589,6 @@
           <t>[HSS Basics] An MME requests authentication vectors for a subscriber attempting to attach to the LTE network. Which service generates these vectors?</t>
         </is>
       </c>
-      <c r="AH7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1762,7 +1756,6 @@
           <t>[UDM Basic] A subscriber roams to another PLMN and the HPLMN needs to securely deliver a preferred PLMN list. Which service secures this SoR data?</t>
         </is>
       </c>
-      <c r="AH8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1930,7 +1923,6 @@
           <t>[Deployment &amp; Troubleshooting] A troubleshooting engineer notices Pods with unusually high error rates and wants automatic isolation and recovery. Which feature addresses this?</t>
         </is>
       </c>
-      <c r="AH9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2098,7 +2090,6 @@
           <t>[Deployment &amp; Troubleshooting] Before running Netconf rpc commands to configure the CDS threshold, what tool must be installed on the operator's machine?</t>
         </is>
       </c>
-      <c r="AH10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2266,7 +2257,6 @@
           <t>[HSS Basics] The operations team notices failures in SS7 message routing toward HLR processing nodes. Which service should be investigated first?</t>
         </is>
       </c>
-      <c r="AH11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2434,7 +2424,6 @@
           <t>[UDM Basic] AUSF NF wants to retrieve authentication data from UDM. Which interface should be used?</t>
         </is>
       </c>
-      <c r="AH12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2602,7 +2591,6 @@
           <t>[HSS Troubleshooting] An engineer wants to verify SCTP connection status for SS7. Which command is recommended instead of relying on netstat?</t>
         </is>
       </c>
-      <c r="AH13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2770,7 +2758,6 @@
           <t>[Deployment &amp; Troubleshooting] When the HTTP/2 LB Pod detects an egress connection failure, where is the failure file written?</t>
         </is>
       </c>
-      <c r="AH14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2938,7 +2925,6 @@
           <t>[UDM Basic] A SUCI needs to be de-concealed to a SUPI. Which service performs this function?</t>
         </is>
       </c>
-      <c r="AH15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3106,7 +3092,6 @@
           <t>[Deployment &amp; Troubleshooting] The NIM leader Pod goes down unexpectedly. What happens to NRF interfacing during the leader re-election?</t>
         </is>
       </c>
-      <c r="AH16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3274,7 +3259,6 @@
           <t>[HSS Deployment] The SS7 pod fails to apply the Telesys license. The license file is named M7-KEY-demo.tar.gz, but the configured VNF ID is hlrcn. What should be checked first?</t>
         </is>
       </c>
-      <c r="AH17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3442,7 +3426,6 @@
           <t>[HSS Troubleshooting] The healthCheck.log shows isRtpReadinessOK: False. Which command should be used next to check RTP-based process status?</t>
         </is>
       </c>
-      <c r="AH18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3610,7 +3593,6 @@
           <t>[HSS Deployment] A deployment engineer is planning external networks for Diameter, LDAP, Trigger, and SS7 pods. Which component is responsible for assigning external network IPs to pods?</t>
         </is>
       </c>
-      <c r="AH19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3778,7 +3760,6 @@
           <t>[Deployment &amp; Troubleshooting] A troubleshooting engineer needs to inspect event logs captured inside the OAM container for a specific service. Which log should be checked?</t>
         </is>
       </c>
-      <c r="AH20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3946,7 +3927,6 @@
           <t>[HSS Basics] Several CNF services cannot locate each other after a cluster restart. Which component provides internal service discovery?</t>
         </is>
       </c>
-      <c r="AH21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4114,7 +4094,6 @@
           <t>[HSS Basics] A telecom operator observes that one HSS-CP instance is overloaded while others remain idle. Which service should be verified to ensure traffic is evenly distributed across all HSS-CP instances?</t>
         </is>
       </c>
-      <c r="AH22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4282,7 +4261,6 @@
           <t>[UDM Planning] The security team wants CSR to be handled with an integrated External rootCA when External CA is enabled. Which mechanism supports this?</t>
         </is>
       </c>
-      <c r="AH23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -4450,7 +4428,6 @@
           <t>[HSS Troubleshooting] NCOM reports: No valid repository configured or found for CaaS. What should be done?</t>
         </is>
       </c>
-      <c r="AH24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4618,7 +4595,6 @@
           <t>[HSS Basics] During IMS registration, communication is required between the HSS and the S-CSCF. Which interface supports this communication?</t>
         </is>
       </c>
-      <c r="AH25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4786,11 +4762,6 @@
           <t>[EIR Planning] What is the main focus of the CIQ document, as distinct from the DNP?</t>
         </is>
       </c>
-      <c r="AH26" t="inlineStr">
-        <is>
-          <t>No question bank mapping for product 'EIR'.</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4958,7 +4929,6 @@
           <t>[HSS Basics] A PCRF needs to store and retrieve subscriber policy-related data from HSS. Which interface should be used?</t>
         </is>
       </c>
-      <c r="AH27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -5126,7 +5096,6 @@
           <t>[HSS Basics] Before delivering an SMS to a subscriber, an SMSC needs routing information from HSS. Which interface is used?</t>
         </is>
       </c>
-      <c r="AH28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -5294,7 +5263,6 @@
           <t>[HSS Troubleshooting] A pod registration check shows envoy status: false. What does this indicate?</t>
         </is>
       </c>
-      <c r="AH29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -5462,7 +5430,6 @@
           <t>[UDM Planning] Planning an in-service software upgrade, the team wants automated pre- and post-upgrade validation. Which mechanism is used for CNF health checks in this feature?</t>
         </is>
       </c>
-      <c r="AH30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -5630,7 +5597,6 @@
           <t>[Basic SDL] A customer wants to move from traditional VNF architecture to cloud-native deployment. Which SDL architecture supports this model?</t>
         </is>
       </c>
-      <c r="AH31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -5798,7 +5764,6 @@
           <t>[Deployment &amp; Troubleshooting] Filesystem utilization alarms are generated. Which command provides disk usage information?</t>
         </is>
       </c>
-      <c r="AH32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -5966,7 +5931,6 @@
           <t>[Basic SDL] A customer wants to move from traditional VNF architecture to cloud-native deployment. Which SDL architecture supports this model?</t>
         </is>
       </c>
-      <c r="AH33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -6134,7 +6098,6 @@
           <t>[Deployment &amp; Troubleshooting] Post deployment where can we check our VM status?</t>
         </is>
       </c>
-      <c r="AH34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -6302,11 +6265,6 @@
           <t>[Basic NDS] An L2 engineer is performing root cause analysis after repeated service outages. Which VM provides diagnostic tools and health checks?</t>
         </is>
       </c>
-      <c r="AH35" t="inlineStr">
-        <is>
-          <t>No question bank mapping for product 'NDS'.</t>
-        </is>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -6474,7 +6432,6 @@
           <t>[Basic SDL] An engineer needs to manage SDL lifecycle operations such as scaling and upgrades. Which VM provides these capabilities?</t>
         </is>
       </c>
-      <c r="AH36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -6642,7 +6599,6 @@
           <t>[Basic SDL] An L2 engineer is performing root cause analysis after repeated service outages. Which VM provides diagnostic tools and health checks?</t>
         </is>
       </c>
-      <c r="AH37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -6810,7 +6766,6 @@
           <t>[Basic SDL] A customer migration project specifically requires synchronization between legacy and SDL databases. Which VM is mandatory?</t>
         </is>
       </c>
-      <c r="AH38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -6978,7 +6933,6 @@
           <t>[Planning &amp; Artifact Preparation] Which document provides the detailed customer network information used for design preparation?</t>
         </is>
       </c>
-      <c r="AH39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -7146,7 +7100,6 @@
           <t>[Planning &amp; Artifact Preparation] Incorrect sizing information mainly impacts which area?</t>
         </is>
       </c>
-      <c r="AH40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -7314,7 +7267,6 @@
           <t>[Deployment &amp; Troubleshooting] SDL instantiation has completed, but verification is required. What should the output show?</t>
         </is>
       </c>
-      <c r="AH41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -7482,7 +7434,6 @@
           <t>[Basic SDL] A storage node failure occurs. Which SDL component is responsible for data durability and recovery?</t>
         </is>
       </c>
-      <c r="AH42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -7650,7 +7601,6 @@
           <t>[Planning &amp; Artifact Preparation] Why is CIQ important for SDL deployment?</t>
         </is>
       </c>
-      <c r="AH43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -7818,7 +7768,6 @@
           <t>[Planning &amp; Artifact Preparation] A customer updates network architecture after the design has been finalized. Which documents may require updates?</t>
         </is>
       </c>
-      <c r="AH44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -7986,7 +7935,6 @@
           <t>[Basic SDL] NetAct is not receiving PM/FM statistics although subscriber operations are functioning normally. Which VM should be checked?</t>
         </is>
       </c>
-      <c r="AH45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -8154,7 +8102,6 @@
           <t>[Deployment &amp; Troubleshooting] Filesystem utilization alarms are generated. Which command provides disk usage information?</t>
         </is>
       </c>
-      <c r="AH46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -8322,7 +8269,6 @@
           <t>[Deployment &amp; Troubleshooting] Several components appear in UNKNOWN state. Which information source should be checked first?</t>
         </is>
       </c>
-      <c r="AH47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -8490,7 +8436,6 @@
           <t>[Deployment &amp; Troubleshooting] Replication alarms are reported on Storage VMs. Which command should be checked first?</t>
         </is>
       </c>
-      <c r="AH48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -8658,7 +8603,6 @@
           <t>[Planning &amp; Artifact Preparation] The customer changes interface VLANs after DND approval. What action is required?</t>
         </is>
       </c>
-      <c r="AH49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -8826,11 +8770,6 @@
           <t>[Planning &amp; Artifact Preparation] The customer provided an incomplete network design sheet without VLAN details. Which document should be revisited first?</t>
         </is>
       </c>
-      <c r="AH50" t="inlineStr">
-        <is>
-          <t>No question bank mapping for product 'NDS'.</t>
-        </is>
-      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -8998,7 +8937,6 @@
           <t>[Deployment &amp; Troubleshooting] A complete health assessment of SDL is required. Which command should be executed?</t>
         </is>
       </c>
-      <c r="AH51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -9166,7 +9104,6 @@
           <t>[Deployment &amp; Troubleshooting] After deployment, an engineer wants to verify that SDL services are running on all VMs. Which command should be used?</t>
         </is>
       </c>
-      <c r="AH52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -9334,7 +9271,6 @@
           <t>[Basic SDL] An L2 engineer is performing root cause analysis after repeated service outages. Which VM provides diagnostic tools and health checks?</t>
         </is>
       </c>
-      <c r="AH53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -9502,7 +9438,6 @@
           <t>[HSS Basics] An external system needs access to subscriber information stored in One-NDS/SDL while hiding internal business logic services. Which component should be used?</t>
         </is>
       </c>
-      <c r="AH54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -9670,7 +9605,6 @@
           <t>[Basic SDL] A storage node failure occurs. Which SDL component is responsible for data durability and recovery?</t>
         </is>
       </c>
-      <c r="AH55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -9838,7 +9772,6 @@
           <t>[Basic SDL] During a capacity planning workshop, the customer expects subscriber growth to double within a year. Which SDL components are typically scaled to handle increased load?</t>
         </is>
       </c>
-      <c r="AH56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -10006,7 +9939,6 @@
           <t>[Deployment &amp; Troubleshooting] SDL bootstrap is suspected to be stuck. Which script should be executed?</t>
         </is>
       </c>
-      <c r="AH57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -10174,7 +10106,6 @@
           <t>[Deployment &amp; Troubleshooting] After running a health check report, what should ideally be displayed?</t>
         </is>
       </c>
-      <c r="AH58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -10342,7 +10273,6 @@
           <t>[UDM Planning] A deployment requires direct NF-to-NF communication without depending on NRF or SCP availability. Which model should be planned for this requirement?</t>
         </is>
       </c>
-      <c r="AH59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -10510,7 +10440,6 @@
           <t>[HSS Basics] The CNF must communicate with management systems through ZTS services instead of directly connecting to EMS/NMS. Which service supports this integration?</t>
         </is>
       </c>
-      <c r="AH60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -10678,7 +10607,6 @@
           <t>[UDM Planning] A planning discussion on rolling upgrades and node draining introduces a function that guarantees a minimum number of available Pods. What is this called?</t>
         </is>
       </c>
-      <c r="AH61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -10846,11 +10774,6 @@
           <t>[EIR Basic] Besides reducing IP requirements, which additional benefit does the centralized HTTP/2 LB provide?</t>
         </is>
       </c>
-      <c r="AH62" t="inlineStr">
-        <is>
-          <t>No question bank mapping for product 'EIR'.</t>
-        </is>
-      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -11018,7 +10941,6 @@
           <t>[UDM Basic] A design review lists 5G core NFs. Which pair correctly represents AUSF_UDM's supported network functions?</t>
         </is>
       </c>
-      <c r="AH63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -11186,7 +11108,6 @@
           <t>[UDM Basic] Which service generates Authentication vectors for AKA based authentications and also supports Ki re-encryption?</t>
         </is>
       </c>
-      <c r="AH64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -11354,11 +11275,7 @@
           <t>[Deployment &amp; Troubleshooting] A customer reports that connectivity from the One-EIR Application towards the backend on port 16611 is not established. What is the first troubleshooting step?</t>
         </is>
       </c>
-      <c r="AH65" t="inlineStr">
-        <is>
-          <t>No question bank mapping for product 'EIR'.</t>
-        </is>
-      </c>
+      <c r="AH65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -11526,7 +11443,6 @@
           <t>[UDM Planning] A capacity design session covers cluster node types used by AUSF_UDM on NCS. Which node types are used?</t>
         </is>
       </c>
-      <c r="AH66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -11694,7 +11610,6 @@
           <t>[UDM Planning] A security planning session discusses which Kubernetes-level policy objects define security conditions for Pods.</t>
         </is>
       </c>
-      <c r="AH67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -11862,7 +11777,6 @@
           <t>[HSS Troubleshooting] The SS7 Telesys process is down. What should be checked first?</t>
         </is>
       </c>
-      <c r="AH68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -12030,7 +11944,6 @@
           <t>[HSS Basics] Several CNF services cannot locate each other after a cluster restart. Which component provides internal service discovery?</t>
         </is>
       </c>
-      <c r="AH69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -12198,7 +12111,6 @@
           <t>[HSS Troubleshooting] A pod is stuck in ImagePullBackOff or ErrImagePull. What is the recommended corrective action?</t>
         </is>
       </c>
-      <c r="AH70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -12366,7 +12278,6 @@
           <t>[Deployment &amp; Troubleshooting] An autoscaling design uses HPA with which primary metric to trigger scale-out or scale-in decisions?</t>
         </is>
       </c>
-      <c r="AH71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -12534,7 +12445,6 @@
           <t>[Deployment &amp; Troubleshooting] Traffic is still being routed to a Pod that is not actually ready to serve requests. Which probe should be checked to correct this?</t>
         </is>
       </c>
-      <c r="AH72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -12702,7 +12612,6 @@
           <t>[HSS Basics] A 5G core deployment requires interworking between a UDM and HSS. Which proprietary Diameter interface supports this requirement?</t>
         </is>
       </c>
-      <c r="AH73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -12870,7 +12779,6 @@
           <t>[UDM Basic] SMS Function needs to register its address and retrieve SMS management subscription data from UDM. Which interface is used?</t>
         </is>
       </c>
-      <c r="AH74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -13038,7 +12946,6 @@
           <t>[Deployment &amp; Troubleshooting] A process heap size configuration file defines thresholds like HEAP_SIZE_CRITICAL and HEAP_SIZE_MAJOR. What action is taken if a process exceeds the critical threshold?</t>
         </is>
       </c>
-      <c r="AH75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -13206,7 +13113,6 @@
           <t>[HSS Troubleshooting] A pod registration check shows envoy status: false. What does this indicate?</t>
         </is>
       </c>
-      <c r="AH76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -13374,7 +13280,6 @@
           <t>[HSS Deployment] The operator wants to run CNF health checks using Helm test or NCOM GUI. Which parameter should be enabled?</t>
         </is>
       </c>
-      <c r="AH77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -13542,7 +13447,6 @@
           <t>[HSS Troubleshooting] A pod registration check shows envoy status: false. What does this indicate?</t>
         </is>
       </c>
-      <c r="AH78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -13710,7 +13614,6 @@
           <t>[HSS Basics] A 5G core deployment requires interworking between a UDM and HSS. Which proprietary Diameter interface supports this requirement?</t>
         </is>
       </c>
-      <c r="AH79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -13878,7 +13781,6 @@
           <t>[HSS Troubleshooting] The HLRCallP pod continuously raises a No Free Dialogue alarm for a DP process. What is the recommended recovery action?</t>
         </is>
       </c>
-      <c r="AH80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -14046,7 +13948,6 @@
           <t>[HSS Troubleshooting] NCOM reports: No valid repository configured or found for CaaS. What should be done?</t>
         </is>
       </c>
-      <c r="AH81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -14214,7 +14115,6 @@
           <t>[Deployment &amp; Troubleshooting] After running a health check report, what should ideally be displayed?</t>
         </is>
       </c>
-      <c r="AH82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -14227,7 +14127,6 @@
           <t>Sanjay Kumar Gupta</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr"/>
       <c r="D83" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -14378,7 +14277,6 @@
           <t>Attach ok but PDN fails. Check?</t>
         </is>
       </c>
-      <c r="AH83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -14391,7 +14289,6 @@
           <t>Bharanidharan</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr"/>
       <c r="D84" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -14542,7 +14439,6 @@
           <t>Purpose of S1-AP on S1-MME?</t>
         </is>
       </c>
-      <c r="AH84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -14555,7 +14451,6 @@
           <t>J Mohammed Sheik Afridi</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr"/>
       <c r="D85" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -14706,7 +14601,6 @@
           <t>Attach ok but PDN fails. Check?</t>
         </is>
       </c>
-      <c r="AH85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -14719,7 +14613,6 @@
           <t>Divyanshu Chauhan</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr"/>
       <c r="D86" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -14870,7 +14763,6 @@
           <t>What is a major functional benefit of CMG in packet core?</t>
         </is>
       </c>
-      <c r="AH86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -14883,7 +14775,6 @@
           <t>Chitrangada Mishra</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr"/>
       <c r="D87" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -15034,7 +14925,6 @@
           <t>In 4G LTE, CMM most commonly provides which network function?</t>
         </is>
       </c>
-      <c r="AH87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -15047,7 +14937,6 @@
           <t>Vibhor Chandra Gupta</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr"/>
       <c r="D88" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -15198,7 +15087,6 @@
           <t>Which CMM component is responsible for OAM functions and northbound interfaces?</t>
         </is>
       </c>
-      <c r="AH88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -15211,7 +15099,6 @@
           <t>Nishu Kumar</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr"/>
       <c r="D89" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -15362,7 +15249,6 @@
           <t>Which technology is highlighted in CMM for performance optimization on x86 platforms?</t>
         </is>
       </c>
-      <c r="AH89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -15375,7 +15261,6 @@
           <t>Satheeshkumar</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr"/>
       <c r="D90" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -15526,7 +15411,6 @@
           <t>In a 4G ATP scenario, what does successful bearer establishment mainly confirm?</t>
         </is>
       </c>
-      <c r="AH90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -15539,7 +15423,6 @@
           <t>Chandan Kumar Singh</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr"/>
       <c r="D91" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -15690,7 +15573,6 @@
           <t>What is a major functional benefit of CMG in packet core?</t>
         </is>
       </c>
-      <c r="AH91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -15703,7 +15585,6 @@
           <t>Sourabh  Khandelwal</t>
         </is>
       </c>
-      <c r="C92" t="inlineStr"/>
       <c r="D92" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -15854,7 +15735,6 @@
           <t>CMG is best described as:</t>
         </is>
       </c>
-      <c r="AH92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -15867,7 +15747,6 @@
           <t>Prateek</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr"/>
       <c r="D93" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -16018,7 +15897,6 @@
           <t>CMM is described by Nokia as having what kind of architecture?</t>
         </is>
       </c>
-      <c r="AH93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -16031,7 +15909,6 @@
           <t>Veerasami</t>
         </is>
       </c>
-      <c r="C94" t="inlineStr"/>
       <c r="D94" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -16182,7 +16059,6 @@
           <t>In 4G LTE, CMM most commonly provides which network function?</t>
         </is>
       </c>
-      <c r="AH94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -16195,7 +16071,6 @@
           <t>Parth Saxena</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr"/>
       <c r="D95" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -16346,7 +16221,6 @@
           <t>CMG supports evolution toward which major core direction?</t>
         </is>
       </c>
-      <c r="AH95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -16359,7 +16233,6 @@
           <t>Satya Prakash Rai</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr"/>
       <c r="D96" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -16510,7 +16383,6 @@
           <t>Purpose of S1-AP on S1-MME?</t>
         </is>
       </c>
-      <c r="AH96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -16523,7 +16395,6 @@
           <t>Meenatchi M</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr"/>
       <c r="D97" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -16674,7 +16545,6 @@
           <t>Which network function is most directly linked to slice selection in NRD-related architecture?</t>
         </is>
       </c>
-      <c r="AH97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -16687,7 +16557,6 @@
           <t>Sunilkumaar Selvaraajan</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr"/>
       <c r="D98" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -16838,7 +16707,6 @@
           <t>What is the primary purpose of Nokia Resource Director (NRD)?</t>
         </is>
       </c>
-      <c r="AH98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -16851,7 +16719,6 @@
           <t>Ashwini Raju</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr"/>
       <c r="D99" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -17002,7 +16869,6 @@
           <t>Which deployment characteristic is strongly associated with CMG?</t>
         </is>
       </c>
-      <c r="AH99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -17015,7 +16881,6 @@
           <t>Sunil Kumar Patel</t>
         </is>
       </c>
-      <c r="C100" t="inlineStr"/>
       <c r="D100" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -17166,7 +17031,6 @@
           <t>Which deployment characteristic is strongly associated with CMG?</t>
         </is>
       </c>
-      <c r="AH100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -17179,7 +17043,6 @@
           <t>Naveenkumar</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr"/>
       <c r="D101" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -17330,7 +17193,6 @@
           <t>What is a major functional benefit of CMG in packet core?</t>
         </is>
       </c>
-      <c r="AH101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -17343,7 +17205,6 @@
           <t>G  Koushik</t>
         </is>
       </c>
-      <c r="C102" t="inlineStr"/>
       <c r="D102" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -17494,7 +17355,6 @@
           <t>CMM is described by Nokia as having what kind of architecture?</t>
         </is>
       </c>
-      <c r="AH102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -17507,7 +17367,6 @@
           <t>Kapil Chaudhary</t>
         </is>
       </c>
-      <c r="C103" t="inlineStr"/>
       <c r="D103" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -17658,7 +17517,6 @@
           <t>Successful ATP indication?</t>
         </is>
       </c>
-      <c r="AH103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -17671,7 +17529,6 @@
           <t>Aryan Kumar</t>
         </is>
       </c>
-      <c r="C104" t="inlineStr"/>
       <c r="D104" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -17822,7 +17679,6 @@
           <t>CMG supports evolution toward which major core direction?</t>
         </is>
       </c>
-      <c r="AH104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -17835,7 +17691,6 @@
           <t>Pratik Raj</t>
         </is>
       </c>
-      <c r="C105" t="inlineStr"/>
       <c r="D105" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -17986,7 +17841,6 @@
           <t>Which ATP case is useful for validating CMG resilience?</t>
         </is>
       </c>
-      <c r="AH105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -17999,7 +17853,6 @@
           <t>Ezhilarasan</t>
         </is>
       </c>
-      <c r="C106" t="inlineStr"/>
       <c r="D106" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -18150,7 +18003,6 @@
           <t>Which protocols relate to CMM control plane?</t>
         </is>
       </c>
-      <c r="AH106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -18163,7 +18015,6 @@
           <t>Santosh Kumar</t>
         </is>
       </c>
-      <c r="C107" t="inlineStr"/>
       <c r="D107" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -18314,7 +18165,6 @@
           <t>CMG is best described as:</t>
         </is>
       </c>
-      <c r="AH107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -18327,7 +18177,6 @@
           <t>Srinath</t>
         </is>
       </c>
-      <c r="C108" t="inlineStr"/>
       <c r="D108" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -18478,7 +18327,6 @@
           <t>Which interface is key for LTE access during ATP?</t>
         </is>
       </c>
-      <c r="AH108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -18491,7 +18339,6 @@
           <t>Kiruthika V</t>
         </is>
       </c>
-      <c r="C109" t="inlineStr"/>
       <c r="D109" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -18642,7 +18489,6 @@
           <t>Which ATP case is useful for validating CMG resilience?</t>
         </is>
       </c>
-      <c r="AH109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -18655,7 +18501,6 @@
           <t>Pratyasa Mohanty</t>
         </is>
       </c>
-      <c r="C110" t="inlineStr"/>
       <c r="D110" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -18806,7 +18651,6 @@
           <t>Which Nokia platform is commonly used for CMM management?</t>
         </is>
       </c>
-      <c r="AH110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -18819,7 +18663,6 @@
           <t>Soumya Smruti Das</t>
         </is>
       </c>
-      <c r="C111" t="inlineStr"/>
       <c r="D111" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -18970,7 +18813,6 @@
           <t>Which outcome indicates a successful CMG onboarding and integration cycle?</t>
         </is>
       </c>
-      <c r="AH111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -18983,7 +18825,6 @@
           <t>Pratyusha Pattanaik</t>
         </is>
       </c>
-      <c r="C112" t="inlineStr"/>
       <c r="D112" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -19134,7 +18975,6 @@
           <t>Which CMM component provides logical interface termination for GTP and Diameter?</t>
         </is>
       </c>
-      <c r="AH112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -19147,7 +18987,6 @@
           <t>Ashutosh</t>
         </is>
       </c>
-      <c r="C113" t="inlineStr"/>
       <c r="D113" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -19298,7 +19137,6 @@
           <t>Which technology is highlighted in CMM for performance optimization on x86 platforms?</t>
         </is>
       </c>
-      <c r="AH113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -19311,7 +19149,6 @@
           <t>Gudluru Lakshmi Narayan</t>
         </is>
       </c>
-      <c r="C114" t="inlineStr"/>
       <c r="D114" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -19462,7 +19299,6 @@
           <t>CMG is best described as:</t>
         </is>
       </c>
-      <c r="AH114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -19475,7 +19311,6 @@
           <t>Madanuru Vishnu Charan</t>
         </is>
       </c>
-      <c r="C115" t="inlineStr"/>
       <c r="D115" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -19626,7 +19461,6 @@
           <t>What is critical to validate for mobility in ATP?</t>
         </is>
       </c>
-      <c r="AH115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -19639,7 +19473,6 @@
           <t>Abhisek Mohanty</t>
         </is>
       </c>
-      <c r="C116" t="inlineStr"/>
       <c r="D116" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -19790,7 +19623,6 @@
           <t>In 4G LTE, CMM most commonly provides which network function?</t>
         </is>
       </c>
-      <c r="AH116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -19803,7 +19635,6 @@
           <t>Avipsa Mohanty</t>
         </is>
       </c>
-      <c r="C117" t="inlineStr"/>
       <c r="D117" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -19954,7 +19785,6 @@
           <t>What is the primary role of Nokia Cloud Mobility Manager (CMM) in a 4G packet core?</t>
         </is>
       </c>
-      <c r="AH117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -19967,7 +19797,6 @@
           <t>Debasish Jena</t>
         </is>
       </c>
-      <c r="C118" t="inlineStr"/>
       <c r="D118" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -20118,7 +19947,6 @@
           <t>Which protocols relate to CMM control plane?</t>
         </is>
       </c>
-      <c r="AH118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -20131,7 +19959,6 @@
           <t>PRITISARATHI BHUYAN</t>
         </is>
       </c>
-      <c r="C119" t="inlineStr"/>
       <c r="D119" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -20282,7 +20109,6 @@
           <t>Best failover ATP test?</t>
         </is>
       </c>
-      <c r="AH119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -20295,7 +20121,6 @@
           <t>Anchal Priyadarshini Swain</t>
         </is>
       </c>
-      <c r="C120" t="inlineStr"/>
       <c r="D120" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -20446,7 +20271,6 @@
           <t>CMG is part of which Nokia family?</t>
         </is>
       </c>
-      <c r="AH120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -20459,7 +20283,6 @@
           <t>Sasmita GIRI</t>
         </is>
       </c>
-      <c r="C121" t="inlineStr"/>
       <c r="D121" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -20610,7 +20433,6 @@
           <t>Which protocols relate to CMM control plane?</t>
         </is>
       </c>
-      <c r="AH121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -20623,7 +20445,6 @@
           <t>Akankshya Rout</t>
         </is>
       </c>
-      <c r="C122" t="inlineStr"/>
       <c r="D122" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -20774,7 +20595,6 @@
           <t>What does NECC stand for in Nokia CMM architecture?</t>
         </is>
       </c>
-      <c r="AH122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -20787,7 +20607,6 @@
           <t>Ajaya Narayan Nayak</t>
         </is>
       </c>
-      <c r="C123" t="inlineStr"/>
       <c r="D123" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -20938,7 +20757,6 @@
           <t>Purpose of S1-AP on S1-MME?</t>
         </is>
       </c>
-      <c r="AH123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -20951,7 +20769,6 @@
           <t>Soumya Ranjan Das</t>
         </is>
       </c>
-      <c r="C124" t="inlineStr"/>
       <c r="D124" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -21102,7 +20919,6 @@
           <t>Purpose of S1-AP on S1-MME?</t>
         </is>
       </c>
-      <c r="AH124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -21115,7 +20931,6 @@
           <t>Vaghela Rahul Rameshbhai</t>
         </is>
       </c>
-      <c r="C125" t="inlineStr"/>
       <c r="D125" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -21266,7 +21081,6 @@
           <t>CMG is best described as:</t>
         </is>
       </c>
-      <c r="AH125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -21279,7 +21093,6 @@
           <t>Asish Nayak</t>
         </is>
       </c>
-      <c r="C126" t="inlineStr"/>
       <c r="D126" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -21430,7 +21243,6 @@
           <t>What is a major functional benefit of CMG in packet core?</t>
         </is>
       </c>
-      <c r="AH126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -21443,7 +21255,6 @@
           <t>Bibhash Dash</t>
         </is>
       </c>
-      <c r="C127" t="inlineStr"/>
       <c r="D127" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -21594,7 +21405,6 @@
           <t>CMM is described by Nokia as having what kind of architecture?</t>
         </is>
       </c>
-      <c r="AH127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -21607,7 +21417,6 @@
           <t>Omm  Sai Roumya RANJAN</t>
         </is>
       </c>
-      <c r="C128" t="inlineStr"/>
       <c r="D128" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -21758,7 +21567,6 @@
           <t>Which aspect is most important during CMG onboarding?</t>
         </is>
       </c>
-      <c r="AH128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -21771,7 +21579,6 @@
           <t>Pradyumna Naik</t>
         </is>
       </c>
-      <c r="C129" t="inlineStr"/>
       <c r="D129" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -21922,7 +21729,6 @@
           <t>CMG is part of which Nokia family?</t>
         </is>
       </c>
-      <c r="AH129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -21935,7 +21741,6 @@
           <t>Abdul Basith Shaik</t>
         </is>
       </c>
-      <c r="C130" t="inlineStr"/>
       <c r="D130" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -22086,7 +21891,6 @@
           <t>Attach succeeds but bearer fails. Likely issue?</t>
         </is>
       </c>
-      <c r="AH130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -22099,7 +21903,6 @@
           <t>Solanki Jigar Ambalal</t>
         </is>
       </c>
-      <c r="C131" t="inlineStr"/>
       <c r="D131" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -22250,7 +22053,6 @@
           <t>Attach ok but PDN fails. Check?</t>
         </is>
       </c>
-      <c r="AH131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -22263,7 +22065,6 @@
           <t>Akash Bairagi</t>
         </is>
       </c>
-      <c r="C132" t="inlineStr"/>
       <c r="D132" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -22414,7 +22215,6 @@
           <t>In a 4G ATP scenario, what does successful bearer establishment mainly confirm?</t>
         </is>
       </c>
-      <c r="AH132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -22427,7 +22227,6 @@
           <t>Anand Babu</t>
         </is>
       </c>
-      <c r="C133" t="inlineStr"/>
       <c r="D133" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -22578,7 +22377,6 @@
           <t>Which protocols relate to CMM control plane?</t>
         </is>
       </c>
-      <c r="AH133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -22591,7 +22389,6 @@
           <t>Chelsea Shalin S</t>
         </is>
       </c>
-      <c r="C134" t="inlineStr"/>
       <c r="D134" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -22742,7 +22539,6 @@
           <t>CMM supports which management interfaces for operations and troubleshooting?</t>
         </is>
       </c>
-      <c r="AH134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -22755,7 +22551,6 @@
           <t>Gopi K</t>
         </is>
       </c>
-      <c r="C135" t="inlineStr"/>
       <c r="D135" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -22906,7 +22701,6 @@
           <t>Purpose of S1-AP on S1-MME?</t>
         </is>
       </c>
-      <c r="AH135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -22919,7 +22713,6 @@
           <t>Malan Subbiah Pandian</t>
         </is>
       </c>
-      <c r="C136" t="inlineStr"/>
       <c r="D136" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -23070,7 +22863,6 @@
           <t>Which is a common integration point for CMG in EPC?</t>
         </is>
       </c>
-      <c r="AH136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -23083,7 +22875,6 @@
           <t>R Krishna Durga</t>
         </is>
       </c>
-      <c r="C137" t="inlineStr"/>
       <c r="D137" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -23234,7 +23025,6 @@
           <t>Purpose of S1-AP on S1-MME?</t>
         </is>
       </c>
-      <c r="AH137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -23247,7 +23037,6 @@
           <t>Sabari Murugesan</t>
         </is>
       </c>
-      <c r="C138" t="inlineStr"/>
       <c r="D138" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -23398,7 +23187,6 @@
           <t>CMM is described by Nokia as having what kind of architecture?</t>
         </is>
       </c>
-      <c r="AH138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -23411,7 +23199,6 @@
           <t>Surya Saravanan</t>
         </is>
       </c>
-      <c r="C139" t="inlineStr"/>
       <c r="D139" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -23562,7 +23349,6 @@
           <t>What is the key purpose of ATP testing for CMG?</t>
         </is>
       </c>
-      <c r="AH139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -23575,7 +23361,6 @@
           <t>Yogaverma V</t>
         </is>
       </c>
-      <c r="C140" t="inlineStr"/>
       <c r="D140" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -23726,7 +23511,6 @@
           <t>Which scenario best tests CMG under mobility conditions?</t>
         </is>
       </c>
-      <c r="AH140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -23739,7 +23523,6 @@
           <t>Varun Pachauri</t>
         </is>
       </c>
-      <c r="C141" t="inlineStr"/>
       <c r="D141" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -23890,7 +23673,6 @@
           <t>CMG supports evolution toward which major core direction?</t>
         </is>
       </c>
-      <c r="AH141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -23903,7 +23685,6 @@
           <t>Buran Sagari Sohail Basha</t>
         </is>
       </c>
-      <c r="C142" t="inlineStr"/>
       <c r="D142" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -24054,7 +23835,6 @@
           <t>Which protocols relate to CMM control plane?</t>
         </is>
       </c>
-      <c r="AH142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -24067,7 +23847,6 @@
           <t>Gadde Yaswanth</t>
         </is>
       </c>
-      <c r="C143" t="inlineStr"/>
       <c r="D143" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -24218,7 +23997,6 @@
           <t>Which Nokia platform is commonly used for CMM management?</t>
         </is>
       </c>
-      <c r="AH143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -24231,7 +24009,6 @@
           <t>Hariharan S</t>
         </is>
       </c>
-      <c r="C144" t="inlineStr"/>
       <c r="D144" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -24382,7 +24159,6 @@
           <t>What does NECC stand for in Nokia CMM architecture?</t>
         </is>
       </c>
-      <c r="AH144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -24395,7 +24171,6 @@
           <t>M Subramanayam</t>
         </is>
       </c>
-      <c r="C145" t="inlineStr"/>
       <c r="D145" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -24546,7 +24321,6 @@
           <t>CMM supports which management interfaces for operations and troubleshooting?</t>
         </is>
       </c>
-      <c r="AH145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -24559,7 +24333,6 @@
           <t>Nekkanti Mahendra Tulasi</t>
         </is>
       </c>
-      <c r="C146" t="inlineStr"/>
       <c r="D146" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -24710,7 +24483,6 @@
           <t>Which interface is key for LTE access during ATP?</t>
         </is>
       </c>
-      <c r="AH146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -24723,7 +24495,6 @@
           <t>V P Sandhiya</t>
         </is>
       </c>
-      <c r="C147" t="inlineStr"/>
       <c r="D147" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -24874,7 +24645,6 @@
           <t>Key onboarding activity for CMM?</t>
         </is>
       </c>
-      <c r="AH147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -24887,7 +24657,6 @@
           <t>Susheel kumar Dwivdi</t>
         </is>
       </c>
-      <c r="C148" t="inlineStr"/>
       <c r="D148" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -25038,7 +24807,6 @@
           <t>In a CMG ATP plan, which test most directly verifies end-user data service?</t>
         </is>
       </c>
-      <c r="AH148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -25051,7 +24819,6 @@
           <t>Vivek Mishra</t>
         </is>
       </c>
-      <c r="C149" t="inlineStr"/>
       <c r="D149" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -25202,7 +24969,6 @@
           <t>If attach succeeds but data service fails, which CMG area should be checked first?</t>
         </is>
       </c>
-      <c r="AH149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -25215,7 +24981,6 @@
           <t>Harshada Vitthal Shinde</t>
         </is>
       </c>
-      <c r="C150" t="inlineStr"/>
       <c r="D150" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -25366,7 +25131,6 @@
           <t>What is the primary role of Nokia Cloud Mobile Gateway (CMG) in packet core?</t>
         </is>
       </c>
-      <c r="AH150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -25379,7 +25143,6 @@
           <t>Nishant Kumar Lal</t>
         </is>
       </c>
-      <c r="C151" t="inlineStr"/>
       <c r="D151" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -25530,7 +25293,6 @@
           <t>What is critical to validate for mobility in ATP?</t>
         </is>
       </c>
-      <c r="AH151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -25543,7 +25305,6 @@
           <t>Vennela Korada</t>
         </is>
       </c>
-      <c r="C152" t="inlineStr"/>
       <c r="D152" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -25694,7 +25455,6 @@
           <t>In a CMG ATP plan, which test most directly verifies end-user data service?</t>
         </is>
       </c>
-      <c r="AH152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -25707,7 +25467,6 @@
           <t>Bommireddy Jaya Prakash Reddy</t>
         </is>
       </c>
-      <c r="C153" t="inlineStr"/>
       <c r="D153" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -25858,7 +25617,6 @@
           <t>Purpose of S1-AP on S1-MME?</t>
         </is>
       </c>
-      <c r="AH153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -25871,7 +25629,6 @@
           <t>Komala Mamidi</t>
         </is>
       </c>
-      <c r="C154" t="inlineStr"/>
       <c r="D154" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -26022,7 +25779,6 @@
           <t>CMM is described by Nokia as having what kind of architecture?</t>
         </is>
       </c>
-      <c r="AH154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -26035,7 +25791,6 @@
           <t>Sundram Kumar</t>
         </is>
       </c>
-      <c r="C155" t="inlineStr"/>
       <c r="D155" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -26186,7 +25941,6 @@
           <t>Key onboarding activity for CMM?</t>
         </is>
       </c>
-      <c r="AH155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -26199,7 +25953,6 @@
           <t>Abhishikha Chauhan</t>
         </is>
       </c>
-      <c r="C156" t="inlineStr"/>
       <c r="D156" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -26350,7 +26103,6 @@
           <t>Why is CMG considered operationally flexible?</t>
         </is>
       </c>
-      <c r="AH156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -26363,7 +26115,6 @@
           <t>Anipeddi Lasya</t>
         </is>
       </c>
-      <c r="C157" t="inlineStr"/>
       <c r="D157" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -26514,7 +26265,6 @@
           <t>Which CMM service hosts the MME functions?</t>
         </is>
       </c>
-      <c r="AH157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -26527,7 +26277,6 @@
           <t>Biruntha</t>
         </is>
       </c>
-      <c r="C158" t="inlineStr"/>
       <c r="D158" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -26678,7 +26427,6 @@
           <t>Which deployment characteristic is strongly associated with CMG?</t>
         </is>
       </c>
-      <c r="AH158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -26691,7 +26439,6 @@
           <t>Himanshu Bungla</t>
         </is>
       </c>
-      <c r="C159" t="inlineStr"/>
       <c r="D159" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -26842,7 +26589,6 @@
           <t>In a 5G ATP test, what should be verified first for NRD?</t>
         </is>
       </c>
-      <c r="AH159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -26855,7 +26601,6 @@
           <t>Nijampatnam Eswar</t>
         </is>
       </c>
-      <c r="C160" t="inlineStr"/>
       <c r="D160" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -27006,7 +26751,6 @@
           <t>What is a practical ATP objective for CMG interworking?</t>
         </is>
       </c>
-      <c r="AH160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -27019,7 +26763,6 @@
           <t>Saiyed Raza Imam</t>
         </is>
       </c>
-      <c r="C161" t="inlineStr"/>
       <c r="D161" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -27170,7 +26913,6 @@
           <t>Which ATP case is useful for validating CMG resilience?</t>
         </is>
       </c>
-      <c r="AH161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -27183,7 +26925,6 @@
           <t>Vaijinath Bhaskar Batule</t>
         </is>
       </c>
-      <c r="C162" t="inlineStr"/>
       <c r="D162" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -27334,7 +27075,6 @@
           <t>Why is CMG considered operationally flexible?</t>
         </is>
       </c>
-      <c r="AH162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -27347,7 +27087,6 @@
           <t>Kamal Kumar Ray</t>
         </is>
       </c>
-      <c r="C163" t="inlineStr"/>
       <c r="D163" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -27498,7 +27237,6 @@
           <t>Which CMM service hosts the MME functions?</t>
         </is>
       </c>
-      <c r="AH163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -27511,7 +27249,6 @@
           <t>Tanmoy Mojumder</t>
         </is>
       </c>
-      <c r="C164" t="inlineStr"/>
       <c r="D164" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -27662,7 +27399,6 @@
           <t>Which technology is highlighted in CMM for performance optimization on x86 platforms?</t>
         </is>
       </c>
-      <c r="AH164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -27675,7 +27411,6 @@
           <t>Shaikh Reshma</t>
         </is>
       </c>
-      <c r="C165" t="inlineStr"/>
       <c r="D165" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -27826,7 +27561,6 @@
           <t>Which CMM component is responsible for OAM functions and northbound interfaces?</t>
         </is>
       </c>
-      <c r="AH165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -27839,7 +27573,6 @@
           <t>Om Prakash Gautam</t>
         </is>
       </c>
-      <c r="C166" t="inlineStr"/>
       <c r="D166" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -27990,7 +27723,6 @@
           <t>What is the primary role of Nokia Cloud Mobile Gateway (CMG) in packet core?</t>
         </is>
       </c>
-      <c r="AH166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -28003,7 +27735,6 @@
           <t>Jaya Vohra</t>
         </is>
       </c>
-      <c r="C167" t="inlineStr"/>
       <c r="D167" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -28154,7 +27885,6 @@
           <t>CMG can support which access evolution model?</t>
         </is>
       </c>
-      <c r="AH167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -28167,7 +27897,6 @@
           <t>S Bijetananda Swain</t>
         </is>
       </c>
-      <c r="C168" t="inlineStr"/>
       <c r="D168" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -28318,7 +28047,6 @@
           <t>If attach succeeds but data service fails, which CMG area should be checked first?</t>
         </is>
       </c>
-      <c r="AH168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -28331,7 +28059,6 @@
           <t>Rohit Kumar</t>
         </is>
       </c>
-      <c r="C169" t="inlineStr"/>
       <c r="D169" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -28482,7 +28209,6 @@
           <t>Which is most likely to be verified in CMG acceptance for 4G?</t>
         </is>
       </c>
-      <c r="AH169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -28495,7 +28221,6 @@
           <t>Sujata Singh</t>
         </is>
       </c>
-      <c r="C170" t="inlineStr"/>
       <c r="D170" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -28646,7 +28371,6 @@
           <t>Why is CMG considered operationally flexible?</t>
         </is>
       </c>
-      <c r="AH170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -28659,7 +28383,6 @@
           <t>SUSHMA CHOLLETI</t>
         </is>
       </c>
-      <c r="C171" t="inlineStr"/>
       <c r="D171" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -28810,7 +28533,6 @@
           <t>Why is CMG considered operationally flexible?</t>
         </is>
       </c>
-      <c r="AH171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -28823,7 +28545,6 @@
           <t>Gaurav Verma</t>
         </is>
       </c>
-      <c r="C172" t="inlineStr"/>
       <c r="D172" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -28974,7 +28695,6 @@
           <t>CMG can support which access evolution model?</t>
         </is>
       </c>
-      <c r="AH172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -28987,7 +28707,6 @@
           <t>Kamna Peyal</t>
         </is>
       </c>
-      <c r="C173" t="inlineStr"/>
       <c r="D173" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -29138,7 +28857,6 @@
           <t>Key onboarding activity for CMM?</t>
         </is>
       </c>
-      <c r="AH173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -29151,7 +28869,6 @@
           <t>Damarasinghu Vinay Kumar</t>
         </is>
       </c>
-      <c r="C174" t="inlineStr"/>
       <c r="D174" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -29302,7 +29019,6 @@
           <t>Which outcome indicates a successful CMG onboarding and integration cycle?</t>
         </is>
       </c>
-      <c r="AH174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -29315,7 +29031,6 @@
           <t>Devarapalli Siva Naga Srivalli</t>
         </is>
       </c>
-      <c r="C175" t="inlineStr"/>
       <c r="D175" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -29466,7 +29181,6 @@
           <t>Which ATP case is useful for validating CMG resilience?</t>
         </is>
       </c>
-      <c r="AH175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -29479,7 +29193,6 @@
           <t>Etakaati Chandan Srinivas</t>
         </is>
       </c>
-      <c r="C176" t="inlineStr"/>
       <c r="D176" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -29630,7 +29343,6 @@
           <t>Which scenario best tests CMG under mobility conditions?</t>
         </is>
       </c>
-      <c r="AH176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -29643,7 +29355,6 @@
           <t>Guttula Vaishnavi</t>
         </is>
       </c>
-      <c r="C177" t="inlineStr"/>
       <c r="D177" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -29794,7 +29505,6 @@
           <t>Attach ok but PDN fails. Check?</t>
         </is>
       </c>
-      <c r="AH177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -29807,7 +29517,6 @@
           <t>Hamsa Yaswanth Paul</t>
         </is>
       </c>
-      <c r="C178" t="inlineStr"/>
       <c r="D178" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -29958,7 +29667,6 @@
           <t>In 4G LTE, CMM most commonly provides which network function?</t>
         </is>
       </c>
-      <c r="AH178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -29971,7 +29679,6 @@
           <t>Kasi Nandini</t>
         </is>
       </c>
-      <c r="C179" t="inlineStr"/>
       <c r="D179" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -30122,7 +29829,6 @@
           <t>Attach fails after MME relocation. What is tested?</t>
         </is>
       </c>
-      <c r="AH179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -30135,7 +29841,6 @@
           <t>Lavanya Seerapu</t>
         </is>
       </c>
-      <c r="C180" t="inlineStr"/>
       <c r="D180" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -30286,7 +29991,6 @@
           <t>What is the best description of a Network Function Instance in NRD/SBA context?</t>
         </is>
       </c>
-      <c r="AH180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -30299,7 +30003,6 @@
           <t>Pappala Sai Kishor</t>
         </is>
       </c>
-      <c r="C181" t="inlineStr"/>
       <c r="D181" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -30450,7 +30153,6 @@
           <t>In a CMG ATP plan, which test most directly verifies end-user data service?</t>
         </is>
       </c>
-      <c r="AH181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -30463,7 +30165,6 @@
           <t>Rachabathula Deepthisri</t>
         </is>
       </c>
-      <c r="C182" t="inlineStr"/>
       <c r="D182" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -30614,7 +30315,6 @@
           <t>CMG supports evolution toward which major core direction?</t>
         </is>
       </c>
-      <c r="AH182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -30627,7 +30327,6 @@
           <t>Srujan Palla</t>
         </is>
       </c>
-      <c r="C183" t="inlineStr"/>
       <c r="D183" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -30778,7 +30477,6 @@
           <t>In a 4G ATP scenario, what does successful bearer establishment mainly confirm?</t>
         </is>
       </c>
-      <c r="AH183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -30791,7 +30489,6 @@
           <t>Swetha Konchada</t>
         </is>
       </c>
-      <c r="C184" t="inlineStr"/>
       <c r="D184" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -30942,7 +30639,6 @@
           <t>CMG supports evolution toward which major core direction?</t>
         </is>
       </c>
-      <c r="AH184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -30955,7 +30651,6 @@
           <t>Vivek Singh</t>
         </is>
       </c>
-      <c r="C185" t="inlineStr"/>
       <c r="D185" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -31106,7 +30801,6 @@
           <t>Which is a common integration point for CMG in EPC?</t>
         </is>
       </c>
-      <c r="AH185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -31119,7 +30813,6 @@
           <t>Akshit Sahni</t>
         </is>
       </c>
-      <c r="C186" t="inlineStr"/>
       <c r="D186" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -31270,7 +30963,6 @@
           <t>Which aspect is most important during CMG onboarding?</t>
         </is>
       </c>
-      <c r="AH186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -31283,7 +30975,6 @@
           <t>Abhiram Jagarlamudi</t>
         </is>
       </c>
-      <c r="C187" t="inlineStr"/>
       <c r="D187" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -31434,7 +31125,6 @@
           <t>Why is CMG considered operationally flexible?</t>
         </is>
       </c>
-      <c r="AH187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -31447,7 +31137,6 @@
           <t>Debopriyo Halder</t>
         </is>
       </c>
-      <c r="C188" t="inlineStr"/>
       <c r="D188" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -31598,7 +31287,6 @@
           <t>Which CMM service is associated with user-plane packet processing and data forwarding?</t>
         </is>
       </c>
-      <c r="AH188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -31611,7 +31299,6 @@
           <t>Alok Kumar Nayak</t>
         </is>
       </c>
-      <c r="C189" t="inlineStr"/>
       <c r="D189" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -31762,7 +31449,6 @@
           <t>Which ATP case is useful for validating CMG resilience?</t>
         </is>
       </c>
-      <c r="AH189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -31775,7 +31461,6 @@
           <t>Archit Bagulia</t>
         </is>
       </c>
-      <c r="C190" t="inlineStr"/>
       <c r="D190" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -31926,7 +31611,6 @@
           <t>Which design goal is central to NRD’s cloud-native approach?</t>
         </is>
       </c>
-      <c r="AH190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -31939,7 +31623,6 @@
           <t>Arunkumar Balappa Pattadakall</t>
         </is>
       </c>
-      <c r="C191" t="inlineStr"/>
       <c r="D191" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -32090,7 +31773,6 @@
           <t>Successful ATP indication?</t>
         </is>
       </c>
-      <c r="AH191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -32103,7 +31785,6 @@
           <t>Dewashish Kumar</t>
         </is>
       </c>
-      <c r="C192" t="inlineStr"/>
       <c r="D192" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -32254,7 +31935,6 @@
           <t>Which design goal is central to NRD’s cloud-native approach?</t>
         </is>
       </c>
-      <c r="AH192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -32267,7 +31947,6 @@
           <t>Subhankar Hazra</t>
         </is>
       </c>
-      <c r="C193" t="inlineStr"/>
       <c r="D193" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -32418,7 +32097,6 @@
           <t>Attach fails after MME relocation. What is tested?</t>
         </is>
       </c>
-      <c r="AH193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -32431,7 +32109,6 @@
           <t>Ajay Kumar</t>
         </is>
       </c>
-      <c r="C194" t="inlineStr"/>
       <c r="D194" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -32582,7 +32259,6 @@
           <t>In a 4G ATP scenario, what does successful bearer establishment mainly confirm?</t>
         </is>
       </c>
-      <c r="AH194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -32595,7 +32271,6 @@
           <t>Altamash Ashfaq</t>
         </is>
       </c>
-      <c r="C195" t="inlineStr"/>
       <c r="D195" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -32746,7 +32421,6 @@
           <t>What is the best description of a Network Function Instance in NRD/SBA context?</t>
         </is>
       </c>
-      <c r="AH195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -32759,7 +32433,6 @@
           <t>Preetam Mehta</t>
         </is>
       </c>
-      <c r="C196" t="inlineStr"/>
       <c r="D196" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -32910,7 +32583,6 @@
           <t>Which protocol family is most relevant to CMG integration with EPC nodes?</t>
         </is>
       </c>
-      <c r="AH196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -32923,7 +32595,6 @@
           <t>Guru Prasad</t>
         </is>
       </c>
-      <c r="C197" t="inlineStr"/>
       <c r="D197" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -33074,7 +32745,6 @@
           <t>Which CMM service handles 2G/3G mobility and session management?</t>
         </is>
       </c>
-      <c r="AH197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -33087,7 +32757,6 @@
           <t>Raviraj Dhondiram Chalikwar</t>
         </is>
       </c>
-      <c r="C198" t="inlineStr"/>
       <c r="D198" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -33238,7 +32907,6 @@
           <t>Which protocol style is most aligned with NRD in an SBA environment?</t>
         </is>
       </c>
-      <c r="AH198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -33251,7 +32919,6 @@
           <t>Snehal Mavale</t>
         </is>
       </c>
-      <c r="C199" t="inlineStr"/>
       <c r="D199" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -33402,7 +33069,6 @@
           <t>Which lifecycle operations are associated with NRD CNF management?</t>
         </is>
       </c>
-      <c r="AH199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -33415,7 +33081,6 @@
           <t>Rakshitha K M</t>
         </is>
       </c>
-      <c r="C200" t="inlineStr"/>
       <c r="D200" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -33566,7 +33231,6 @@
           <t>Key onboarding activity for CMM?</t>
         </is>
       </c>
-      <c r="AH200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -33579,7 +33243,6 @@
           <t>Sakshi Srivastava</t>
         </is>
       </c>
-      <c r="C201" t="inlineStr"/>
       <c r="D201" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -33730,7 +33393,6 @@
           <t>Attach ok but PDN fails. Check?</t>
         </is>
       </c>
-      <c r="AH201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -33743,7 +33405,6 @@
           <t>Sukanya</t>
         </is>
       </c>
-      <c r="C202" t="inlineStr"/>
       <c r="D202" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -33894,7 +33555,6 @@
           <t>CMM is described by Nokia as having what kind of architecture?</t>
         </is>
       </c>
-      <c r="AH202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -33907,7 +33567,6 @@
           <t>Vijay Laxman Dhomase</t>
         </is>
       </c>
-      <c r="C203" t="inlineStr"/>
       <c r="D203" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -34058,7 +33717,6 @@
           <t>Which CMM service hosts the MME functions?</t>
         </is>
       </c>
-      <c r="AH203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -34071,7 +33729,6 @@
           <t>Angshuman Sarma</t>
         </is>
       </c>
-      <c r="C204" t="inlineStr"/>
       <c r="D204" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -34222,7 +33879,6 @@
           <t>What is the best description of a Network Function Instance in NRD/SBA context?</t>
         </is>
       </c>
-      <c r="AH204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -34235,7 +33891,6 @@
           <t>Nisha Kailas Mali</t>
         </is>
       </c>
-      <c r="C205" t="inlineStr"/>
       <c r="D205" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -34386,7 +34041,6 @@
           <t>Which is a common integration point for CMG in EPC?</t>
         </is>
       </c>
-      <c r="AH205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -34399,7 +34053,6 @@
           <t>Ravi Ranjan</t>
         </is>
       </c>
-      <c r="C206" t="inlineStr"/>
       <c r="D206" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -34550,7 +34203,6 @@
           <t>In 4G LTE, CMM most commonly provides which network function?</t>
         </is>
       </c>
-      <c r="AH206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -34563,7 +34215,6 @@
           <t>Sarjitkumar Rajyaguru</t>
         </is>
       </c>
-      <c r="C207" t="inlineStr"/>
       <c r="D207" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -34714,7 +34365,6 @@
           <t>Which symptom during ATP most likely indicates a control-plane integration problem?</t>
         </is>
       </c>
-      <c r="AH207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -34727,7 +34377,6 @@
           <t>Ajith V A</t>
         </is>
       </c>
-      <c r="C208" t="inlineStr"/>
       <c r="D208" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -34878,7 +34527,6 @@
           <t>Which CMM component provides logical interface termination for GTP and Diameter?</t>
         </is>
       </c>
-      <c r="AH208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -34891,7 +34539,6 @@
           <t>Sugat Bhalshankar</t>
         </is>
       </c>
-      <c r="C209" t="inlineStr"/>
       <c r="D209" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -35042,7 +34689,6 @@
           <t>Which is most likely to be verified in CMG acceptance for 4G?</t>
         </is>
       </c>
-      <c r="AH209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -35055,7 +34701,6 @@
           <t>Altaf Ahmad</t>
         </is>
       </c>
-      <c r="C210" t="inlineStr"/>
       <c r="D210" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -35206,7 +34851,6 @@
           <t>What is critical to validate for mobility in ATP?</t>
         </is>
       </c>
-      <c r="AH210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -35219,7 +34863,6 @@
           <t>Dhruv Kant Goyal</t>
         </is>
       </c>
-      <c r="C211" t="inlineStr"/>
       <c r="D211" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -35370,7 +35013,6 @@
           <t>Which design goal is central to NRD’s cloud-native approach?</t>
         </is>
       </c>
-      <c r="AH211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -35383,7 +35025,6 @@
           <t>Mohammad Ayyub</t>
         </is>
       </c>
-      <c r="C212" t="inlineStr"/>
       <c r="D212" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -35534,7 +35175,6 @@
           <t>What is the primary role of Nokia Cloud Mobile Gateway (CMG) in packet core?</t>
         </is>
       </c>
-      <c r="AH212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -35547,7 +35187,6 @@
           <t>Vivek Mishra</t>
         </is>
       </c>
-      <c r="C213" t="inlineStr"/>
       <c r="D213" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -35698,7 +35337,6 @@
           <t>Which statement best describes NRD deployment architecture?</t>
         </is>
       </c>
-      <c r="AH213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -35711,7 +35349,6 @@
           <t>Abhishek Kumar Patel</t>
         </is>
       </c>
-      <c r="C214" t="inlineStr"/>
       <c r="D214" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -35862,7 +35499,6 @@
           <t>Key onboarding activity for CMM?</t>
         </is>
       </c>
-      <c r="AH214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -35875,7 +35511,6 @@
           <t>Chandra Sen</t>
         </is>
       </c>
-      <c r="C215" t="inlineStr"/>
       <c r="D215" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -36026,7 +35661,6 @@
           <t>CMG is best described as:</t>
         </is>
       </c>
-      <c r="AH215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -36039,7 +35673,6 @@
           <t>Depankar Kumar</t>
         </is>
       </c>
-      <c r="C216" t="inlineStr"/>
       <c r="D216" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -36190,7 +35823,6 @@
           <t>Which protocol family is most relevant to CMG integration with EPC nodes?</t>
         </is>
       </c>
-      <c r="AH216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -36203,7 +35835,6 @@
           <t>Mohanram G</t>
         </is>
       </c>
-      <c r="C217" t="inlineStr"/>
       <c r="D217" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -36354,7 +35985,6 @@
           <t>Which statement best reflects CMG architecture?</t>
         </is>
       </c>
-      <c r="AH217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -36367,7 +35997,6 @@
           <t>Manpreet Kaur</t>
         </is>
       </c>
-      <c r="C218" t="inlineStr"/>
       <c r="D218" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -36518,7 +36147,6 @@
           <t>Attach succeeds but bearer fails. Likely issue?</t>
         </is>
       </c>
-      <c r="AH218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -36531,7 +36159,6 @@
           <t>R Timmappa</t>
         </is>
       </c>
-      <c r="C219" t="inlineStr"/>
       <c r="D219" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -36682,7 +36309,6 @@
           <t>Which Nokia platform is commonly used for CMM management?</t>
         </is>
       </c>
-      <c r="AH219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -36695,7 +36321,6 @@
           <t>Smruti Snigdha Sahoo</t>
         </is>
       </c>
-      <c r="C220" t="inlineStr"/>
       <c r="D220" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -36846,7 +36471,6 @@
           <t>In a CMG ATP plan, which test most directly verifies end-user data service?</t>
         </is>
       </c>
-      <c r="AH220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -36859,7 +36483,6 @@
           <t>Tejaswini Patel</t>
         </is>
       </c>
-      <c r="C221" t="inlineStr"/>
       <c r="D221" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -37010,7 +36633,6 @@
           <t>Which ATP case is useful for validating CMG resilience?</t>
         </is>
       </c>
-      <c r="AH221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -37023,7 +36645,6 @@
           <t>Amit Ravindra Ghadge</t>
         </is>
       </c>
-      <c r="C222" t="inlineStr"/>
       <c r="D222" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -37174,7 +36795,6 @@
           <t>Which scenario best tests CMG under mobility conditions?</t>
         </is>
       </c>
-      <c r="AH222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -37187,7 +36807,6 @@
           <t>Sayanth A V</t>
         </is>
       </c>
-      <c r="C223" t="inlineStr"/>
       <c r="D223" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -37338,7 +36957,6 @@
           <t>CMM supports which management interfaces for operations and troubleshooting?</t>
         </is>
       </c>
-      <c r="AH223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -37351,7 +36969,6 @@
           <t>Abhishek Kumar</t>
         </is>
       </c>
-      <c r="C224" t="inlineStr"/>
       <c r="D224" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -37502,7 +37119,6 @@
           <t>Which aspect is most important during CMG onboarding?</t>
         </is>
       </c>
-      <c r="AH224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -37515,7 +37131,6 @@
           <t>Avinash Yadav</t>
         </is>
       </c>
-      <c r="C225" t="inlineStr"/>
       <c r="D225" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -37666,7 +37281,6 @@
           <t>Attach ok but PDN fails. Check?</t>
         </is>
       </c>
-      <c r="AH225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -37679,7 +37293,6 @@
           <t>Mohammad Ali Ahmed Jameel</t>
         </is>
       </c>
-      <c r="C226" t="inlineStr"/>
       <c r="D226" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -37830,7 +37443,6 @@
           <t>CMG is best described as:</t>
         </is>
       </c>
-      <c r="AH226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -37843,7 +37455,6 @@
           <t>Mohammad Mohasin Khan</t>
         </is>
       </c>
-      <c r="C227" t="inlineStr"/>
       <c r="D227" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -37994,7 +37605,6 @@
           <t>Attach fails after MME relocation. What is tested?</t>
         </is>
       </c>
-      <c r="AH227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -38007,7 +37617,6 @@
           <t>Naredla Nirosha</t>
         </is>
       </c>
-      <c r="C228" t="inlineStr"/>
       <c r="D228" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -38158,7 +37767,6 @@
           <t>What is a major functional benefit of CMG in packet core?</t>
         </is>
       </c>
-      <c r="AH228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -38171,7 +37779,6 @@
           <t>Sachin P Gilbile</t>
         </is>
       </c>
-      <c r="C229" t="inlineStr"/>
       <c r="D229" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -38322,7 +37929,6 @@
           <t>CMG is best described as:</t>
         </is>
       </c>
-      <c r="AH229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -38335,7 +37941,6 @@
           <t>Liji Babu</t>
         </is>
       </c>
-      <c r="C230" t="inlineStr"/>
       <c r="D230" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -38486,7 +38091,6 @@
           <t>CMM supports which management interfaces for operations and troubleshooting?</t>
         </is>
       </c>
-      <c r="AH230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -38499,7 +38103,6 @@
           <t>Arvind Kumar Singh</t>
         </is>
       </c>
-      <c r="C231" t="inlineStr"/>
       <c r="D231" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -38650,7 +38253,6 @@
           <t>Successful ATP indication?</t>
         </is>
       </c>
-      <c r="AH231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -38663,7 +38265,6 @@
           <t>Aparajita Shankar</t>
         </is>
       </c>
-      <c r="C232" t="inlineStr"/>
       <c r="D232" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -38814,7 +38415,6 @@
           <t>What is the best description of a Network Function Instance in NRD/SBA context?</t>
         </is>
       </c>
-      <c r="AH232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -38827,7 +38427,6 @@
           <t>Phani Shree</t>
         </is>
       </c>
-      <c r="C233" t="inlineStr"/>
       <c r="D233" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -38978,7 +38577,6 @@
           <t>Attach fails for specific IMSI range. Cause?</t>
         </is>
       </c>
-      <c r="AH233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -38991,7 +38589,6 @@
           <t>S Mohankumar</t>
         </is>
       </c>
-      <c r="C234" t="inlineStr"/>
       <c r="D234" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -39142,7 +38739,6 @@
           <t>In onboarding, which item is usually validated first?</t>
         </is>
       </c>
-      <c r="AH234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -39155,7 +38751,6 @@
           <t>Manojkannan</t>
         </is>
       </c>
-      <c r="C235" t="inlineStr"/>
       <c r="D235" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -39306,7 +38901,6 @@
           <t>If attach succeeds but data service fails, which CMG area should be checked first?</t>
         </is>
       </c>
-      <c r="AH235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -39319,7 +38913,6 @@
           <t>Srivani Supraja</t>
         </is>
       </c>
-      <c r="C236" t="inlineStr"/>
       <c r="D236" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -39470,7 +39063,6 @@
           <t>CMM is described by Nokia as having what kind of architecture?</t>
         </is>
       </c>
-      <c r="AH236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -39483,7 +39075,6 @@
           <t>Nutan Rani</t>
         </is>
       </c>
-      <c r="C237" t="inlineStr"/>
       <c r="D237" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -39634,7 +39225,6 @@
           <t>First ATP validation step should be?</t>
         </is>
       </c>
-      <c r="AH237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -39647,7 +39237,6 @@
           <t>Prasanth S</t>
         </is>
       </c>
-      <c r="C238" t="inlineStr"/>
       <c r="D238" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -39798,7 +39387,6 @@
           <t>Which aspect is most important during CMG onboarding?</t>
         </is>
       </c>
-      <c r="AH238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -39811,7 +39399,6 @@
           <t>Pankaj Verma</t>
         </is>
       </c>
-      <c r="C239" t="inlineStr"/>
       <c r="D239" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -39962,7 +39549,6 @@
           <t>Which protocol family is most relevant to CMG integration with EPC nodes?</t>
         </is>
       </c>
-      <c r="AH239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -39975,7 +39561,6 @@
           <t>Madhura Atul Kulkarni</t>
         </is>
       </c>
-      <c r="C240" t="inlineStr"/>
       <c r="D240" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -40126,7 +39711,6 @@
           <t>Which interface is key for LTE access during ATP?</t>
         </is>
       </c>
-      <c r="AH240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -40139,7 +39723,6 @@
           <t>Sahil Mantrao</t>
         </is>
       </c>
-      <c r="C241" t="inlineStr"/>
       <c r="D241" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -40290,7 +39873,6 @@
           <t>What is the primary role of Nokia Cloud Mobility Manager (CMM) in a 4G packet core?</t>
         </is>
       </c>
-      <c r="AH241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -40303,7 +39885,6 @@
           <t>Satish Maurya</t>
         </is>
       </c>
-      <c r="C242" t="inlineStr"/>
       <c r="D242" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -40454,7 +40035,6 @@
           <t>If attach succeeds but data service fails, which CMG area should be checked first?</t>
         </is>
       </c>
-      <c r="AH242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -40467,7 +40047,6 @@
           <t>Janardan Singh</t>
         </is>
       </c>
-      <c r="C243" t="inlineStr"/>
       <c r="D243" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -40618,7 +40197,6 @@
           <t>CMM is described by Nokia as having what kind of architecture?</t>
         </is>
       </c>
-      <c r="AH243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -40631,7 +40209,6 @@
           <t>Kushagra Chaudhary</t>
         </is>
       </c>
-      <c r="C244" t="inlineStr"/>
       <c r="D244" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -40782,7 +40359,6 @@
           <t>Which ATP case is useful for validating CMG resilience?</t>
         </is>
       </c>
-      <c r="AH244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -40795,7 +40371,6 @@
           <t>Ayan Kumar Roy</t>
         </is>
       </c>
-      <c r="C245" t="inlineStr"/>
       <c r="D245" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -40946,7 +40521,6 @@
           <t>Which is a common integration point for CMG in EPC?</t>
         </is>
       </c>
-      <c r="AH245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -40959,7 +40533,6 @@
           <t>Yashi Gupta</t>
         </is>
       </c>
-      <c r="C246" t="inlineStr"/>
       <c r="D246" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -41110,7 +40683,6 @@
           <t>Best failover ATP test?</t>
         </is>
       </c>
-      <c r="AH246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -41123,7 +40695,6 @@
           <t>Anita KM</t>
         </is>
       </c>
-      <c r="C247" t="inlineStr"/>
       <c r="D247" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -41274,7 +40845,6 @@
           <t>Attach fails after MME relocation. What is tested?</t>
         </is>
       </c>
-      <c r="AH247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -41287,7 +40857,6 @@
           <t>Nitesh Kumar</t>
         </is>
       </c>
-      <c r="C248" t="inlineStr"/>
       <c r="D248" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -41438,7 +41007,6 @@
           <t>In 4G EPC, CMG is most closely associated with which gateway role?</t>
         </is>
       </c>
-      <c r="AH248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -41451,7 +41019,6 @@
           <t>Pratibha Singh</t>
         </is>
       </c>
-      <c r="C249" t="inlineStr"/>
       <c r="D249" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -41602,7 +41169,6 @@
           <t>Which ATP check best confirms attach-related functionality?</t>
         </is>
       </c>
-      <c r="AH249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -41615,7 +41181,6 @@
           <t>Neha Ojha</t>
         </is>
       </c>
-      <c r="C250" t="inlineStr"/>
       <c r="D250" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -41766,7 +41331,6 @@
           <t>If attach succeeds but data service fails, which CMG area should be checked first?</t>
         </is>
       </c>
-      <c r="AH250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -41779,7 +41343,6 @@
           <t>P Vishnu</t>
         </is>
       </c>
-      <c r="C251" t="inlineStr"/>
       <c r="D251" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -41930,7 +41493,6 @@
           <t>Which ATP outcome best confirms correct NRD functionality?</t>
         </is>
       </c>
-      <c r="AH251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -41943,7 +41505,6 @@
           <t>khusboo Mantoo</t>
         </is>
       </c>
-      <c r="C252" t="inlineStr"/>
       <c r="D252" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -42094,7 +41655,6 @@
           <t>In 4G EPC, CMG is most closely associated with which gateway role?</t>
         </is>
       </c>
-      <c r="AH252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -42107,7 +41667,6 @@
           <t>Shridhar Patange</t>
         </is>
       </c>
-      <c r="C253" t="inlineStr"/>
       <c r="D253" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -42258,7 +41817,6 @@
           <t>What is the primary role of Nokia Cloud Mobile Gateway (CMG) in packet core?</t>
         </is>
       </c>
-      <c r="AH253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -42271,7 +41829,6 @@
           <t>Vishal Chaudhary</t>
         </is>
       </c>
-      <c r="C254" t="inlineStr"/>
       <c r="D254" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -42422,7 +41979,6 @@
           <t>NRD implements which kind of services?</t>
         </is>
       </c>
-      <c r="AH254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -42435,7 +41991,6 @@
           <t>Niteesh Pandey</t>
         </is>
       </c>
-      <c r="C255" t="inlineStr"/>
       <c r="D255" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -42586,7 +42141,6 @@
           <t>Which outcome indicates a successful CMG onboarding and integration cycle?</t>
         </is>
       </c>
-      <c r="AH255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -42599,7 +42153,6 @@
           <t>Akanksha Haste</t>
         </is>
       </c>
-      <c r="C256" t="inlineStr"/>
       <c r="D256" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -42750,7 +42303,6 @@
           <t>In onboarding, which item is usually validated first?</t>
         </is>
       </c>
-      <c r="AH256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -42763,7 +42315,6 @@
           <t>Abdullah Ahmed</t>
         </is>
       </c>
-      <c r="C257" t="inlineStr"/>
       <c r="D257" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -42914,7 +42465,6 @@
           <t>In a 4G ATP scenario, what does successful bearer establishment mainly confirm?</t>
         </is>
       </c>
-      <c r="AH257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -42927,7 +42477,6 @@
           <t>Devendra Pratap Gupta</t>
         </is>
       </c>
-      <c r="C258" t="inlineStr"/>
       <c r="D258" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -43078,7 +42627,6 @@
           <t>Which aspect is most important during CMG onboarding?</t>
         </is>
       </c>
-      <c r="AH258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -43091,7 +42639,6 @@
           <t>Mukkollu Nagababu</t>
         </is>
       </c>
-      <c r="C259" t="inlineStr"/>
       <c r="D259" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -43242,7 +42789,6 @@
           <t>Which is a common integration point for CMG in EPC?</t>
         </is>
       </c>
-      <c r="AH259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -43255,7 +42801,6 @@
           <t>Divyanshu Vikram Bhadouria</t>
         </is>
       </c>
-      <c r="C260" t="inlineStr"/>
       <c r="D260" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -43406,7 +42951,6 @@
           <t>What is a practical ATP objective for CMG interworking?</t>
         </is>
       </c>
-      <c r="AH260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -43419,7 +42963,6 @@
           <t>Harshraj Sharma</t>
         </is>
       </c>
-      <c r="C261" t="inlineStr"/>
       <c r="D261" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -43570,7 +43113,6 @@
           <t>What is a practical ATP objective for CMG interworking?</t>
         </is>
       </c>
-      <c r="AH261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -43583,7 +43125,6 @@
           <t>Deepak Kumar Sharma</t>
         </is>
       </c>
-      <c r="C262" t="inlineStr"/>
       <c r="D262" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -43734,7 +43275,6 @@
           <t>In 4G EPC, CMG is most closely associated with which gateway role?</t>
         </is>
       </c>
-      <c r="AH262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -43747,7 +43287,6 @@
           <t>Anand Kumar</t>
         </is>
       </c>
-      <c r="C263" t="inlineStr"/>
       <c r="D263" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -43898,7 +43437,6 @@
           <t>Which is a common integration point for CMG in EPC?</t>
         </is>
       </c>
-      <c r="AH263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -43911,7 +43449,6 @@
           <t>Priya  M</t>
         </is>
       </c>
-      <c r="C264" t="inlineStr"/>
       <c r="D264" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -44062,7 +43599,6 @@
           <t>Which ATP check best confirms attach-related functionality?</t>
         </is>
       </c>
-      <c r="AH264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -44075,7 +43611,6 @@
           <t>Navyasri Neelapu</t>
         </is>
       </c>
-      <c r="C265" t="inlineStr"/>
       <c r="D265" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -44226,7 +43761,6 @@
           <t>CMG is best described as:</t>
         </is>
       </c>
-      <c r="AH265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -44239,7 +43773,6 @@
           <t>Deepika  S</t>
         </is>
       </c>
-      <c r="C266" t="inlineStr"/>
       <c r="D266" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -44390,7 +43923,6 @@
           <t>CMG can support which access evolution model?</t>
         </is>
       </c>
-      <c r="AH266" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix SDM question mapping to use QB-new.xlsx as the sole question source.
Parse HLR-HSS from QB-new correctly, remove legacy Question Bank exports, regenerate employee mappings, and add Supabase reassignment scripts for SDM employees.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Resource_Question_Mapping.xlsx
+++ b/Resource_Question_Mapping.xlsx
@@ -754,6 +754,7 @@
           <t>[HSS Troubleshooting] The healthCheck.log shows isRtpReadinessOK: False. Which command should be used next to check RTP-based process status?</t>
         </is>
       </c>
+      <c r="AH2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -921,6 +922,7 @@
           <t>[HSS Troubleshooting] An operator runs kubectl get pod -n hss and notices one pod shows 2/3 Running in the Ready column. What does this indicate?</t>
         </is>
       </c>
+      <c r="AH3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1088,6 +1090,7 @@
           <t>[HSS Deployment] After deploying Nokia HSS CNF through NCOM, the engineer must confirm whether all pods are running in the target namespace. Which command should be used?</t>
         </is>
       </c>
+      <c r="AH4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1255,6 +1258,7 @@
           <t>[UDM Planning] Planning for LLB failover requires historical CFR statistics on each connection to influence PG server selection. What is this called?</t>
         </is>
       </c>
+      <c r="AH5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1422,6 +1426,7 @@
           <t>[Deployment &amp; Troubleshooting] If all HTTP/2 LB Pods run into Http/2 egress connection failure simultaneously, what happens at the NRF level?</t>
         </is>
       </c>
+      <c r="AH6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1589,6 +1594,7 @@
           <t>[HSS Basics] An MME requests authentication vectors for a subscriber attempting to attach to the LTE network. Which service generates these vectors?</t>
         </is>
       </c>
+      <c r="AH7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1756,6 +1762,7 @@
           <t>[UDM Basic] A subscriber roams to another PLMN and the HPLMN needs to securely deliver a preferred PLMN list. Which service secures this SoR data?</t>
         </is>
       </c>
+      <c r="AH8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1923,6 +1930,7 @@
           <t>[Deployment &amp; Troubleshooting] A troubleshooting engineer notices Pods with unusually high error rates and wants automatic isolation and recovery. Which feature addresses this?</t>
         </is>
       </c>
+      <c r="AH9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2090,6 +2098,7 @@
           <t>[Deployment &amp; Troubleshooting] Before running Netconf rpc commands to configure the CDS threshold, what tool must be installed on the operator's machine?</t>
         </is>
       </c>
+      <c r="AH10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2257,6 +2266,7 @@
           <t>[HSS Basics] The operations team notices failures in SS7 message routing toward HLR processing nodes. Which service should be investigated first?</t>
         </is>
       </c>
+      <c r="AH11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2424,6 +2434,7 @@
           <t>[UDM Basic] AUSF NF wants to retrieve authentication data from UDM. Which interface should be used?</t>
         </is>
       </c>
+      <c r="AH12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2591,6 +2602,7 @@
           <t>[HSS Troubleshooting] An engineer wants to verify SCTP connection status for SS7. Which command is recommended instead of relying on netstat?</t>
         </is>
       </c>
+      <c r="AH13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2758,6 +2770,7 @@
           <t>[Deployment &amp; Troubleshooting] When the HTTP/2 LB Pod detects an egress connection failure, where is the failure file written?</t>
         </is>
       </c>
+      <c r="AH14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2925,6 +2938,7 @@
           <t>[UDM Basic] A SUCI needs to be de-concealed to a SUPI. Which service performs this function?</t>
         </is>
       </c>
+      <c r="AH15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3092,6 +3106,7 @@
           <t>[Deployment &amp; Troubleshooting] The NIM leader Pod goes down unexpectedly. What happens to NRF interfacing during the leader re-election?</t>
         </is>
       </c>
+      <c r="AH16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3259,6 +3274,7 @@
           <t>[HSS Deployment] The SS7 pod fails to apply the Telesys license. The license file is named M7-KEY-demo.tar.gz, but the configured VNF ID is hlrcn. What should be checked first?</t>
         </is>
       </c>
+      <c r="AH17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3426,6 +3442,7 @@
           <t>[HSS Troubleshooting] The healthCheck.log shows isRtpReadinessOK: False. Which command should be used next to check RTP-based process status?</t>
         </is>
       </c>
+      <c r="AH18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3593,6 +3610,7 @@
           <t>[HSS Deployment] A deployment engineer is planning external networks for Diameter, LDAP, Trigger, and SS7 pods. Which component is responsible for assigning external network IPs to pods?</t>
         </is>
       </c>
+      <c r="AH19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3760,6 +3778,7 @@
           <t>[Deployment &amp; Troubleshooting] A troubleshooting engineer needs to inspect event logs captured inside the OAM container for a specific service. Which log should be checked?</t>
         </is>
       </c>
+      <c r="AH20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3927,6 +3946,7 @@
           <t>[HSS Basics] Several CNF services cannot locate each other after a cluster restart. Which component provides internal service discovery?</t>
         </is>
       </c>
+      <c r="AH21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4094,6 +4114,7 @@
           <t>[HSS Basics] A telecom operator observes that one HSS-CP instance is overloaded while others remain idle. Which service should be verified to ensure traffic is evenly distributed across all HSS-CP instances?</t>
         </is>
       </c>
+      <c r="AH22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4261,6 +4282,7 @@
           <t>[UDM Planning] The security team wants CSR to be handled with an integrated External rootCA when External CA is enabled. Which mechanism supports this?</t>
         </is>
       </c>
+      <c r="AH23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -4428,6 +4450,7 @@
           <t>[HSS Troubleshooting] NCOM reports: No valid repository configured or found for CaaS. What should be done?</t>
         </is>
       </c>
+      <c r="AH24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4595,6 +4618,7 @@
           <t>[HSS Basics] During IMS registration, communication is required between the HSS and the S-CSCF. Which interface supports this communication?</t>
         </is>
       </c>
+      <c r="AH25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4762,6 +4786,7 @@
           <t>[EIR Planning] What is the main focus of the CIQ document, as distinct from the DNP?</t>
         </is>
       </c>
+      <c r="AH26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4929,6 +4954,7 @@
           <t>[HSS Basics] A PCRF needs to store and retrieve subscriber policy-related data from HSS. Which interface should be used?</t>
         </is>
       </c>
+      <c r="AH27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -5096,6 +5122,7 @@
           <t>[HSS Basics] Before delivering an SMS to a subscriber, an SMSC needs routing information from HSS. Which interface is used?</t>
         </is>
       </c>
+      <c r="AH28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -5263,6 +5290,7 @@
           <t>[HSS Troubleshooting] A pod registration check shows envoy status: false. What does this indicate?</t>
         </is>
       </c>
+      <c r="AH29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -5430,6 +5458,7 @@
           <t>[UDM Planning] Planning an in-service software upgrade, the team wants automated pre- and post-upgrade validation. Which mechanism is used for CNF health checks in this feature?</t>
         </is>
       </c>
+      <c r="AH30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -5597,6 +5626,7 @@
           <t>[Basic SDL] A customer wants to move from traditional VNF architecture to cloud-native deployment. Which SDL architecture supports this model?</t>
         </is>
       </c>
+      <c r="AH31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -5764,6 +5794,7 @@
           <t>[Deployment &amp; Troubleshooting] Filesystem utilization alarms are generated. Which command provides disk usage information?</t>
         </is>
       </c>
+      <c r="AH32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -5931,6 +5962,7 @@
           <t>[Basic SDL] A customer wants to move from traditional VNF architecture to cloud-native deployment. Which SDL architecture supports this model?</t>
         </is>
       </c>
+      <c r="AH33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -6098,6 +6130,7 @@
           <t>[Deployment &amp; Troubleshooting] Post deployment where can we check our VM status?</t>
         </is>
       </c>
+      <c r="AH34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -6265,6 +6298,7 @@
           <t>[Basic NDS] An L2 engineer is performing root cause analysis after repeated service outages. Which VM provides diagnostic tools and health checks?</t>
         </is>
       </c>
+      <c r="AH35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -6432,6 +6466,7 @@
           <t>[Basic SDL] An engineer needs to manage SDL lifecycle operations such as scaling and upgrades. Which VM provides these capabilities?</t>
         </is>
       </c>
+      <c r="AH36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -6599,6 +6634,7 @@
           <t>[Basic SDL] An L2 engineer is performing root cause analysis after repeated service outages. Which VM provides diagnostic tools and health checks?</t>
         </is>
       </c>
+      <c r="AH37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -6766,6 +6802,7 @@
           <t>[Basic SDL] A customer migration project specifically requires synchronization between legacy and SDL databases. Which VM is mandatory?</t>
         </is>
       </c>
+      <c r="AH38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -6933,6 +6970,7 @@
           <t>[Planning &amp; Artifact Preparation] Which document provides the detailed customer network information used for design preparation?</t>
         </is>
       </c>
+      <c r="AH39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -7100,6 +7138,7 @@
           <t>[Planning &amp; Artifact Preparation] Incorrect sizing information mainly impacts which area?</t>
         </is>
       </c>
+      <c r="AH40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -7267,6 +7306,7 @@
           <t>[Deployment &amp; Troubleshooting] SDL instantiation has completed, but verification is required. What should the output show?</t>
         </is>
       </c>
+      <c r="AH41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -7434,6 +7474,7 @@
           <t>[Basic SDL] A storage node failure occurs. Which SDL component is responsible for data durability and recovery?</t>
         </is>
       </c>
+      <c r="AH42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -7601,6 +7642,7 @@
           <t>[Planning &amp; Artifact Preparation] Why is CIQ important for SDL deployment?</t>
         </is>
       </c>
+      <c r="AH43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -7768,6 +7810,7 @@
           <t>[Planning &amp; Artifact Preparation] A customer updates network architecture after the design has been finalized. Which documents may require updates?</t>
         </is>
       </c>
+      <c r="AH44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -7935,6 +7978,7 @@
           <t>[Basic SDL] NetAct is not receiving PM/FM statistics although subscriber operations are functioning normally. Which VM should be checked?</t>
         </is>
       </c>
+      <c r="AH45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -8102,6 +8146,7 @@
           <t>[Deployment &amp; Troubleshooting] Filesystem utilization alarms are generated. Which command provides disk usage information?</t>
         </is>
       </c>
+      <c r="AH46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -8269,6 +8314,7 @@
           <t>[Deployment &amp; Troubleshooting] Several components appear in UNKNOWN state. Which information source should be checked first?</t>
         </is>
       </c>
+      <c r="AH47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -8436,6 +8482,7 @@
           <t>[Deployment &amp; Troubleshooting] Replication alarms are reported on Storage VMs. Which command should be checked first?</t>
         </is>
       </c>
+      <c r="AH48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -8603,6 +8650,7 @@
           <t>[Planning &amp; Artifact Preparation] The customer changes interface VLANs after DND approval. What action is required?</t>
         </is>
       </c>
+      <c r="AH49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -8770,6 +8818,7 @@
           <t>[Planning &amp; Artifact Preparation] The customer provided an incomplete network design sheet without VLAN details. Which document should be revisited first?</t>
         </is>
       </c>
+      <c r="AH50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -8937,6 +8986,7 @@
           <t>[Deployment &amp; Troubleshooting] A complete health assessment of SDL is required. Which command should be executed?</t>
         </is>
       </c>
+      <c r="AH51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -9104,6 +9154,7 @@
           <t>[Deployment &amp; Troubleshooting] After deployment, an engineer wants to verify that SDL services are running on all VMs. Which command should be used?</t>
         </is>
       </c>
+      <c r="AH52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -9271,6 +9322,7 @@
           <t>[Basic SDL] An L2 engineer is performing root cause analysis after repeated service outages. Which VM provides diagnostic tools and health checks?</t>
         </is>
       </c>
+      <c r="AH53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -9438,6 +9490,7 @@
           <t>[HSS Basics] An external system needs access to subscriber information stored in One-NDS/SDL while hiding internal business logic services. Which component should be used?</t>
         </is>
       </c>
+      <c r="AH54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -9605,6 +9658,7 @@
           <t>[Basic SDL] A storage node failure occurs. Which SDL component is responsible for data durability and recovery?</t>
         </is>
       </c>
+      <c r="AH55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -9772,6 +9826,7 @@
           <t>[Basic SDL] During a capacity planning workshop, the customer expects subscriber growth to double within a year. Which SDL components are typically scaled to handle increased load?</t>
         </is>
       </c>
+      <c r="AH56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -9939,6 +9994,7 @@
           <t>[Deployment &amp; Troubleshooting] SDL bootstrap is suspected to be stuck. Which script should be executed?</t>
         </is>
       </c>
+      <c r="AH57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -10106,6 +10162,7 @@
           <t>[Deployment &amp; Troubleshooting] After running a health check report, what should ideally be displayed?</t>
         </is>
       </c>
+      <c r="AH58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -10273,6 +10330,7 @@
           <t>[UDM Planning] A deployment requires direct NF-to-NF communication without depending on NRF or SCP availability. Which model should be planned for this requirement?</t>
         </is>
       </c>
+      <c r="AH59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -10440,6 +10498,7 @@
           <t>[HSS Basics] The CNF must communicate with management systems through ZTS services instead of directly connecting to EMS/NMS. Which service supports this integration?</t>
         </is>
       </c>
+      <c r="AH60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -10607,6 +10666,7 @@
           <t>[UDM Planning] A planning discussion on rolling upgrades and node draining introduces a function that guarantees a minimum number of available Pods. What is this called?</t>
         </is>
       </c>
+      <c r="AH61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -10774,6 +10834,7 @@
           <t>[EIR Basic] Besides reducing IP requirements, which additional benefit does the centralized HTTP/2 LB provide?</t>
         </is>
       </c>
+      <c r="AH62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -10941,6 +11002,7 @@
           <t>[UDM Basic] A design review lists 5G core NFs. Which pair correctly represents AUSF_UDM's supported network functions?</t>
         </is>
       </c>
+      <c r="AH63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -11108,6 +11170,7 @@
           <t>[UDM Basic] Which service generates Authentication vectors for AKA based authentications and also supports Ki re-encryption?</t>
         </is>
       </c>
+      <c r="AH64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -11443,6 +11506,7 @@
           <t>[UDM Planning] A capacity design session covers cluster node types used by AUSF_UDM on NCS. Which node types are used?</t>
         </is>
       </c>
+      <c r="AH66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -11610,6 +11674,7 @@
           <t>[UDM Planning] A security planning session discusses which Kubernetes-level policy objects define security conditions for Pods.</t>
         </is>
       </c>
+      <c r="AH67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -11777,6 +11842,7 @@
           <t>[HSS Troubleshooting] The SS7 Telesys process is down. What should be checked first?</t>
         </is>
       </c>
+      <c r="AH68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -11944,6 +12010,7 @@
           <t>[HSS Basics] Several CNF services cannot locate each other after a cluster restart. Which component provides internal service discovery?</t>
         </is>
       </c>
+      <c r="AH69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -12111,6 +12178,7 @@
           <t>[HSS Troubleshooting] A pod is stuck in ImagePullBackOff or ErrImagePull. What is the recommended corrective action?</t>
         </is>
       </c>
+      <c r="AH70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -12278,6 +12346,7 @@
           <t>[Deployment &amp; Troubleshooting] An autoscaling design uses HPA with which primary metric to trigger scale-out or scale-in decisions?</t>
         </is>
       </c>
+      <c r="AH71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -12445,6 +12514,7 @@
           <t>[Deployment &amp; Troubleshooting] Traffic is still being routed to a Pod that is not actually ready to serve requests. Which probe should be checked to correct this?</t>
         </is>
       </c>
+      <c r="AH72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -12612,6 +12682,7 @@
           <t>[HSS Basics] A 5G core deployment requires interworking between a UDM and HSS. Which proprietary Diameter interface supports this requirement?</t>
         </is>
       </c>
+      <c r="AH73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -12779,6 +12850,7 @@
           <t>[UDM Basic] SMS Function needs to register its address and retrieve SMS management subscription data from UDM. Which interface is used?</t>
         </is>
       </c>
+      <c r="AH74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -12946,6 +13018,7 @@
           <t>[Deployment &amp; Troubleshooting] A process heap size configuration file defines thresholds like HEAP_SIZE_CRITICAL and HEAP_SIZE_MAJOR. What action is taken if a process exceeds the critical threshold?</t>
         </is>
       </c>
+      <c r="AH75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -13113,6 +13186,7 @@
           <t>[HSS Troubleshooting] A pod registration check shows envoy status: false. What does this indicate?</t>
         </is>
       </c>
+      <c r="AH76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -13280,6 +13354,7 @@
           <t>[HSS Deployment] The operator wants to run CNF health checks using Helm test or NCOM GUI. Which parameter should be enabled?</t>
         </is>
       </c>
+      <c r="AH77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -13447,6 +13522,7 @@
           <t>[HSS Troubleshooting] A pod registration check shows envoy status: false. What does this indicate?</t>
         </is>
       </c>
+      <c r="AH78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -13614,6 +13690,7 @@
           <t>[HSS Basics] A 5G core deployment requires interworking between a UDM and HSS. Which proprietary Diameter interface supports this requirement?</t>
         </is>
       </c>
+      <c r="AH79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -13781,6 +13858,7 @@
           <t>[HSS Troubleshooting] The HLRCallP pod continuously raises a No Free Dialogue alarm for a DP process. What is the recommended recovery action?</t>
         </is>
       </c>
+      <c r="AH80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -13948,6 +14026,7 @@
           <t>[HSS Troubleshooting] NCOM reports: No valid repository configured or found for CaaS. What should be done?</t>
         </is>
       </c>
+      <c r="AH81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -14115,6 +14194,7 @@
           <t>[Deployment &amp; Troubleshooting] After running a health check report, what should ideally be displayed?</t>
         </is>
       </c>
+      <c r="AH82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -14127,6 +14207,7 @@
           <t>Sanjay Kumar Gupta</t>
         </is>
       </c>
+      <c r="C83" t="inlineStr"/>
       <c r="D83" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -14277,6 +14358,7 @@
           <t>Attach ok but PDN fails. Check?</t>
         </is>
       </c>
+      <c r="AH83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -14289,6 +14371,7 @@
           <t>Bharanidharan</t>
         </is>
       </c>
+      <c r="C84" t="inlineStr"/>
       <c r="D84" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -14439,6 +14522,7 @@
           <t>Purpose of S1-AP on S1-MME?</t>
         </is>
       </c>
+      <c r="AH84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -14451,6 +14535,7 @@
           <t>J Mohammed Sheik Afridi</t>
         </is>
       </c>
+      <c r="C85" t="inlineStr"/>
       <c r="D85" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -14601,6 +14686,7 @@
           <t>Attach ok but PDN fails. Check?</t>
         </is>
       </c>
+      <c r="AH85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -14613,6 +14699,7 @@
           <t>Divyanshu Chauhan</t>
         </is>
       </c>
+      <c r="C86" t="inlineStr"/>
       <c r="D86" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -14763,6 +14850,7 @@
           <t>What is a major functional benefit of CMG in packet core?</t>
         </is>
       </c>
+      <c r="AH86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -14775,6 +14863,7 @@
           <t>Chitrangada Mishra</t>
         </is>
       </c>
+      <c r="C87" t="inlineStr"/>
       <c r="D87" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -14925,6 +15014,7 @@
           <t>In 4G LTE, CMM most commonly provides which network function?</t>
         </is>
       </c>
+      <c r="AH87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -14937,6 +15027,7 @@
           <t>Vibhor Chandra Gupta</t>
         </is>
       </c>
+      <c r="C88" t="inlineStr"/>
       <c r="D88" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -15087,6 +15178,7 @@
           <t>Which CMM component is responsible for OAM functions and northbound interfaces?</t>
         </is>
       </c>
+      <c r="AH88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -15099,6 +15191,7 @@
           <t>Nishu Kumar</t>
         </is>
       </c>
+      <c r="C89" t="inlineStr"/>
       <c r="D89" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -15249,6 +15342,7 @@
           <t>Which technology is highlighted in CMM for performance optimization on x86 platforms?</t>
         </is>
       </c>
+      <c r="AH89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -15261,6 +15355,7 @@
           <t>Satheeshkumar</t>
         </is>
       </c>
+      <c r="C90" t="inlineStr"/>
       <c r="D90" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -15411,6 +15506,7 @@
           <t>In a 4G ATP scenario, what does successful bearer establishment mainly confirm?</t>
         </is>
       </c>
+      <c r="AH90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -15423,6 +15519,7 @@
           <t>Chandan Kumar Singh</t>
         </is>
       </c>
+      <c r="C91" t="inlineStr"/>
       <c r="D91" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -15573,6 +15670,7 @@
           <t>What is a major functional benefit of CMG in packet core?</t>
         </is>
       </c>
+      <c r="AH91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -15585,6 +15683,7 @@
           <t>Sourabh  Khandelwal</t>
         </is>
       </c>
+      <c r="C92" t="inlineStr"/>
       <c r="D92" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -15735,6 +15834,7 @@
           <t>CMG is best described as:</t>
         </is>
       </c>
+      <c r="AH92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -15747,6 +15847,7 @@
           <t>Prateek</t>
         </is>
       </c>
+      <c r="C93" t="inlineStr"/>
       <c r="D93" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -15897,6 +15998,7 @@
           <t>CMM is described by Nokia as having what kind of architecture?</t>
         </is>
       </c>
+      <c r="AH93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -15909,6 +16011,7 @@
           <t>Veerasami</t>
         </is>
       </c>
+      <c r="C94" t="inlineStr"/>
       <c r="D94" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -16059,6 +16162,7 @@
           <t>In 4G LTE, CMM most commonly provides which network function?</t>
         </is>
       </c>
+      <c r="AH94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -16071,6 +16175,7 @@
           <t>Parth Saxena</t>
         </is>
       </c>
+      <c r="C95" t="inlineStr"/>
       <c r="D95" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -16221,6 +16326,7 @@
           <t>CMG supports evolution toward which major core direction?</t>
         </is>
       </c>
+      <c r="AH95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -16233,6 +16339,7 @@
           <t>Satya Prakash Rai</t>
         </is>
       </c>
+      <c r="C96" t="inlineStr"/>
       <c r="D96" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -16383,6 +16490,7 @@
           <t>Purpose of S1-AP on S1-MME?</t>
         </is>
       </c>
+      <c r="AH96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -16395,6 +16503,7 @@
           <t>Meenatchi M</t>
         </is>
       </c>
+      <c r="C97" t="inlineStr"/>
       <c r="D97" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -16545,6 +16654,7 @@
           <t>Which network function is most directly linked to slice selection in NRD-related architecture?</t>
         </is>
       </c>
+      <c r="AH97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -16557,6 +16667,7 @@
           <t>Sunilkumaar Selvaraajan</t>
         </is>
       </c>
+      <c r="C98" t="inlineStr"/>
       <c r="D98" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -16707,6 +16818,7 @@
           <t>What is the primary purpose of Nokia Resource Director (NRD)?</t>
         </is>
       </c>
+      <c r="AH98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -16719,6 +16831,7 @@
           <t>Ashwini Raju</t>
         </is>
       </c>
+      <c r="C99" t="inlineStr"/>
       <c r="D99" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -16869,6 +16982,7 @@
           <t>Which deployment characteristic is strongly associated with CMG?</t>
         </is>
       </c>
+      <c r="AH99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -16881,6 +16995,7 @@
           <t>Sunil Kumar Patel</t>
         </is>
       </c>
+      <c r="C100" t="inlineStr"/>
       <c r="D100" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -17031,6 +17146,7 @@
           <t>Which deployment characteristic is strongly associated with CMG?</t>
         </is>
       </c>
+      <c r="AH100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -17043,6 +17159,7 @@
           <t>Naveenkumar</t>
         </is>
       </c>
+      <c r="C101" t="inlineStr"/>
       <c r="D101" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -17193,6 +17310,7 @@
           <t>What is a major functional benefit of CMG in packet core?</t>
         </is>
       </c>
+      <c r="AH101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -17205,6 +17323,7 @@
           <t>G  Koushik</t>
         </is>
       </c>
+      <c r="C102" t="inlineStr"/>
       <c r="D102" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -17355,6 +17474,7 @@
           <t>CMM is described by Nokia as having what kind of architecture?</t>
         </is>
       </c>
+      <c r="AH102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -17367,6 +17487,7 @@
           <t>Kapil Chaudhary</t>
         </is>
       </c>
+      <c r="C103" t="inlineStr"/>
       <c r="D103" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -17517,6 +17638,7 @@
           <t>Successful ATP indication?</t>
         </is>
       </c>
+      <c r="AH103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -17529,6 +17651,7 @@
           <t>Aryan Kumar</t>
         </is>
       </c>
+      <c r="C104" t="inlineStr"/>
       <c r="D104" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -17679,6 +17802,7 @@
           <t>CMG supports evolution toward which major core direction?</t>
         </is>
       </c>
+      <c r="AH104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -17691,6 +17815,7 @@
           <t>Pratik Raj</t>
         </is>
       </c>
+      <c r="C105" t="inlineStr"/>
       <c r="D105" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -17841,6 +17966,7 @@
           <t>Which ATP case is useful for validating CMG resilience?</t>
         </is>
       </c>
+      <c r="AH105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -17853,6 +17979,7 @@
           <t>Ezhilarasan</t>
         </is>
       </c>
+      <c r="C106" t="inlineStr"/>
       <c r="D106" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -18003,6 +18130,7 @@
           <t>Which protocols relate to CMM control plane?</t>
         </is>
       </c>
+      <c r="AH106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -18015,6 +18143,7 @@
           <t>Santosh Kumar</t>
         </is>
       </c>
+      <c r="C107" t="inlineStr"/>
       <c r="D107" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -18165,6 +18294,7 @@
           <t>CMG is best described as:</t>
         </is>
       </c>
+      <c r="AH107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -18177,6 +18307,7 @@
           <t>Srinath</t>
         </is>
       </c>
+      <c r="C108" t="inlineStr"/>
       <c r="D108" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -18327,6 +18458,7 @@
           <t>Which interface is key for LTE access during ATP?</t>
         </is>
       </c>
+      <c r="AH108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -18339,6 +18471,7 @@
           <t>Kiruthika V</t>
         </is>
       </c>
+      <c r="C109" t="inlineStr"/>
       <c r="D109" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -18489,6 +18622,7 @@
           <t>Which ATP case is useful for validating CMG resilience?</t>
         </is>
       </c>
+      <c r="AH109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -18501,6 +18635,7 @@
           <t>Pratyasa Mohanty</t>
         </is>
       </c>
+      <c r="C110" t="inlineStr"/>
       <c r="D110" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -18651,6 +18786,7 @@
           <t>Which Nokia platform is commonly used for CMM management?</t>
         </is>
       </c>
+      <c r="AH110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -18663,6 +18799,7 @@
           <t>Soumya Smruti Das</t>
         </is>
       </c>
+      <c r="C111" t="inlineStr"/>
       <c r="D111" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -18813,6 +18950,7 @@
           <t>Which outcome indicates a successful CMG onboarding and integration cycle?</t>
         </is>
       </c>
+      <c r="AH111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -18825,6 +18963,7 @@
           <t>Pratyusha Pattanaik</t>
         </is>
       </c>
+      <c r="C112" t="inlineStr"/>
       <c r="D112" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -18975,6 +19114,7 @@
           <t>Which CMM component provides logical interface termination for GTP and Diameter?</t>
         </is>
       </c>
+      <c r="AH112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -18987,6 +19127,7 @@
           <t>Ashutosh</t>
         </is>
       </c>
+      <c r="C113" t="inlineStr"/>
       <c r="D113" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -19137,6 +19278,7 @@
           <t>Which technology is highlighted in CMM for performance optimization on x86 platforms?</t>
         </is>
       </c>
+      <c r="AH113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -19149,6 +19291,7 @@
           <t>Gudluru Lakshmi Narayan</t>
         </is>
       </c>
+      <c r="C114" t="inlineStr"/>
       <c r="D114" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -19299,6 +19442,7 @@
           <t>CMG is best described as:</t>
         </is>
       </c>
+      <c r="AH114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -19311,6 +19455,7 @@
           <t>Madanuru Vishnu Charan</t>
         </is>
       </c>
+      <c r="C115" t="inlineStr"/>
       <c r="D115" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -19461,6 +19606,7 @@
           <t>What is critical to validate for mobility in ATP?</t>
         </is>
       </c>
+      <c r="AH115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -19473,6 +19619,7 @@
           <t>Abhisek Mohanty</t>
         </is>
       </c>
+      <c r="C116" t="inlineStr"/>
       <c r="D116" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -19623,6 +19770,7 @@
           <t>In 4G LTE, CMM most commonly provides which network function?</t>
         </is>
       </c>
+      <c r="AH116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -19635,6 +19783,7 @@
           <t>Avipsa Mohanty</t>
         </is>
       </c>
+      <c r="C117" t="inlineStr"/>
       <c r="D117" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -19785,6 +19934,7 @@
           <t>What is the primary role of Nokia Cloud Mobility Manager (CMM) in a 4G packet core?</t>
         </is>
       </c>
+      <c r="AH117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -19797,6 +19947,7 @@
           <t>Debasish Jena</t>
         </is>
       </c>
+      <c r="C118" t="inlineStr"/>
       <c r="D118" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -19947,6 +20098,7 @@
           <t>Which protocols relate to CMM control plane?</t>
         </is>
       </c>
+      <c r="AH118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -19959,6 +20111,7 @@
           <t>PRITISARATHI BHUYAN</t>
         </is>
       </c>
+      <c r="C119" t="inlineStr"/>
       <c r="D119" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -20109,6 +20262,7 @@
           <t>Best failover ATP test?</t>
         </is>
       </c>
+      <c r="AH119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -20121,6 +20275,7 @@
           <t>Anchal Priyadarshini Swain</t>
         </is>
       </c>
+      <c r="C120" t="inlineStr"/>
       <c r="D120" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -20271,6 +20426,7 @@
           <t>CMG is part of which Nokia family?</t>
         </is>
       </c>
+      <c r="AH120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -20283,6 +20439,7 @@
           <t>Sasmita GIRI</t>
         </is>
       </c>
+      <c r="C121" t="inlineStr"/>
       <c r="D121" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -20433,6 +20590,7 @@
           <t>Which protocols relate to CMM control plane?</t>
         </is>
       </c>
+      <c r="AH121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -20445,6 +20603,7 @@
           <t>Akankshya Rout</t>
         </is>
       </c>
+      <c r="C122" t="inlineStr"/>
       <c r="D122" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -20595,6 +20754,7 @@
           <t>What does NECC stand for in Nokia CMM architecture?</t>
         </is>
       </c>
+      <c r="AH122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -20607,6 +20767,7 @@
           <t>Ajaya Narayan Nayak</t>
         </is>
       </c>
+      <c r="C123" t="inlineStr"/>
       <c r="D123" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -20757,6 +20918,7 @@
           <t>Purpose of S1-AP on S1-MME?</t>
         </is>
       </c>
+      <c r="AH123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -20769,6 +20931,7 @@
           <t>Soumya Ranjan Das</t>
         </is>
       </c>
+      <c r="C124" t="inlineStr"/>
       <c r="D124" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -20919,6 +21082,7 @@
           <t>Purpose of S1-AP on S1-MME?</t>
         </is>
       </c>
+      <c r="AH124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -20931,6 +21095,7 @@
           <t>Vaghela Rahul Rameshbhai</t>
         </is>
       </c>
+      <c r="C125" t="inlineStr"/>
       <c r="D125" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -21081,6 +21246,7 @@
           <t>CMG is best described as:</t>
         </is>
       </c>
+      <c r="AH125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -21093,6 +21259,7 @@
           <t>Asish Nayak</t>
         </is>
       </c>
+      <c r="C126" t="inlineStr"/>
       <c r="D126" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -21243,6 +21410,7 @@
           <t>What is a major functional benefit of CMG in packet core?</t>
         </is>
       </c>
+      <c r="AH126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -21255,6 +21423,7 @@
           <t>Bibhash Dash</t>
         </is>
       </c>
+      <c r="C127" t="inlineStr"/>
       <c r="D127" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -21405,6 +21574,7 @@
           <t>CMM is described by Nokia as having what kind of architecture?</t>
         </is>
       </c>
+      <c r="AH127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -21417,6 +21587,7 @@
           <t>Omm  Sai Roumya RANJAN</t>
         </is>
       </c>
+      <c r="C128" t="inlineStr"/>
       <c r="D128" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -21567,6 +21738,7 @@
           <t>Which aspect is most important during CMG onboarding?</t>
         </is>
       </c>
+      <c r="AH128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -21579,6 +21751,7 @@
           <t>Pradyumna Naik</t>
         </is>
       </c>
+      <c r="C129" t="inlineStr"/>
       <c r="D129" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -21729,6 +21902,7 @@
           <t>CMG is part of which Nokia family?</t>
         </is>
       </c>
+      <c r="AH129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -21741,6 +21915,7 @@
           <t>Abdul Basith Shaik</t>
         </is>
       </c>
+      <c r="C130" t="inlineStr"/>
       <c r="D130" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -21891,6 +22066,7 @@
           <t>Attach succeeds but bearer fails. Likely issue?</t>
         </is>
       </c>
+      <c r="AH130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -21903,6 +22079,7 @@
           <t>Solanki Jigar Ambalal</t>
         </is>
       </c>
+      <c r="C131" t="inlineStr"/>
       <c r="D131" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -22053,6 +22230,7 @@
           <t>Attach ok but PDN fails. Check?</t>
         </is>
       </c>
+      <c r="AH131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -22065,6 +22243,7 @@
           <t>Akash Bairagi</t>
         </is>
       </c>
+      <c r="C132" t="inlineStr"/>
       <c r="D132" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -22215,6 +22394,7 @@
           <t>In a 4G ATP scenario, what does successful bearer establishment mainly confirm?</t>
         </is>
       </c>
+      <c r="AH132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -22227,6 +22407,7 @@
           <t>Anand Babu</t>
         </is>
       </c>
+      <c r="C133" t="inlineStr"/>
       <c r="D133" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -22377,6 +22558,7 @@
           <t>Which protocols relate to CMM control plane?</t>
         </is>
       </c>
+      <c r="AH133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -22389,6 +22571,7 @@
           <t>Chelsea Shalin S</t>
         </is>
       </c>
+      <c r="C134" t="inlineStr"/>
       <c r="D134" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -22539,6 +22722,7 @@
           <t>CMM supports which management interfaces for operations and troubleshooting?</t>
         </is>
       </c>
+      <c r="AH134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -22551,6 +22735,7 @@
           <t>Gopi K</t>
         </is>
       </c>
+      <c r="C135" t="inlineStr"/>
       <c r="D135" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -22701,6 +22886,7 @@
           <t>Purpose of S1-AP on S1-MME?</t>
         </is>
       </c>
+      <c r="AH135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -22713,6 +22899,7 @@
           <t>Malan Subbiah Pandian</t>
         </is>
       </c>
+      <c r="C136" t="inlineStr"/>
       <c r="D136" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -22863,6 +23050,7 @@
           <t>Which is a common integration point for CMG in EPC?</t>
         </is>
       </c>
+      <c r="AH136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -22875,6 +23063,7 @@
           <t>R Krishna Durga</t>
         </is>
       </c>
+      <c r="C137" t="inlineStr"/>
       <c r="D137" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -23025,6 +23214,7 @@
           <t>Purpose of S1-AP on S1-MME?</t>
         </is>
       </c>
+      <c r="AH137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -23037,6 +23227,7 @@
           <t>Sabari Murugesan</t>
         </is>
       </c>
+      <c r="C138" t="inlineStr"/>
       <c r="D138" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -23187,6 +23378,7 @@
           <t>CMM is described by Nokia as having what kind of architecture?</t>
         </is>
       </c>
+      <c r="AH138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -23199,6 +23391,7 @@
           <t>Surya Saravanan</t>
         </is>
       </c>
+      <c r="C139" t="inlineStr"/>
       <c r="D139" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -23349,6 +23542,7 @@
           <t>What is the key purpose of ATP testing for CMG?</t>
         </is>
       </c>
+      <c r="AH139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -23361,6 +23555,7 @@
           <t>Yogaverma V</t>
         </is>
       </c>
+      <c r="C140" t="inlineStr"/>
       <c r="D140" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -23511,6 +23706,7 @@
           <t>Which scenario best tests CMG under mobility conditions?</t>
         </is>
       </c>
+      <c r="AH140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -23523,6 +23719,7 @@
           <t>Varun Pachauri</t>
         </is>
       </c>
+      <c r="C141" t="inlineStr"/>
       <c r="D141" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -23673,6 +23870,7 @@
           <t>CMG supports evolution toward which major core direction?</t>
         </is>
       </c>
+      <c r="AH141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -23685,6 +23883,7 @@
           <t>Buran Sagari Sohail Basha</t>
         </is>
       </c>
+      <c r="C142" t="inlineStr"/>
       <c r="D142" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -23835,6 +24034,7 @@
           <t>Which protocols relate to CMM control plane?</t>
         </is>
       </c>
+      <c r="AH142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -23847,6 +24047,7 @@
           <t>Gadde Yaswanth</t>
         </is>
       </c>
+      <c r="C143" t="inlineStr"/>
       <c r="D143" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -23997,6 +24198,7 @@
           <t>Which Nokia platform is commonly used for CMM management?</t>
         </is>
       </c>
+      <c r="AH143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -24009,6 +24211,7 @@
           <t>Hariharan S</t>
         </is>
       </c>
+      <c r="C144" t="inlineStr"/>
       <c r="D144" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -24159,6 +24362,7 @@
           <t>What does NECC stand for in Nokia CMM architecture?</t>
         </is>
       </c>
+      <c r="AH144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -24171,6 +24375,7 @@
           <t>M Subramanayam</t>
         </is>
       </c>
+      <c r="C145" t="inlineStr"/>
       <c r="D145" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -24321,6 +24526,7 @@
           <t>CMM supports which management interfaces for operations and troubleshooting?</t>
         </is>
       </c>
+      <c r="AH145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -24333,6 +24539,7 @@
           <t>Nekkanti Mahendra Tulasi</t>
         </is>
       </c>
+      <c r="C146" t="inlineStr"/>
       <c r="D146" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -24483,6 +24690,7 @@
           <t>Which interface is key for LTE access during ATP?</t>
         </is>
       </c>
+      <c r="AH146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -24495,6 +24703,7 @@
           <t>V P Sandhiya</t>
         </is>
       </c>
+      <c r="C147" t="inlineStr"/>
       <c r="D147" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -24645,6 +24854,7 @@
           <t>Key onboarding activity for CMM?</t>
         </is>
       </c>
+      <c r="AH147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -24657,6 +24867,7 @@
           <t>Susheel kumar Dwivdi</t>
         </is>
       </c>
+      <c r="C148" t="inlineStr"/>
       <c r="D148" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -24807,6 +25018,7 @@
           <t>In a CMG ATP plan, which test most directly verifies end-user data service?</t>
         </is>
       </c>
+      <c r="AH148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -24819,6 +25031,7 @@
           <t>Vivek Mishra</t>
         </is>
       </c>
+      <c r="C149" t="inlineStr"/>
       <c r="D149" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -24969,6 +25182,7 @@
           <t>If attach succeeds but data service fails, which CMG area should be checked first?</t>
         </is>
       </c>
+      <c r="AH149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -24981,6 +25195,7 @@
           <t>Harshada Vitthal Shinde</t>
         </is>
       </c>
+      <c r="C150" t="inlineStr"/>
       <c r="D150" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -25131,6 +25346,7 @@
           <t>What is the primary role of Nokia Cloud Mobile Gateway (CMG) in packet core?</t>
         </is>
       </c>
+      <c r="AH150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -25143,6 +25359,7 @@
           <t>Nishant Kumar Lal</t>
         </is>
       </c>
+      <c r="C151" t="inlineStr"/>
       <c r="D151" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -25293,6 +25510,7 @@
           <t>What is critical to validate for mobility in ATP?</t>
         </is>
       </c>
+      <c r="AH151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -25305,6 +25523,7 @@
           <t>Vennela Korada</t>
         </is>
       </c>
+      <c r="C152" t="inlineStr"/>
       <c r="D152" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -25455,6 +25674,7 @@
           <t>In a CMG ATP plan, which test most directly verifies end-user data service?</t>
         </is>
       </c>
+      <c r="AH152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -25467,6 +25687,7 @@
           <t>Bommireddy Jaya Prakash Reddy</t>
         </is>
       </c>
+      <c r="C153" t="inlineStr"/>
       <c r="D153" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -25617,6 +25838,7 @@
           <t>Purpose of S1-AP on S1-MME?</t>
         </is>
       </c>
+      <c r="AH153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -25629,6 +25851,7 @@
           <t>Komala Mamidi</t>
         </is>
       </c>
+      <c r="C154" t="inlineStr"/>
       <c r="D154" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -25779,6 +26002,7 @@
           <t>CMM is described by Nokia as having what kind of architecture?</t>
         </is>
       </c>
+      <c r="AH154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -25791,6 +26015,7 @@
           <t>Sundram Kumar</t>
         </is>
       </c>
+      <c r="C155" t="inlineStr"/>
       <c r="D155" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -25941,6 +26166,7 @@
           <t>Key onboarding activity for CMM?</t>
         </is>
       </c>
+      <c r="AH155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -25953,6 +26179,7 @@
           <t>Abhishikha Chauhan</t>
         </is>
       </c>
+      <c r="C156" t="inlineStr"/>
       <c r="D156" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -26103,6 +26330,7 @@
           <t>Why is CMG considered operationally flexible?</t>
         </is>
       </c>
+      <c r="AH156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -26115,6 +26343,7 @@
           <t>Anipeddi Lasya</t>
         </is>
       </c>
+      <c r="C157" t="inlineStr"/>
       <c r="D157" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -26265,6 +26494,7 @@
           <t>Which CMM service hosts the MME functions?</t>
         </is>
       </c>
+      <c r="AH157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -26277,6 +26507,7 @@
           <t>Biruntha</t>
         </is>
       </c>
+      <c r="C158" t="inlineStr"/>
       <c r="D158" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -26427,6 +26658,7 @@
           <t>Which deployment characteristic is strongly associated with CMG?</t>
         </is>
       </c>
+      <c r="AH158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -26439,6 +26671,7 @@
           <t>Himanshu Bungla</t>
         </is>
       </c>
+      <c r="C159" t="inlineStr"/>
       <c r="D159" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -26589,6 +26822,7 @@
           <t>In a 5G ATP test, what should be verified first for NRD?</t>
         </is>
       </c>
+      <c r="AH159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -26601,6 +26835,7 @@
           <t>Nijampatnam Eswar</t>
         </is>
       </c>
+      <c r="C160" t="inlineStr"/>
       <c r="D160" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -26751,6 +26986,7 @@
           <t>What is a practical ATP objective for CMG interworking?</t>
         </is>
       </c>
+      <c r="AH160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -26763,6 +26999,7 @@
           <t>Saiyed Raza Imam</t>
         </is>
       </c>
+      <c r="C161" t="inlineStr"/>
       <c r="D161" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -26913,6 +27150,7 @@
           <t>Which ATP case is useful for validating CMG resilience?</t>
         </is>
       </c>
+      <c r="AH161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -26925,6 +27163,7 @@
           <t>Vaijinath Bhaskar Batule</t>
         </is>
       </c>
+      <c r="C162" t="inlineStr"/>
       <c r="D162" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -27075,6 +27314,7 @@
           <t>Why is CMG considered operationally flexible?</t>
         </is>
       </c>
+      <c r="AH162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -27087,6 +27327,7 @@
           <t>Kamal Kumar Ray</t>
         </is>
       </c>
+      <c r="C163" t="inlineStr"/>
       <c r="D163" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -27237,6 +27478,7 @@
           <t>Which CMM service hosts the MME functions?</t>
         </is>
       </c>
+      <c r="AH163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -27249,6 +27491,7 @@
           <t>Tanmoy Mojumder</t>
         </is>
       </c>
+      <c r="C164" t="inlineStr"/>
       <c r="D164" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -27399,6 +27642,7 @@
           <t>Which technology is highlighted in CMM for performance optimization on x86 platforms?</t>
         </is>
       </c>
+      <c r="AH164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -27411,6 +27655,7 @@
           <t>Shaikh Reshma</t>
         </is>
       </c>
+      <c r="C165" t="inlineStr"/>
       <c r="D165" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -27561,6 +27806,7 @@
           <t>Which CMM component is responsible for OAM functions and northbound interfaces?</t>
         </is>
       </c>
+      <c r="AH165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -27573,6 +27819,7 @@
           <t>Om Prakash Gautam</t>
         </is>
       </c>
+      <c r="C166" t="inlineStr"/>
       <c r="D166" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -27723,6 +27970,7 @@
           <t>What is the primary role of Nokia Cloud Mobile Gateway (CMG) in packet core?</t>
         </is>
       </c>
+      <c r="AH166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -27735,6 +27983,7 @@
           <t>Jaya Vohra</t>
         </is>
       </c>
+      <c r="C167" t="inlineStr"/>
       <c r="D167" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -27885,6 +28134,7 @@
           <t>CMG can support which access evolution model?</t>
         </is>
       </c>
+      <c r="AH167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -27897,6 +28147,7 @@
           <t>S Bijetananda Swain</t>
         </is>
       </c>
+      <c r="C168" t="inlineStr"/>
       <c r="D168" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -28047,6 +28298,7 @@
           <t>If attach succeeds but data service fails, which CMG area should be checked first?</t>
         </is>
       </c>
+      <c r="AH168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -28059,6 +28311,7 @@
           <t>Rohit Kumar</t>
         </is>
       </c>
+      <c r="C169" t="inlineStr"/>
       <c r="D169" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -28209,6 +28462,7 @@
           <t>Which is most likely to be verified in CMG acceptance for 4G?</t>
         </is>
       </c>
+      <c r="AH169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -28221,6 +28475,7 @@
           <t>Sujata Singh</t>
         </is>
       </c>
+      <c r="C170" t="inlineStr"/>
       <c r="D170" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -28371,6 +28626,7 @@
           <t>Why is CMG considered operationally flexible?</t>
         </is>
       </c>
+      <c r="AH170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -28383,6 +28639,7 @@
           <t>SUSHMA CHOLLETI</t>
         </is>
       </c>
+      <c r="C171" t="inlineStr"/>
       <c r="D171" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -28533,6 +28790,7 @@
           <t>Why is CMG considered operationally flexible?</t>
         </is>
       </c>
+      <c r="AH171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -28545,6 +28803,7 @@
           <t>Gaurav Verma</t>
         </is>
       </c>
+      <c r="C172" t="inlineStr"/>
       <c r="D172" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -28695,6 +28954,7 @@
           <t>CMG can support which access evolution model?</t>
         </is>
       </c>
+      <c r="AH172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -28707,6 +28967,7 @@
           <t>Kamna Peyal</t>
         </is>
       </c>
+      <c r="C173" t="inlineStr"/>
       <c r="D173" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -28857,6 +29118,7 @@
           <t>Key onboarding activity for CMM?</t>
         </is>
       </c>
+      <c r="AH173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -28869,6 +29131,7 @@
           <t>Damarasinghu Vinay Kumar</t>
         </is>
       </c>
+      <c r="C174" t="inlineStr"/>
       <c r="D174" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -29019,6 +29282,7 @@
           <t>Which outcome indicates a successful CMG onboarding and integration cycle?</t>
         </is>
       </c>
+      <c r="AH174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -29031,6 +29295,7 @@
           <t>Devarapalli Siva Naga Srivalli</t>
         </is>
       </c>
+      <c r="C175" t="inlineStr"/>
       <c r="D175" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -29181,6 +29446,7 @@
           <t>Which ATP case is useful for validating CMG resilience?</t>
         </is>
       </c>
+      <c r="AH175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -29193,6 +29459,7 @@
           <t>Etakaati Chandan Srinivas</t>
         </is>
       </c>
+      <c r="C176" t="inlineStr"/>
       <c r="D176" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -29343,6 +29610,7 @@
           <t>Which scenario best tests CMG under mobility conditions?</t>
         </is>
       </c>
+      <c r="AH176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -29355,6 +29623,7 @@
           <t>Guttula Vaishnavi</t>
         </is>
       </c>
+      <c r="C177" t="inlineStr"/>
       <c r="D177" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -29505,6 +29774,7 @@
           <t>Attach ok but PDN fails. Check?</t>
         </is>
       </c>
+      <c r="AH177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -29517,6 +29787,7 @@
           <t>Hamsa Yaswanth Paul</t>
         </is>
       </c>
+      <c r="C178" t="inlineStr"/>
       <c r="D178" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -29667,6 +29938,7 @@
           <t>In 4G LTE, CMM most commonly provides which network function?</t>
         </is>
       </c>
+      <c r="AH178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -29679,6 +29951,7 @@
           <t>Kasi Nandini</t>
         </is>
       </c>
+      <c r="C179" t="inlineStr"/>
       <c r="D179" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -29829,6 +30102,7 @@
           <t>Attach fails after MME relocation. What is tested?</t>
         </is>
       </c>
+      <c r="AH179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -29841,6 +30115,7 @@
           <t>Lavanya Seerapu</t>
         </is>
       </c>
+      <c r="C180" t="inlineStr"/>
       <c r="D180" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -29991,6 +30266,7 @@
           <t>What is the best description of a Network Function Instance in NRD/SBA context?</t>
         </is>
       </c>
+      <c r="AH180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -30003,6 +30279,7 @@
           <t>Pappala Sai Kishor</t>
         </is>
       </c>
+      <c r="C181" t="inlineStr"/>
       <c r="D181" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -30153,6 +30430,7 @@
           <t>In a CMG ATP plan, which test most directly verifies end-user data service?</t>
         </is>
       </c>
+      <c r="AH181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -30165,6 +30443,7 @@
           <t>Rachabathula Deepthisri</t>
         </is>
       </c>
+      <c r="C182" t="inlineStr"/>
       <c r="D182" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -30315,6 +30594,7 @@
           <t>CMG supports evolution toward which major core direction?</t>
         </is>
       </c>
+      <c r="AH182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -30327,6 +30607,7 @@
           <t>Srujan Palla</t>
         </is>
       </c>
+      <c r="C183" t="inlineStr"/>
       <c r="D183" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -30477,6 +30758,7 @@
           <t>In a 4G ATP scenario, what does successful bearer establishment mainly confirm?</t>
         </is>
       </c>
+      <c r="AH183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -30489,6 +30771,7 @@
           <t>Swetha Konchada</t>
         </is>
       </c>
+      <c r="C184" t="inlineStr"/>
       <c r="D184" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -30639,6 +30922,7 @@
           <t>CMG supports evolution toward which major core direction?</t>
         </is>
       </c>
+      <c r="AH184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -30651,6 +30935,7 @@
           <t>Vivek Singh</t>
         </is>
       </c>
+      <c r="C185" t="inlineStr"/>
       <c r="D185" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -30801,6 +31086,7 @@
           <t>Which is a common integration point for CMG in EPC?</t>
         </is>
       </c>
+      <c r="AH185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -30813,6 +31099,7 @@
           <t>Akshit Sahni</t>
         </is>
       </c>
+      <c r="C186" t="inlineStr"/>
       <c r="D186" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -30963,6 +31250,7 @@
           <t>Which aspect is most important during CMG onboarding?</t>
         </is>
       </c>
+      <c r="AH186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -30975,6 +31263,7 @@
           <t>Abhiram Jagarlamudi</t>
         </is>
       </c>
+      <c r="C187" t="inlineStr"/>
       <c r="D187" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -31125,6 +31414,7 @@
           <t>Why is CMG considered operationally flexible?</t>
         </is>
       </c>
+      <c r="AH187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -31137,6 +31427,7 @@
           <t>Debopriyo Halder</t>
         </is>
       </c>
+      <c r="C188" t="inlineStr"/>
       <c r="D188" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -31287,6 +31578,7 @@
           <t>Which CMM service is associated with user-plane packet processing and data forwarding?</t>
         </is>
       </c>
+      <c r="AH188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -31299,6 +31591,7 @@
           <t>Alok Kumar Nayak</t>
         </is>
       </c>
+      <c r="C189" t="inlineStr"/>
       <c r="D189" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -31449,6 +31742,7 @@
           <t>Which ATP case is useful for validating CMG resilience?</t>
         </is>
       </c>
+      <c r="AH189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -31461,6 +31755,7 @@
           <t>Archit Bagulia</t>
         </is>
       </c>
+      <c r="C190" t="inlineStr"/>
       <c r="D190" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -31611,6 +31906,7 @@
           <t>Which design goal is central to NRD’s cloud-native approach?</t>
         </is>
       </c>
+      <c r="AH190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -31623,6 +31919,7 @@
           <t>Arunkumar Balappa Pattadakall</t>
         </is>
       </c>
+      <c r="C191" t="inlineStr"/>
       <c r="D191" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -31773,6 +32070,7 @@
           <t>Successful ATP indication?</t>
         </is>
       </c>
+      <c r="AH191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -31785,6 +32083,7 @@
           <t>Dewashish Kumar</t>
         </is>
       </c>
+      <c r="C192" t="inlineStr"/>
       <c r="D192" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -31935,6 +32234,7 @@
           <t>Which design goal is central to NRD’s cloud-native approach?</t>
         </is>
       </c>
+      <c r="AH192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -31947,6 +32247,7 @@
           <t>Subhankar Hazra</t>
         </is>
       </c>
+      <c r="C193" t="inlineStr"/>
       <c r="D193" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -32097,6 +32398,7 @@
           <t>Attach fails after MME relocation. What is tested?</t>
         </is>
       </c>
+      <c r="AH193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -32109,6 +32411,7 @@
           <t>Ajay Kumar</t>
         </is>
       </c>
+      <c r="C194" t="inlineStr"/>
       <c r="D194" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -32259,6 +32562,7 @@
           <t>In a 4G ATP scenario, what does successful bearer establishment mainly confirm?</t>
         </is>
       </c>
+      <c r="AH194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -32271,6 +32575,7 @@
           <t>Altamash Ashfaq</t>
         </is>
       </c>
+      <c r="C195" t="inlineStr"/>
       <c r="D195" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -32421,6 +32726,7 @@
           <t>What is the best description of a Network Function Instance in NRD/SBA context?</t>
         </is>
       </c>
+      <c r="AH195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -32433,6 +32739,7 @@
           <t>Preetam Mehta</t>
         </is>
       </c>
+      <c r="C196" t="inlineStr"/>
       <c r="D196" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -32583,6 +32890,7 @@
           <t>Which protocol family is most relevant to CMG integration with EPC nodes?</t>
         </is>
       </c>
+      <c r="AH196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -32595,6 +32903,7 @@
           <t>Guru Prasad</t>
         </is>
       </c>
+      <c r="C197" t="inlineStr"/>
       <c r="D197" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -32745,6 +33054,7 @@
           <t>Which CMM service handles 2G/3G mobility and session management?</t>
         </is>
       </c>
+      <c r="AH197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -32757,6 +33067,7 @@
           <t>Raviraj Dhondiram Chalikwar</t>
         </is>
       </c>
+      <c r="C198" t="inlineStr"/>
       <c r="D198" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -32907,6 +33218,7 @@
           <t>Which protocol style is most aligned with NRD in an SBA environment?</t>
         </is>
       </c>
+      <c r="AH198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -32919,6 +33231,7 @@
           <t>Snehal Mavale</t>
         </is>
       </c>
+      <c r="C199" t="inlineStr"/>
       <c r="D199" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -33069,6 +33382,7 @@
           <t>Which lifecycle operations are associated with NRD CNF management?</t>
         </is>
       </c>
+      <c r="AH199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -33081,6 +33395,7 @@
           <t>Rakshitha K M</t>
         </is>
       </c>
+      <c r="C200" t="inlineStr"/>
       <c r="D200" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -33231,6 +33546,7 @@
           <t>Key onboarding activity for CMM?</t>
         </is>
       </c>
+      <c r="AH200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -33243,6 +33559,7 @@
           <t>Sakshi Srivastava</t>
         </is>
       </c>
+      <c r="C201" t="inlineStr"/>
       <c r="D201" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -33393,6 +33710,7 @@
           <t>Attach ok but PDN fails. Check?</t>
         </is>
       </c>
+      <c r="AH201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -33405,6 +33723,7 @@
           <t>Sukanya</t>
         </is>
       </c>
+      <c r="C202" t="inlineStr"/>
       <c r="D202" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -33555,6 +33874,7 @@
           <t>CMM is described by Nokia as having what kind of architecture?</t>
         </is>
       </c>
+      <c r="AH202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -33567,6 +33887,7 @@
           <t>Vijay Laxman Dhomase</t>
         </is>
       </c>
+      <c r="C203" t="inlineStr"/>
       <c r="D203" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -33717,6 +34038,7 @@
           <t>Which CMM service hosts the MME functions?</t>
         </is>
       </c>
+      <c r="AH203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -33729,6 +34051,7 @@
           <t>Angshuman Sarma</t>
         </is>
       </c>
+      <c r="C204" t="inlineStr"/>
       <c r="D204" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -33879,6 +34202,7 @@
           <t>What is the best description of a Network Function Instance in NRD/SBA context?</t>
         </is>
       </c>
+      <c r="AH204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -33891,6 +34215,7 @@
           <t>Nisha Kailas Mali</t>
         </is>
       </c>
+      <c r="C205" t="inlineStr"/>
       <c r="D205" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -34041,6 +34366,7 @@
           <t>Which is a common integration point for CMG in EPC?</t>
         </is>
       </c>
+      <c r="AH205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -34053,6 +34379,7 @@
           <t>Ravi Ranjan</t>
         </is>
       </c>
+      <c r="C206" t="inlineStr"/>
       <c r="D206" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -34203,6 +34530,7 @@
           <t>In 4G LTE, CMM most commonly provides which network function?</t>
         </is>
       </c>
+      <c r="AH206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -34215,6 +34543,7 @@
           <t>Sarjitkumar Rajyaguru</t>
         </is>
       </c>
+      <c r="C207" t="inlineStr"/>
       <c r="D207" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -34365,6 +34694,7 @@
           <t>Which symptom during ATP most likely indicates a control-plane integration problem?</t>
         </is>
       </c>
+      <c r="AH207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -34377,6 +34707,7 @@
           <t>Ajith V A</t>
         </is>
       </c>
+      <c r="C208" t="inlineStr"/>
       <c r="D208" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -34527,6 +34858,7 @@
           <t>Which CMM component provides logical interface termination for GTP and Diameter?</t>
         </is>
       </c>
+      <c r="AH208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -34539,6 +34871,7 @@
           <t>Sugat Bhalshankar</t>
         </is>
       </c>
+      <c r="C209" t="inlineStr"/>
       <c r="D209" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -34689,6 +35022,7 @@
           <t>Which is most likely to be verified in CMG acceptance for 4G?</t>
         </is>
       </c>
+      <c r="AH209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -34701,6 +35035,7 @@
           <t>Altaf Ahmad</t>
         </is>
       </c>
+      <c r="C210" t="inlineStr"/>
       <c r="D210" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -34851,6 +35186,7 @@
           <t>What is critical to validate for mobility in ATP?</t>
         </is>
       </c>
+      <c r="AH210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -34863,6 +35199,7 @@
           <t>Dhruv Kant Goyal</t>
         </is>
       </c>
+      <c r="C211" t="inlineStr"/>
       <c r="D211" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -35013,6 +35350,7 @@
           <t>Which design goal is central to NRD’s cloud-native approach?</t>
         </is>
       </c>
+      <c r="AH211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -35025,6 +35363,7 @@
           <t>Mohammad Ayyub</t>
         </is>
       </c>
+      <c r="C212" t="inlineStr"/>
       <c r="D212" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -35175,6 +35514,7 @@
           <t>What is the primary role of Nokia Cloud Mobile Gateway (CMG) in packet core?</t>
         </is>
       </c>
+      <c r="AH212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -35187,6 +35527,7 @@
           <t>Vivek Mishra</t>
         </is>
       </c>
+      <c r="C213" t="inlineStr"/>
       <c r="D213" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -35337,6 +35678,7 @@
           <t>Which statement best describes NRD deployment architecture?</t>
         </is>
       </c>
+      <c r="AH213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -35349,6 +35691,7 @@
           <t>Abhishek Kumar Patel</t>
         </is>
       </c>
+      <c r="C214" t="inlineStr"/>
       <c r="D214" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -35499,6 +35842,7 @@
           <t>Key onboarding activity for CMM?</t>
         </is>
       </c>
+      <c r="AH214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -35511,6 +35855,7 @@
           <t>Chandra Sen</t>
         </is>
       </c>
+      <c r="C215" t="inlineStr"/>
       <c r="D215" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -35661,6 +36006,7 @@
           <t>CMG is best described as:</t>
         </is>
       </c>
+      <c r="AH215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -35673,6 +36019,7 @@
           <t>Depankar Kumar</t>
         </is>
       </c>
+      <c r="C216" t="inlineStr"/>
       <c r="D216" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -35823,6 +36170,7 @@
           <t>Which protocol family is most relevant to CMG integration with EPC nodes?</t>
         </is>
       </c>
+      <c r="AH216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -35835,6 +36183,7 @@
           <t>Mohanram G</t>
         </is>
       </c>
+      <c r="C217" t="inlineStr"/>
       <c r="D217" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -35985,6 +36334,7 @@
           <t>Which statement best reflects CMG architecture?</t>
         </is>
       </c>
+      <c r="AH217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -35997,6 +36347,7 @@
           <t>Manpreet Kaur</t>
         </is>
       </c>
+      <c r="C218" t="inlineStr"/>
       <c r="D218" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -36147,6 +36498,7 @@
           <t>Attach succeeds but bearer fails. Likely issue?</t>
         </is>
       </c>
+      <c r="AH218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -36159,6 +36511,7 @@
           <t>R Timmappa</t>
         </is>
       </c>
+      <c r="C219" t="inlineStr"/>
       <c r="D219" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -36309,6 +36662,7 @@
           <t>Which Nokia platform is commonly used for CMM management?</t>
         </is>
       </c>
+      <c r="AH219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -36321,6 +36675,7 @@
           <t>Smruti Snigdha Sahoo</t>
         </is>
       </c>
+      <c r="C220" t="inlineStr"/>
       <c r="D220" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -36471,6 +36826,7 @@
           <t>In a CMG ATP plan, which test most directly verifies end-user data service?</t>
         </is>
       </c>
+      <c r="AH220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -36483,6 +36839,7 @@
           <t>Tejaswini Patel</t>
         </is>
       </c>
+      <c r="C221" t="inlineStr"/>
       <c r="D221" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -36633,6 +36990,7 @@
           <t>Which ATP case is useful for validating CMG resilience?</t>
         </is>
       </c>
+      <c r="AH221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -36645,6 +37003,7 @@
           <t>Amit Ravindra Ghadge</t>
         </is>
       </c>
+      <c r="C222" t="inlineStr"/>
       <c r="D222" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -36795,6 +37154,7 @@
           <t>Which scenario best tests CMG under mobility conditions?</t>
         </is>
       </c>
+      <c r="AH222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -36807,6 +37167,7 @@
           <t>Sayanth A V</t>
         </is>
       </c>
+      <c r="C223" t="inlineStr"/>
       <c r="D223" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -36957,6 +37318,7 @@
           <t>CMM supports which management interfaces for operations and troubleshooting?</t>
         </is>
       </c>
+      <c r="AH223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -36969,6 +37331,7 @@
           <t>Abhishek Kumar</t>
         </is>
       </c>
+      <c r="C224" t="inlineStr"/>
       <c r="D224" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -37119,6 +37482,7 @@
           <t>Which aspect is most important during CMG onboarding?</t>
         </is>
       </c>
+      <c r="AH224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -37131,6 +37495,7 @@
           <t>Avinash Yadav</t>
         </is>
       </c>
+      <c r="C225" t="inlineStr"/>
       <c r="D225" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -37281,6 +37646,7 @@
           <t>Attach ok but PDN fails. Check?</t>
         </is>
       </c>
+      <c r="AH225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -37293,6 +37659,7 @@
           <t>Mohammad Ali Ahmed Jameel</t>
         </is>
       </c>
+      <c r="C226" t="inlineStr"/>
       <c r="D226" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -37443,6 +37810,7 @@
           <t>CMG is best described as:</t>
         </is>
       </c>
+      <c r="AH226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -37455,6 +37823,7 @@
           <t>Mohammad Mohasin Khan</t>
         </is>
       </c>
+      <c r="C227" t="inlineStr"/>
       <c r="D227" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -37605,6 +37974,7 @@
           <t>Attach fails after MME relocation. What is tested?</t>
         </is>
       </c>
+      <c r="AH227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -37617,6 +37987,7 @@
           <t>Naredla Nirosha</t>
         </is>
       </c>
+      <c r="C228" t="inlineStr"/>
       <c r="D228" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -37767,6 +38138,7 @@
           <t>What is a major functional benefit of CMG in packet core?</t>
         </is>
       </c>
+      <c r="AH228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -37779,6 +38151,7 @@
           <t>Sachin P Gilbile</t>
         </is>
       </c>
+      <c r="C229" t="inlineStr"/>
       <c r="D229" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -37929,6 +38302,7 @@
           <t>CMG is best described as:</t>
         </is>
       </c>
+      <c r="AH229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -37941,6 +38315,7 @@
           <t>Liji Babu</t>
         </is>
       </c>
+      <c r="C230" t="inlineStr"/>
       <c r="D230" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -38091,6 +38466,7 @@
           <t>CMM supports which management interfaces for operations and troubleshooting?</t>
         </is>
       </c>
+      <c r="AH230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -38103,6 +38479,7 @@
           <t>Arvind Kumar Singh</t>
         </is>
       </c>
+      <c r="C231" t="inlineStr"/>
       <c r="D231" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -38253,6 +38630,7 @@
           <t>Successful ATP indication?</t>
         </is>
       </c>
+      <c r="AH231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -38265,6 +38643,7 @@
           <t>Aparajita Shankar</t>
         </is>
       </c>
+      <c r="C232" t="inlineStr"/>
       <c r="D232" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -38415,6 +38794,7 @@
           <t>What is the best description of a Network Function Instance in NRD/SBA context?</t>
         </is>
       </c>
+      <c r="AH232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -38427,6 +38807,7 @@
           <t>Phani Shree</t>
         </is>
       </c>
+      <c r="C233" t="inlineStr"/>
       <c r="D233" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -38577,6 +38958,7 @@
           <t>Attach fails for specific IMSI range. Cause?</t>
         </is>
       </c>
+      <c r="AH233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -38589,6 +38971,7 @@
           <t>S Mohankumar</t>
         </is>
       </c>
+      <c r="C234" t="inlineStr"/>
       <c r="D234" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -38739,6 +39122,7 @@
           <t>In onboarding, which item is usually validated first?</t>
         </is>
       </c>
+      <c r="AH234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -38751,6 +39135,7 @@
           <t>Manojkannan</t>
         </is>
       </c>
+      <c r="C235" t="inlineStr"/>
       <c r="D235" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -38901,6 +39286,7 @@
           <t>If attach succeeds but data service fails, which CMG area should be checked first?</t>
         </is>
       </c>
+      <c r="AH235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -38913,6 +39299,7 @@
           <t>Srivani Supraja</t>
         </is>
       </c>
+      <c r="C236" t="inlineStr"/>
       <c r="D236" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -39063,6 +39450,7 @@
           <t>CMM is described by Nokia as having what kind of architecture?</t>
         </is>
       </c>
+      <c r="AH236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -39075,6 +39463,7 @@
           <t>Nutan Rani</t>
         </is>
       </c>
+      <c r="C237" t="inlineStr"/>
       <c r="D237" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -39225,6 +39614,7 @@
           <t>First ATP validation step should be?</t>
         </is>
       </c>
+      <c r="AH237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -39237,6 +39627,7 @@
           <t>Prasanth S</t>
         </is>
       </c>
+      <c r="C238" t="inlineStr"/>
       <c r="D238" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -39387,6 +39778,7 @@
           <t>Which aspect is most important during CMG onboarding?</t>
         </is>
       </c>
+      <c r="AH238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -39399,6 +39791,7 @@
           <t>Pankaj Verma</t>
         </is>
       </c>
+      <c r="C239" t="inlineStr"/>
       <c r="D239" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -39549,6 +39942,7 @@
           <t>Which protocol family is most relevant to CMG integration with EPC nodes?</t>
         </is>
       </c>
+      <c r="AH239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -39561,6 +39955,7 @@
           <t>Madhura Atul Kulkarni</t>
         </is>
       </c>
+      <c r="C240" t="inlineStr"/>
       <c r="D240" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -39711,6 +40106,7 @@
           <t>Which interface is key for LTE access during ATP?</t>
         </is>
       </c>
+      <c r="AH240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -39723,6 +40119,7 @@
           <t>Sahil Mantrao</t>
         </is>
       </c>
+      <c r="C241" t="inlineStr"/>
       <c r="D241" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -39873,6 +40270,7 @@
           <t>What is the primary role of Nokia Cloud Mobility Manager (CMM) in a 4G packet core?</t>
         </is>
       </c>
+      <c r="AH241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -39885,6 +40283,7 @@
           <t>Satish Maurya</t>
         </is>
       </c>
+      <c r="C242" t="inlineStr"/>
       <c r="D242" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -40035,6 +40434,7 @@
           <t>If attach succeeds but data service fails, which CMG area should be checked first?</t>
         </is>
       </c>
+      <c r="AH242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -40047,6 +40447,7 @@
           <t>Janardan Singh</t>
         </is>
       </c>
+      <c r="C243" t="inlineStr"/>
       <c r="D243" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -40197,6 +40598,7 @@
           <t>CMM is described by Nokia as having what kind of architecture?</t>
         </is>
       </c>
+      <c r="AH243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -40209,6 +40611,7 @@
           <t>Kushagra Chaudhary</t>
         </is>
       </c>
+      <c r="C244" t="inlineStr"/>
       <c r="D244" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -40359,6 +40762,7 @@
           <t>Which ATP case is useful for validating CMG resilience?</t>
         </is>
       </c>
+      <c r="AH244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -40371,6 +40775,7 @@
           <t>Ayan Kumar Roy</t>
         </is>
       </c>
+      <c r="C245" t="inlineStr"/>
       <c r="D245" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -40521,6 +40926,7 @@
           <t>Which is a common integration point for CMG in EPC?</t>
         </is>
       </c>
+      <c r="AH245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -40533,6 +40939,7 @@
           <t>Yashi Gupta</t>
         </is>
       </c>
+      <c r="C246" t="inlineStr"/>
       <c r="D246" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -40683,6 +41090,7 @@
           <t>Best failover ATP test?</t>
         </is>
       </c>
+      <c r="AH246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -40695,6 +41103,7 @@
           <t>Anita KM</t>
         </is>
       </c>
+      <c r="C247" t="inlineStr"/>
       <c r="D247" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -40845,6 +41254,7 @@
           <t>Attach fails after MME relocation. What is tested?</t>
         </is>
       </c>
+      <c r="AH247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -40857,6 +41267,7 @@
           <t>Nitesh Kumar</t>
         </is>
       </c>
+      <c r="C248" t="inlineStr"/>
       <c r="D248" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -41007,6 +41418,7 @@
           <t>In 4G EPC, CMG is most closely associated with which gateway role?</t>
         </is>
       </c>
+      <c r="AH248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -41019,6 +41431,7 @@
           <t>Pratibha Singh</t>
         </is>
       </c>
+      <c r="C249" t="inlineStr"/>
       <c r="D249" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -41169,6 +41582,7 @@
           <t>Which ATP check best confirms attach-related functionality?</t>
         </is>
       </c>
+      <c r="AH249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -41181,6 +41595,7 @@
           <t>Neha Ojha</t>
         </is>
       </c>
+      <c r="C250" t="inlineStr"/>
       <c r="D250" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -41331,6 +41746,7 @@
           <t>If attach succeeds but data service fails, which CMG area should be checked first?</t>
         </is>
       </c>
+      <c r="AH250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -41343,6 +41759,7 @@
           <t>P Vishnu</t>
         </is>
       </c>
+      <c r="C251" t="inlineStr"/>
       <c r="D251" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -41493,6 +41910,7 @@
           <t>Which ATP outcome best confirms correct NRD functionality?</t>
         </is>
       </c>
+      <c r="AH251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -41505,6 +41923,7 @@
           <t>khusboo Mantoo</t>
         </is>
       </c>
+      <c r="C252" t="inlineStr"/>
       <c r="D252" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -41655,6 +42074,7 @@
           <t>In 4G EPC, CMG is most closely associated with which gateway role?</t>
         </is>
       </c>
+      <c r="AH252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -41667,6 +42087,7 @@
           <t>Shridhar Patange</t>
         </is>
       </c>
+      <c r="C253" t="inlineStr"/>
       <c r="D253" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -41817,6 +42238,7 @@
           <t>What is the primary role of Nokia Cloud Mobile Gateway (CMG) in packet core?</t>
         </is>
       </c>
+      <c r="AH253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -41829,6 +42251,7 @@
           <t>Vishal Chaudhary</t>
         </is>
       </c>
+      <c r="C254" t="inlineStr"/>
       <c r="D254" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -41979,6 +42402,7 @@
           <t>NRD implements which kind of services?</t>
         </is>
       </c>
+      <c r="AH254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -41991,6 +42415,7 @@
           <t>Niteesh Pandey</t>
         </is>
       </c>
+      <c r="C255" t="inlineStr"/>
       <c r="D255" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -42141,6 +42566,7 @@
           <t>Which outcome indicates a successful CMG onboarding and integration cycle?</t>
         </is>
       </c>
+      <c r="AH255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -42153,6 +42579,7 @@
           <t>Akanksha Haste</t>
         </is>
       </c>
+      <c r="C256" t="inlineStr"/>
       <c r="D256" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -42303,6 +42730,7 @@
           <t>In onboarding, which item is usually validated first?</t>
         </is>
       </c>
+      <c r="AH256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -42315,6 +42743,7 @@
           <t>Abdullah Ahmed</t>
         </is>
       </c>
+      <c r="C257" t="inlineStr"/>
       <c r="D257" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -42465,6 +42894,7 @@
           <t>In a 4G ATP scenario, what does successful bearer establishment mainly confirm?</t>
         </is>
       </c>
+      <c r="AH257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -42477,6 +42907,7 @@
           <t>Devendra Pratap Gupta</t>
         </is>
       </c>
+      <c r="C258" t="inlineStr"/>
       <c r="D258" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -42627,6 +43058,7 @@
           <t>Which aspect is most important during CMG onboarding?</t>
         </is>
       </c>
+      <c r="AH258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -42639,6 +43071,7 @@
           <t>Mukkollu Nagababu</t>
         </is>
       </c>
+      <c r="C259" t="inlineStr"/>
       <c r="D259" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -42789,6 +43222,7 @@
           <t>Which is a common integration point for CMG in EPC?</t>
         </is>
       </c>
+      <c r="AH259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -42801,6 +43235,7 @@
           <t>Divyanshu Vikram Bhadouria</t>
         </is>
       </c>
+      <c r="C260" t="inlineStr"/>
       <c r="D260" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -42951,6 +43386,7 @@
           <t>What is a practical ATP objective for CMG interworking?</t>
         </is>
       </c>
+      <c r="AH260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -42963,6 +43399,7 @@
           <t>Harshraj Sharma</t>
         </is>
       </c>
+      <c r="C261" t="inlineStr"/>
       <c r="D261" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -43113,6 +43550,7 @@
           <t>What is a practical ATP objective for CMG interworking?</t>
         </is>
       </c>
+      <c r="AH261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -43125,6 +43563,7 @@
           <t>Deepak Kumar Sharma</t>
         </is>
       </c>
+      <c r="C262" t="inlineStr"/>
       <c r="D262" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -43275,6 +43714,7 @@
           <t>In 4G EPC, CMG is most closely associated with which gateway role?</t>
         </is>
       </c>
+      <c r="AH262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -43287,6 +43727,7 @@
           <t>Anand Kumar</t>
         </is>
       </c>
+      <c r="C263" t="inlineStr"/>
       <c r="D263" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -43437,6 +43878,7 @@
           <t>Which is a common integration point for CMG in EPC?</t>
         </is>
       </c>
+      <c r="AH263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -43449,6 +43891,7 @@
           <t>Priya  M</t>
         </is>
       </c>
+      <c r="C264" t="inlineStr"/>
       <c r="D264" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -43599,6 +44042,7 @@
           <t>Which ATP check best confirms attach-related functionality?</t>
         </is>
       </c>
+      <c r="AH264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -43611,6 +44055,7 @@
           <t>Navyasri Neelapu</t>
         </is>
       </c>
+      <c r="C265" t="inlineStr"/>
       <c r="D265" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -43761,6 +44206,7 @@
           <t>CMG is best described as:</t>
         </is>
       </c>
+      <c r="AH265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -43773,6 +44219,7 @@
           <t>Deepika  S</t>
         </is>
       </c>
+      <c r="C266" t="inlineStr"/>
       <c r="D266" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -43923,6 +44370,7 @@
           <t>CMG can support which access evolution model?</t>
         </is>
       </c>
+      <c r="AH266" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Show live employee product on the portal and remap 1042323 from CMG to CMM.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Resource_Question_Mapping.xlsx
+++ b/Resource_Question_Mapping.xlsx
@@ -754,7 +754,6 @@
           <t>[HSS Troubleshooting] The healthCheck.log shows isRtpReadinessOK: False. Which command should be used next to check RTP-based process status?</t>
         </is>
       </c>
-      <c r="AH2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -922,7 +921,6 @@
           <t>[HSS Troubleshooting] An operator runs kubectl get pod -n hss and notices one pod shows 2/3 Running in the Ready column. What does this indicate?</t>
         </is>
       </c>
-      <c r="AH3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1090,7 +1088,6 @@
           <t>[HSS Deployment] After deploying Nokia HSS CNF through NCOM, the engineer must confirm whether all pods are running in the target namespace. Which command should be used?</t>
         </is>
       </c>
-      <c r="AH4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1258,7 +1255,6 @@
           <t>[UDM Planning] Planning for LLB failover requires historical CFR statistics on each connection to influence PG server selection. What is this called?</t>
         </is>
       </c>
-      <c r="AH5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1426,7 +1422,6 @@
           <t>[Deployment &amp; Troubleshooting] If all HTTP/2 LB Pods run into Http/2 egress connection failure simultaneously, what happens at the NRF level?</t>
         </is>
       </c>
-      <c r="AH6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1594,7 +1589,6 @@
           <t>[HSS Basics] An MME requests authentication vectors for a subscriber attempting to attach to the LTE network. Which service generates these vectors?</t>
         </is>
       </c>
-      <c r="AH7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1762,7 +1756,6 @@
           <t>[UDM Basic] A subscriber roams to another PLMN and the HPLMN needs to securely deliver a preferred PLMN list. Which service secures this SoR data?</t>
         </is>
       </c>
-      <c r="AH8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1930,7 +1923,6 @@
           <t>[Deployment &amp; Troubleshooting] A troubleshooting engineer notices Pods with unusually high error rates and wants automatic isolation and recovery. Which feature addresses this?</t>
         </is>
       </c>
-      <c r="AH9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2098,7 +2090,6 @@
           <t>[Deployment &amp; Troubleshooting] Before running Netconf rpc commands to configure the CDS threshold, what tool must be installed on the operator's machine?</t>
         </is>
       </c>
-      <c r="AH10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2266,7 +2257,6 @@
           <t>[HSS Basics] The operations team notices failures in SS7 message routing toward HLR processing nodes. Which service should be investigated first?</t>
         </is>
       </c>
-      <c r="AH11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2434,7 +2424,6 @@
           <t>[UDM Basic] AUSF NF wants to retrieve authentication data from UDM. Which interface should be used?</t>
         </is>
       </c>
-      <c r="AH12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2602,7 +2591,6 @@
           <t>[HSS Troubleshooting] An engineer wants to verify SCTP connection status for SS7. Which command is recommended instead of relying on netstat?</t>
         </is>
       </c>
-      <c r="AH13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2770,7 +2758,6 @@
           <t>[Deployment &amp; Troubleshooting] When the HTTP/2 LB Pod detects an egress connection failure, where is the failure file written?</t>
         </is>
       </c>
-      <c r="AH14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2938,7 +2925,6 @@
           <t>[UDM Basic] A SUCI needs to be de-concealed to a SUPI. Which service performs this function?</t>
         </is>
       </c>
-      <c r="AH15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3106,7 +3092,6 @@
           <t>[Deployment &amp; Troubleshooting] The NIM leader Pod goes down unexpectedly. What happens to NRF interfacing during the leader re-election?</t>
         </is>
       </c>
-      <c r="AH16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3274,7 +3259,6 @@
           <t>[HSS Deployment] The SS7 pod fails to apply the Telesys license. The license file is named M7-KEY-demo.tar.gz, but the configured VNF ID is hlrcn. What should be checked first?</t>
         </is>
       </c>
-      <c r="AH17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3442,7 +3426,6 @@
           <t>[HSS Troubleshooting] The healthCheck.log shows isRtpReadinessOK: False. Which command should be used next to check RTP-based process status?</t>
         </is>
       </c>
-      <c r="AH18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3610,7 +3593,6 @@
           <t>[HSS Deployment] A deployment engineer is planning external networks for Diameter, LDAP, Trigger, and SS7 pods. Which component is responsible for assigning external network IPs to pods?</t>
         </is>
       </c>
-      <c r="AH19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3778,7 +3760,6 @@
           <t>[Deployment &amp; Troubleshooting] A troubleshooting engineer needs to inspect event logs captured inside the OAM container for a specific service. Which log should be checked?</t>
         </is>
       </c>
-      <c r="AH20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3946,7 +3927,6 @@
           <t>[HSS Basics] Several CNF services cannot locate each other after a cluster restart. Which component provides internal service discovery?</t>
         </is>
       </c>
-      <c r="AH21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4114,7 +4094,6 @@
           <t>[HSS Basics] A telecom operator observes that one HSS-CP instance is overloaded while others remain idle. Which service should be verified to ensure traffic is evenly distributed across all HSS-CP instances?</t>
         </is>
       </c>
-      <c r="AH22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4282,7 +4261,6 @@
           <t>[UDM Planning] The security team wants CSR to be handled with an integrated External rootCA when External CA is enabled. Which mechanism supports this?</t>
         </is>
       </c>
-      <c r="AH23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -4450,7 +4428,6 @@
           <t>[HSS Troubleshooting] NCOM reports: No valid repository configured or found for CaaS. What should be done?</t>
         </is>
       </c>
-      <c r="AH24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4618,7 +4595,6 @@
           <t>[HSS Basics] During IMS registration, communication is required between the HSS and the S-CSCF. Which interface supports this communication?</t>
         </is>
       </c>
-      <c r="AH25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4786,7 +4762,6 @@
           <t>[EIR Planning] What is the main focus of the CIQ document, as distinct from the DNP?</t>
         </is>
       </c>
-      <c r="AH26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4954,7 +4929,6 @@
           <t>[HSS Basics] A PCRF needs to store and retrieve subscriber policy-related data from HSS. Which interface should be used?</t>
         </is>
       </c>
-      <c r="AH27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -5122,7 +5096,6 @@
           <t>[HSS Basics] Before delivering an SMS to a subscriber, an SMSC needs routing information from HSS. Which interface is used?</t>
         </is>
       </c>
-      <c r="AH28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -5290,7 +5263,6 @@
           <t>[HSS Troubleshooting] A pod registration check shows envoy status: false. What does this indicate?</t>
         </is>
       </c>
-      <c r="AH29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -5458,7 +5430,6 @@
           <t>[UDM Planning] Planning an in-service software upgrade, the team wants automated pre- and post-upgrade validation. Which mechanism is used for CNF health checks in this feature?</t>
         </is>
       </c>
-      <c r="AH30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -5626,7 +5597,6 @@
           <t>[Basic SDL] A customer wants to move from traditional VNF architecture to cloud-native deployment. Which SDL architecture supports this model?</t>
         </is>
       </c>
-      <c r="AH31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -5794,7 +5764,6 @@
           <t>[Deployment &amp; Troubleshooting] Filesystem utilization alarms are generated. Which command provides disk usage information?</t>
         </is>
       </c>
-      <c r="AH32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -5962,7 +5931,6 @@
           <t>[Basic SDL] A customer wants to move from traditional VNF architecture to cloud-native deployment. Which SDL architecture supports this model?</t>
         </is>
       </c>
-      <c r="AH33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -6130,7 +6098,6 @@
           <t>[Deployment &amp; Troubleshooting] Post deployment where can we check our VM status?</t>
         </is>
       </c>
-      <c r="AH34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -6298,7 +6265,6 @@
           <t>[Basic NDS] An L2 engineer is performing root cause analysis after repeated service outages. Which VM provides diagnostic tools and health checks?</t>
         </is>
       </c>
-      <c r="AH35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -6466,7 +6432,6 @@
           <t>[Basic SDL] An engineer needs to manage SDL lifecycle operations such as scaling and upgrades. Which VM provides these capabilities?</t>
         </is>
       </c>
-      <c r="AH36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -6634,7 +6599,6 @@
           <t>[Basic SDL] An L2 engineer is performing root cause analysis after repeated service outages. Which VM provides diagnostic tools and health checks?</t>
         </is>
       </c>
-      <c r="AH37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -6802,7 +6766,6 @@
           <t>[Basic SDL] A customer migration project specifically requires synchronization between legacy and SDL databases. Which VM is mandatory?</t>
         </is>
       </c>
-      <c r="AH38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -6970,7 +6933,6 @@
           <t>[Planning &amp; Artifact Preparation] Which document provides the detailed customer network information used for design preparation?</t>
         </is>
       </c>
-      <c r="AH39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -7138,7 +7100,6 @@
           <t>[Planning &amp; Artifact Preparation] Incorrect sizing information mainly impacts which area?</t>
         </is>
       </c>
-      <c r="AH40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -7306,7 +7267,6 @@
           <t>[Deployment &amp; Troubleshooting] SDL instantiation has completed, but verification is required. What should the output show?</t>
         </is>
       </c>
-      <c r="AH41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -7474,7 +7434,6 @@
           <t>[Basic SDL] A storage node failure occurs. Which SDL component is responsible for data durability and recovery?</t>
         </is>
       </c>
-      <c r="AH42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -7642,7 +7601,6 @@
           <t>[Planning &amp; Artifact Preparation] Why is CIQ important for SDL deployment?</t>
         </is>
       </c>
-      <c r="AH43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -7810,7 +7768,6 @@
           <t>[Planning &amp; Artifact Preparation] A customer updates network architecture after the design has been finalized. Which documents may require updates?</t>
         </is>
       </c>
-      <c r="AH44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -7978,7 +7935,6 @@
           <t>[Basic SDL] NetAct is not receiving PM/FM statistics although subscriber operations are functioning normally. Which VM should be checked?</t>
         </is>
       </c>
-      <c r="AH45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -8146,7 +8102,6 @@
           <t>[Deployment &amp; Troubleshooting] Filesystem utilization alarms are generated. Which command provides disk usage information?</t>
         </is>
       </c>
-      <c r="AH46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -8314,7 +8269,6 @@
           <t>[Deployment &amp; Troubleshooting] Several components appear in UNKNOWN state. Which information source should be checked first?</t>
         </is>
       </c>
-      <c r="AH47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -8482,7 +8436,6 @@
           <t>[Deployment &amp; Troubleshooting] Replication alarms are reported on Storage VMs. Which command should be checked first?</t>
         </is>
       </c>
-      <c r="AH48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -8650,7 +8603,6 @@
           <t>[Planning &amp; Artifact Preparation] The customer changes interface VLANs after DND approval. What action is required?</t>
         </is>
       </c>
-      <c r="AH49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -8818,7 +8770,6 @@
           <t>[Planning &amp; Artifact Preparation] The customer provided an incomplete network design sheet without VLAN details. Which document should be revisited first?</t>
         </is>
       </c>
-      <c r="AH50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -8986,7 +8937,6 @@
           <t>[Deployment &amp; Troubleshooting] A complete health assessment of SDL is required. Which command should be executed?</t>
         </is>
       </c>
-      <c r="AH51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -9154,7 +9104,6 @@
           <t>[Deployment &amp; Troubleshooting] After deployment, an engineer wants to verify that SDL services are running on all VMs. Which command should be used?</t>
         </is>
       </c>
-      <c r="AH52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -9322,7 +9271,6 @@
           <t>[Basic SDL] An L2 engineer is performing root cause analysis after repeated service outages. Which VM provides diagnostic tools and health checks?</t>
         </is>
       </c>
-      <c r="AH53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -9490,7 +9438,6 @@
           <t>[HSS Basics] An external system needs access to subscriber information stored in One-NDS/SDL while hiding internal business logic services. Which component should be used?</t>
         </is>
       </c>
-      <c r="AH54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -9658,7 +9605,6 @@
           <t>[Basic SDL] A storage node failure occurs. Which SDL component is responsible for data durability and recovery?</t>
         </is>
       </c>
-      <c r="AH55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -9826,7 +9772,6 @@
           <t>[Basic SDL] During a capacity planning workshop, the customer expects subscriber growth to double within a year. Which SDL components are typically scaled to handle increased load?</t>
         </is>
       </c>
-      <c r="AH56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -9994,7 +9939,6 @@
           <t>[Deployment &amp; Troubleshooting] SDL bootstrap is suspected to be stuck. Which script should be executed?</t>
         </is>
       </c>
-      <c r="AH57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -10162,7 +10106,6 @@
           <t>[Deployment &amp; Troubleshooting] After running a health check report, what should ideally be displayed?</t>
         </is>
       </c>
-      <c r="AH58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -10330,7 +10273,6 @@
           <t>[UDM Planning] A deployment requires direct NF-to-NF communication without depending on NRF or SCP availability. Which model should be planned for this requirement?</t>
         </is>
       </c>
-      <c r="AH59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -10498,7 +10440,6 @@
           <t>[HSS Basics] The CNF must communicate with management systems through ZTS services instead of directly connecting to EMS/NMS. Which service supports this integration?</t>
         </is>
       </c>
-      <c r="AH60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -10666,7 +10607,6 @@
           <t>[UDM Planning] A planning discussion on rolling upgrades and node draining introduces a function that guarantees a minimum number of available Pods. What is this called?</t>
         </is>
       </c>
-      <c r="AH61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -10834,7 +10774,6 @@
           <t>[EIR Basic] Besides reducing IP requirements, which additional benefit does the centralized HTTP/2 LB provide?</t>
         </is>
       </c>
-      <c r="AH62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -11002,7 +10941,6 @@
           <t>[UDM Basic] A design review lists 5G core NFs. Which pair correctly represents AUSF_UDM's supported network functions?</t>
         </is>
       </c>
-      <c r="AH63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -11170,7 +11108,6 @@
           <t>[UDM Basic] Which service generates Authentication vectors for AKA based authentications and also supports Ki re-encryption?</t>
         </is>
       </c>
-      <c r="AH64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -11338,7 +11275,6 @@
           <t>[Deployment &amp; Troubleshooting] A customer reports that connectivity from the One-EIR Application towards the backend on port 16611 is not established. What is the first troubleshooting step?</t>
         </is>
       </c>
-      <c r="AH65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -11506,7 +11442,6 @@
           <t>[UDM Planning] A capacity design session covers cluster node types used by AUSF_UDM on NCS. Which node types are used?</t>
         </is>
       </c>
-      <c r="AH66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -11674,7 +11609,6 @@
           <t>[UDM Planning] A security planning session discusses which Kubernetes-level policy objects define security conditions for Pods.</t>
         </is>
       </c>
-      <c r="AH67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -11842,7 +11776,6 @@
           <t>[HSS Troubleshooting] The SS7 Telesys process is down. What should be checked first?</t>
         </is>
       </c>
-      <c r="AH68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -12010,7 +11943,6 @@
           <t>[HSS Basics] Several CNF services cannot locate each other after a cluster restart. Which component provides internal service discovery?</t>
         </is>
       </c>
-      <c r="AH69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -12178,7 +12110,6 @@
           <t>[HSS Troubleshooting] A pod is stuck in ImagePullBackOff or ErrImagePull. What is the recommended corrective action?</t>
         </is>
       </c>
-      <c r="AH70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -12346,7 +12277,6 @@
           <t>[Deployment &amp; Troubleshooting] An autoscaling design uses HPA with which primary metric to trigger scale-out or scale-in decisions?</t>
         </is>
       </c>
-      <c r="AH71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -12514,7 +12444,6 @@
           <t>[Deployment &amp; Troubleshooting] Traffic is still being routed to a Pod that is not actually ready to serve requests. Which probe should be checked to correct this?</t>
         </is>
       </c>
-      <c r="AH72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -12682,7 +12611,6 @@
           <t>[HSS Basics] A 5G core deployment requires interworking between a UDM and HSS. Which proprietary Diameter interface supports this requirement?</t>
         </is>
       </c>
-      <c r="AH73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -12850,7 +12778,6 @@
           <t>[UDM Basic] SMS Function needs to register its address and retrieve SMS management subscription data from UDM. Which interface is used?</t>
         </is>
       </c>
-      <c r="AH74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -13018,7 +12945,6 @@
           <t>[Deployment &amp; Troubleshooting] A process heap size configuration file defines thresholds like HEAP_SIZE_CRITICAL and HEAP_SIZE_MAJOR. What action is taken if a process exceeds the critical threshold?</t>
         </is>
       </c>
-      <c r="AH75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -13186,7 +13112,6 @@
           <t>[HSS Troubleshooting] A pod registration check shows envoy status: false. What does this indicate?</t>
         </is>
       </c>
-      <c r="AH76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -13354,7 +13279,6 @@
           <t>[HSS Deployment] The operator wants to run CNF health checks using Helm test or NCOM GUI. Which parameter should be enabled?</t>
         </is>
       </c>
-      <c r="AH77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -13522,7 +13446,6 @@
           <t>[HSS Troubleshooting] A pod registration check shows envoy status: false. What does this indicate?</t>
         </is>
       </c>
-      <c r="AH78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -13690,7 +13613,6 @@
           <t>[HSS Basics] A 5G core deployment requires interworking between a UDM and HSS. Which proprietary Diameter interface supports this requirement?</t>
         </is>
       </c>
-      <c r="AH79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -13858,7 +13780,6 @@
           <t>[HSS Troubleshooting] The HLRCallP pod continuously raises a No Free Dialogue alarm for a DP process. What is the recommended recovery action?</t>
         </is>
       </c>
-      <c r="AH80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -14026,7 +13947,6 @@
           <t>[HSS Troubleshooting] NCOM reports: No valid repository configured or found for CaaS. What should be done?</t>
         </is>
       </c>
-      <c r="AH81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -14194,7 +14114,6 @@
           <t>[Deployment &amp; Troubleshooting] After running a health check report, what should ideally be displayed?</t>
         </is>
       </c>
-      <c r="AH82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -14207,7 +14126,6 @@
           <t>Sanjay Kumar Gupta</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr"/>
       <c r="D83" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -14358,7 +14276,6 @@
           <t>Attach ok but PDN fails. Check?</t>
         </is>
       </c>
-      <c r="AH83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -14371,7 +14288,6 @@
           <t>Bharanidharan</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr"/>
       <c r="D84" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -14522,7 +14438,6 @@
           <t>Purpose of S1-AP on S1-MME?</t>
         </is>
       </c>
-      <c r="AH84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -14535,7 +14450,6 @@
           <t>J Mohammed Sheik Afridi</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr"/>
       <c r="D85" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -14686,7 +14600,6 @@
           <t>Attach ok but PDN fails. Check?</t>
         </is>
       </c>
-      <c r="AH85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -14699,7 +14612,6 @@
           <t>Divyanshu Chauhan</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr"/>
       <c r="D86" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -14850,7 +14762,6 @@
           <t>What is a major functional benefit of CMG in packet core?</t>
         </is>
       </c>
-      <c r="AH86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -14863,7 +14774,6 @@
           <t>Chitrangada Mishra</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr"/>
       <c r="D87" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -15014,7 +14924,6 @@
           <t>In 4G LTE, CMM most commonly provides which network function?</t>
         </is>
       </c>
-      <c r="AH87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -15027,7 +14936,6 @@
           <t>Vibhor Chandra Gupta</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr"/>
       <c r="D88" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -15178,7 +15086,6 @@
           <t>Which CMM component is responsible for OAM functions and northbound interfaces?</t>
         </is>
       </c>
-      <c r="AH88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -15191,7 +15098,6 @@
           <t>Nishu Kumar</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr"/>
       <c r="D89" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -15342,7 +15248,6 @@
           <t>Which technology is highlighted in CMM for performance optimization on x86 platforms?</t>
         </is>
       </c>
-      <c r="AH89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -15355,7 +15260,6 @@
           <t>Satheeshkumar</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr"/>
       <c r="D90" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -15506,7 +15410,6 @@
           <t>In a 4G ATP scenario, what does successful bearer establishment mainly confirm?</t>
         </is>
       </c>
-      <c r="AH90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -15519,7 +15422,6 @@
           <t>Chandan Kumar Singh</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr"/>
       <c r="D91" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -15670,7 +15572,6 @@
           <t>What is a major functional benefit of CMG in packet core?</t>
         </is>
       </c>
-      <c r="AH91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -15683,7 +15584,6 @@
           <t>Sourabh  Khandelwal</t>
         </is>
       </c>
-      <c r="C92" t="inlineStr"/>
       <c r="D92" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -15834,7 +15734,6 @@
           <t>CMG is best described as:</t>
         </is>
       </c>
-      <c r="AH92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -15847,7 +15746,6 @@
           <t>Prateek</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr"/>
       <c r="D93" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -15998,7 +15896,6 @@
           <t>CMM is described by Nokia as having what kind of architecture?</t>
         </is>
       </c>
-      <c r="AH93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -16011,7 +15908,6 @@
           <t>Veerasami</t>
         </is>
       </c>
-      <c r="C94" t="inlineStr"/>
       <c r="D94" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -16162,7 +16058,6 @@
           <t>In 4G LTE, CMM most commonly provides which network function?</t>
         </is>
       </c>
-      <c r="AH94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -16175,7 +16070,6 @@
           <t>Parth Saxena</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr"/>
       <c r="D95" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -16326,7 +16220,6 @@
           <t>CMG supports evolution toward which major core direction?</t>
         </is>
       </c>
-      <c r="AH95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -16339,7 +16232,6 @@
           <t>Satya Prakash Rai</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr"/>
       <c r="D96" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -16490,7 +16382,6 @@
           <t>Purpose of S1-AP on S1-MME?</t>
         </is>
       </c>
-      <c r="AH96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -16503,7 +16394,6 @@
           <t>Meenatchi M</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr"/>
       <c r="D97" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -16654,7 +16544,6 @@
           <t>Which network function is most directly linked to slice selection in NRD-related architecture?</t>
         </is>
       </c>
-      <c r="AH97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -16667,7 +16556,6 @@
           <t>Sunilkumaar Selvaraajan</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr"/>
       <c r="D98" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -16818,7 +16706,6 @@
           <t>What is the primary purpose of Nokia Resource Director (NRD)?</t>
         </is>
       </c>
-      <c r="AH98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -16831,7 +16718,6 @@
           <t>Ashwini Raju</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr"/>
       <c r="D99" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -16982,7 +16868,6 @@
           <t>Which deployment characteristic is strongly associated with CMG?</t>
         </is>
       </c>
-      <c r="AH99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -16995,7 +16880,6 @@
           <t>Sunil Kumar Patel</t>
         </is>
       </c>
-      <c r="C100" t="inlineStr"/>
       <c r="D100" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -17146,7 +17030,6 @@
           <t>Which deployment characteristic is strongly associated with CMG?</t>
         </is>
       </c>
-      <c r="AH100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -17159,7 +17042,6 @@
           <t>Naveenkumar</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr"/>
       <c r="D101" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -17310,7 +17192,6 @@
           <t>What is a major functional benefit of CMG in packet core?</t>
         </is>
       </c>
-      <c r="AH101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -17323,7 +17204,6 @@
           <t>G  Koushik</t>
         </is>
       </c>
-      <c r="C102" t="inlineStr"/>
       <c r="D102" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -17474,7 +17354,6 @@
           <t>CMM is described by Nokia as having what kind of architecture?</t>
         </is>
       </c>
-      <c r="AH102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -17487,7 +17366,6 @@
           <t>Kapil Chaudhary</t>
         </is>
       </c>
-      <c r="C103" t="inlineStr"/>
       <c r="D103" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -17638,7 +17516,6 @@
           <t>Successful ATP indication?</t>
         </is>
       </c>
-      <c r="AH103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -17651,7 +17528,6 @@
           <t>Aryan Kumar</t>
         </is>
       </c>
-      <c r="C104" t="inlineStr"/>
       <c r="D104" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -17802,7 +17678,6 @@
           <t>CMG supports evolution toward which major core direction?</t>
         </is>
       </c>
-      <c r="AH104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -17815,7 +17690,6 @@
           <t>Pratik Raj</t>
         </is>
       </c>
-      <c r="C105" t="inlineStr"/>
       <c r="D105" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -17966,7 +17840,6 @@
           <t>Which ATP case is useful for validating CMG resilience?</t>
         </is>
       </c>
-      <c r="AH105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -17979,7 +17852,6 @@
           <t>Ezhilarasan</t>
         </is>
       </c>
-      <c r="C106" t="inlineStr"/>
       <c r="D106" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -18130,7 +18002,6 @@
           <t>Which protocols relate to CMM control plane?</t>
         </is>
       </c>
-      <c r="AH106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -18143,7 +18014,6 @@
           <t>Santosh Kumar</t>
         </is>
       </c>
-      <c r="C107" t="inlineStr"/>
       <c r="D107" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -18294,7 +18164,6 @@
           <t>CMG is best described as:</t>
         </is>
       </c>
-      <c r="AH107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -18307,7 +18176,6 @@
           <t>Srinath</t>
         </is>
       </c>
-      <c r="C108" t="inlineStr"/>
       <c r="D108" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -18458,7 +18326,6 @@
           <t>Which interface is key for LTE access during ATP?</t>
         </is>
       </c>
-      <c r="AH108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -18471,7 +18338,6 @@
           <t>Kiruthika V</t>
         </is>
       </c>
-      <c r="C109" t="inlineStr"/>
       <c r="D109" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -18622,7 +18488,6 @@
           <t>Which ATP case is useful for validating CMG resilience?</t>
         </is>
       </c>
-      <c r="AH109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -18635,7 +18500,6 @@
           <t>Pratyasa Mohanty</t>
         </is>
       </c>
-      <c r="C110" t="inlineStr"/>
       <c r="D110" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -18786,7 +18650,6 @@
           <t>Which Nokia platform is commonly used for CMM management?</t>
         </is>
       </c>
-      <c r="AH110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -18799,7 +18662,6 @@
           <t>Soumya Smruti Das</t>
         </is>
       </c>
-      <c r="C111" t="inlineStr"/>
       <c r="D111" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -18950,7 +18812,6 @@
           <t>Which outcome indicates a successful CMG onboarding and integration cycle?</t>
         </is>
       </c>
-      <c r="AH111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -18963,7 +18824,6 @@
           <t>Pratyusha Pattanaik</t>
         </is>
       </c>
-      <c r="C112" t="inlineStr"/>
       <c r="D112" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -19114,7 +18974,6 @@
           <t>Which CMM component provides logical interface termination for GTP and Diameter?</t>
         </is>
       </c>
-      <c r="AH112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -19127,7 +18986,6 @@
           <t>Ashutosh</t>
         </is>
       </c>
-      <c r="C113" t="inlineStr"/>
       <c r="D113" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -19278,7 +19136,6 @@
           <t>Which technology is highlighted in CMM for performance optimization on x86 platforms?</t>
         </is>
       </c>
-      <c r="AH113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -19291,7 +19148,6 @@
           <t>Gudluru Lakshmi Narayan</t>
         </is>
       </c>
-      <c r="C114" t="inlineStr"/>
       <c r="D114" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -19442,7 +19298,6 @@
           <t>CMG is best described as:</t>
         </is>
       </c>
-      <c r="AH114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -19455,7 +19310,6 @@
           <t>Madanuru Vishnu Charan</t>
         </is>
       </c>
-      <c r="C115" t="inlineStr"/>
       <c r="D115" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -19606,7 +19460,6 @@
           <t>What is critical to validate for mobility in ATP?</t>
         </is>
       </c>
-      <c r="AH115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -19619,7 +19472,6 @@
           <t>Abhisek Mohanty</t>
         </is>
       </c>
-      <c r="C116" t="inlineStr"/>
       <c r="D116" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -19770,7 +19622,6 @@
           <t>In 4G LTE, CMM most commonly provides which network function?</t>
         </is>
       </c>
-      <c r="AH116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -19783,7 +19634,6 @@
           <t>Avipsa Mohanty</t>
         </is>
       </c>
-      <c r="C117" t="inlineStr"/>
       <c r="D117" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -19934,7 +19784,6 @@
           <t>What is the primary role of Nokia Cloud Mobility Manager (CMM) in a 4G packet core?</t>
         </is>
       </c>
-      <c r="AH117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -19947,7 +19796,6 @@
           <t>Debasish Jena</t>
         </is>
       </c>
-      <c r="C118" t="inlineStr"/>
       <c r="D118" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -20098,7 +19946,6 @@
           <t>Which protocols relate to CMM control plane?</t>
         </is>
       </c>
-      <c r="AH118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -20111,7 +19958,6 @@
           <t>PRITISARATHI BHUYAN</t>
         </is>
       </c>
-      <c r="C119" t="inlineStr"/>
       <c r="D119" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -20262,7 +20108,6 @@
           <t>Best failover ATP test?</t>
         </is>
       </c>
-      <c r="AH119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -20275,7 +20120,6 @@
           <t>Anchal Priyadarshini Swain</t>
         </is>
       </c>
-      <c r="C120" t="inlineStr"/>
       <c r="D120" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -20426,7 +20270,6 @@
           <t>CMG is part of which Nokia family?</t>
         </is>
       </c>
-      <c r="AH120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -20439,7 +20282,6 @@
           <t>Sasmita GIRI</t>
         </is>
       </c>
-      <c r="C121" t="inlineStr"/>
       <c r="D121" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -20590,7 +20432,6 @@
           <t>Which protocols relate to CMM control plane?</t>
         </is>
       </c>
-      <c r="AH121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -20603,7 +20444,6 @@
           <t>Akankshya Rout</t>
         </is>
       </c>
-      <c r="C122" t="inlineStr"/>
       <c r="D122" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -20754,7 +20594,6 @@
           <t>What does NECC stand for in Nokia CMM architecture?</t>
         </is>
       </c>
-      <c r="AH122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -20767,7 +20606,6 @@
           <t>Ajaya Narayan Nayak</t>
         </is>
       </c>
-      <c r="C123" t="inlineStr"/>
       <c r="D123" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -20918,7 +20756,6 @@
           <t>Purpose of S1-AP on S1-MME?</t>
         </is>
       </c>
-      <c r="AH123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -20931,7 +20768,6 @@
           <t>Soumya Ranjan Das</t>
         </is>
       </c>
-      <c r="C124" t="inlineStr"/>
       <c r="D124" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -21082,7 +20918,6 @@
           <t>Purpose of S1-AP on S1-MME?</t>
         </is>
       </c>
-      <c r="AH124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -21095,7 +20930,6 @@
           <t>Vaghela Rahul Rameshbhai</t>
         </is>
       </c>
-      <c r="C125" t="inlineStr"/>
       <c r="D125" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -21246,7 +21080,6 @@
           <t>CMG is best described as:</t>
         </is>
       </c>
-      <c r="AH125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -21259,7 +21092,6 @@
           <t>Asish Nayak</t>
         </is>
       </c>
-      <c r="C126" t="inlineStr"/>
       <c r="D126" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -21410,7 +21242,6 @@
           <t>What is a major functional benefit of CMG in packet core?</t>
         </is>
       </c>
-      <c r="AH126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -21423,7 +21254,6 @@
           <t>Bibhash Dash</t>
         </is>
       </c>
-      <c r="C127" t="inlineStr"/>
       <c r="D127" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -21574,7 +21404,6 @@
           <t>CMM is described by Nokia as having what kind of architecture?</t>
         </is>
       </c>
-      <c r="AH127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -21587,7 +21416,6 @@
           <t>Omm  Sai Roumya RANJAN</t>
         </is>
       </c>
-      <c r="C128" t="inlineStr"/>
       <c r="D128" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -21738,7 +21566,6 @@
           <t>Which aspect is most important during CMG onboarding?</t>
         </is>
       </c>
-      <c r="AH128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -21751,7 +21578,6 @@
           <t>Pradyumna Naik</t>
         </is>
       </c>
-      <c r="C129" t="inlineStr"/>
       <c r="D129" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -21902,7 +21728,6 @@
           <t>CMG is part of which Nokia family?</t>
         </is>
       </c>
-      <c r="AH129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -21915,7 +21740,6 @@
           <t>Abdul Basith Shaik</t>
         </is>
       </c>
-      <c r="C130" t="inlineStr"/>
       <c r="D130" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -22066,7 +21890,6 @@
           <t>Attach succeeds but bearer fails. Likely issue?</t>
         </is>
       </c>
-      <c r="AH130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -22079,7 +21902,6 @@
           <t>Solanki Jigar Ambalal</t>
         </is>
       </c>
-      <c r="C131" t="inlineStr"/>
       <c r="D131" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -22230,7 +22052,6 @@
           <t>Attach ok but PDN fails. Check?</t>
         </is>
       </c>
-      <c r="AH131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -22243,7 +22064,6 @@
           <t>Akash Bairagi</t>
         </is>
       </c>
-      <c r="C132" t="inlineStr"/>
       <c r="D132" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -22394,7 +22214,6 @@
           <t>In a 4G ATP scenario, what does successful bearer establishment mainly confirm?</t>
         </is>
       </c>
-      <c r="AH132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -22407,7 +22226,6 @@
           <t>Anand Babu</t>
         </is>
       </c>
-      <c r="C133" t="inlineStr"/>
       <c r="D133" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -22558,7 +22376,6 @@
           <t>Which protocols relate to CMM control plane?</t>
         </is>
       </c>
-      <c r="AH133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -22571,7 +22388,6 @@
           <t>Chelsea Shalin S</t>
         </is>
       </c>
-      <c r="C134" t="inlineStr"/>
       <c r="D134" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -22722,7 +22538,6 @@
           <t>CMM supports which management interfaces for operations and troubleshooting?</t>
         </is>
       </c>
-      <c r="AH134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -22735,7 +22550,6 @@
           <t>Gopi K</t>
         </is>
       </c>
-      <c r="C135" t="inlineStr"/>
       <c r="D135" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -22886,7 +22700,6 @@
           <t>Purpose of S1-AP on S1-MME?</t>
         </is>
       </c>
-      <c r="AH135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -22899,7 +22712,6 @@
           <t>Malan Subbiah Pandian</t>
         </is>
       </c>
-      <c r="C136" t="inlineStr"/>
       <c r="D136" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -23050,7 +22862,6 @@
           <t>Which is a common integration point for CMG in EPC?</t>
         </is>
       </c>
-      <c r="AH136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -23063,7 +22874,6 @@
           <t>R Krishna Durga</t>
         </is>
       </c>
-      <c r="C137" t="inlineStr"/>
       <c r="D137" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -23214,7 +23024,6 @@
           <t>Purpose of S1-AP on S1-MME?</t>
         </is>
       </c>
-      <c r="AH137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -23227,7 +23036,6 @@
           <t>Sabari Murugesan</t>
         </is>
       </c>
-      <c r="C138" t="inlineStr"/>
       <c r="D138" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -23378,7 +23186,6 @@
           <t>CMM is described by Nokia as having what kind of architecture?</t>
         </is>
       </c>
-      <c r="AH138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -23391,7 +23198,6 @@
           <t>Surya Saravanan</t>
         </is>
       </c>
-      <c r="C139" t="inlineStr"/>
       <c r="D139" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -23542,7 +23348,6 @@
           <t>What is the key purpose of ATP testing for CMG?</t>
         </is>
       </c>
-      <c r="AH139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -23555,7 +23360,6 @@
           <t>Yogaverma V</t>
         </is>
       </c>
-      <c r="C140" t="inlineStr"/>
       <c r="D140" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -23706,7 +23510,6 @@
           <t>Which scenario best tests CMG under mobility conditions?</t>
         </is>
       </c>
-      <c r="AH140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -23719,7 +23522,6 @@
           <t>Varun Pachauri</t>
         </is>
       </c>
-      <c r="C141" t="inlineStr"/>
       <c r="D141" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -23870,7 +23672,6 @@
           <t>CMG supports evolution toward which major core direction?</t>
         </is>
       </c>
-      <c r="AH141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -23883,7 +23684,6 @@
           <t>Buran Sagari Sohail Basha</t>
         </is>
       </c>
-      <c r="C142" t="inlineStr"/>
       <c r="D142" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -24034,7 +23834,6 @@
           <t>Which protocols relate to CMM control plane?</t>
         </is>
       </c>
-      <c r="AH142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -24047,7 +23846,6 @@
           <t>Gadde Yaswanth</t>
         </is>
       </c>
-      <c r="C143" t="inlineStr"/>
       <c r="D143" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -24198,7 +23996,6 @@
           <t>Which Nokia platform is commonly used for CMM management?</t>
         </is>
       </c>
-      <c r="AH143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -24211,7 +24008,6 @@
           <t>Hariharan S</t>
         </is>
       </c>
-      <c r="C144" t="inlineStr"/>
       <c r="D144" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -24362,7 +24158,6 @@
           <t>What does NECC stand for in Nokia CMM architecture?</t>
         </is>
       </c>
-      <c r="AH144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -24375,7 +24170,6 @@
           <t>M Subramanayam</t>
         </is>
       </c>
-      <c r="C145" t="inlineStr"/>
       <c r="D145" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -24526,7 +24320,6 @@
           <t>CMM supports which management interfaces for operations and troubleshooting?</t>
         </is>
       </c>
-      <c r="AH145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -24539,7 +24332,6 @@
           <t>Nekkanti Mahendra Tulasi</t>
         </is>
       </c>
-      <c r="C146" t="inlineStr"/>
       <c r="D146" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -24690,7 +24482,6 @@
           <t>Which interface is key for LTE access during ATP?</t>
         </is>
       </c>
-      <c r="AH146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -24703,7 +24494,6 @@
           <t>V P Sandhiya</t>
         </is>
       </c>
-      <c r="C147" t="inlineStr"/>
       <c r="D147" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -24854,7 +24644,6 @@
           <t>Key onboarding activity for CMM?</t>
         </is>
       </c>
-      <c r="AH147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -24867,7 +24656,6 @@
           <t>Susheel kumar Dwivdi</t>
         </is>
       </c>
-      <c r="C148" t="inlineStr"/>
       <c r="D148" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -25018,7 +24806,6 @@
           <t>In a CMG ATP plan, which test most directly verifies end-user data service?</t>
         </is>
       </c>
-      <c r="AH148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -25031,7 +24818,6 @@
           <t>Vivek Mishra</t>
         </is>
       </c>
-      <c r="C149" t="inlineStr"/>
       <c r="D149" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -25182,7 +24968,6 @@
           <t>If attach succeeds but data service fails, which CMG area should be checked first?</t>
         </is>
       </c>
-      <c r="AH149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -25195,7 +24980,6 @@
           <t>Harshada Vitthal Shinde</t>
         </is>
       </c>
-      <c r="C150" t="inlineStr"/>
       <c r="D150" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -25346,7 +25130,6 @@
           <t>What is the primary role of Nokia Cloud Mobile Gateway (CMG) in packet core?</t>
         </is>
       </c>
-      <c r="AH150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -25359,7 +25142,6 @@
           <t>Nishant Kumar Lal</t>
         </is>
       </c>
-      <c r="C151" t="inlineStr"/>
       <c r="D151" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -25510,7 +25292,6 @@
           <t>What is critical to validate for mobility in ATP?</t>
         </is>
       </c>
-      <c r="AH151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -25523,7 +25304,6 @@
           <t>Vennela Korada</t>
         </is>
       </c>
-      <c r="C152" t="inlineStr"/>
       <c r="D152" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -25674,7 +25454,6 @@
           <t>In a CMG ATP plan, which test most directly verifies end-user data service?</t>
         </is>
       </c>
-      <c r="AH152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -25687,7 +25466,6 @@
           <t>Bommireddy Jaya Prakash Reddy</t>
         </is>
       </c>
-      <c r="C153" t="inlineStr"/>
       <c r="D153" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -25838,7 +25616,6 @@
           <t>Purpose of S1-AP on S1-MME?</t>
         </is>
       </c>
-      <c r="AH153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -25851,7 +25628,6 @@
           <t>Komala Mamidi</t>
         </is>
       </c>
-      <c r="C154" t="inlineStr"/>
       <c r="D154" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -26002,7 +25778,6 @@
           <t>CMM is described by Nokia as having what kind of architecture?</t>
         </is>
       </c>
-      <c r="AH154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -26015,7 +25790,6 @@
           <t>Sundram Kumar</t>
         </is>
       </c>
-      <c r="C155" t="inlineStr"/>
       <c r="D155" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -26166,7 +25940,6 @@
           <t>Key onboarding activity for CMM?</t>
         </is>
       </c>
-      <c r="AH155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -26179,7 +25952,6 @@
           <t>Abhishikha Chauhan</t>
         </is>
       </c>
-      <c r="C156" t="inlineStr"/>
       <c r="D156" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -26330,7 +26102,6 @@
           <t>Why is CMG considered operationally flexible?</t>
         </is>
       </c>
-      <c r="AH156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -26343,7 +26114,6 @@
           <t>Anipeddi Lasya</t>
         </is>
       </c>
-      <c r="C157" t="inlineStr"/>
       <c r="D157" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -26494,7 +26264,6 @@
           <t>Which CMM service hosts the MME functions?</t>
         </is>
       </c>
-      <c r="AH157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -26507,7 +26276,6 @@
           <t>Biruntha</t>
         </is>
       </c>
-      <c r="C158" t="inlineStr"/>
       <c r="D158" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -26658,7 +26426,6 @@
           <t>Which deployment characteristic is strongly associated with CMG?</t>
         </is>
       </c>
-      <c r="AH158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -26671,7 +26438,6 @@
           <t>Himanshu Bungla</t>
         </is>
       </c>
-      <c r="C159" t="inlineStr"/>
       <c r="D159" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -26822,7 +26588,6 @@
           <t>In a 5G ATP test, what should be verified first for NRD?</t>
         </is>
       </c>
-      <c r="AH159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -26835,7 +26600,6 @@
           <t>Nijampatnam Eswar</t>
         </is>
       </c>
-      <c r="C160" t="inlineStr"/>
       <c r="D160" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -26986,7 +26750,6 @@
           <t>What is a practical ATP objective for CMG interworking?</t>
         </is>
       </c>
-      <c r="AH160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -26999,7 +26762,6 @@
           <t>Saiyed Raza Imam</t>
         </is>
       </c>
-      <c r="C161" t="inlineStr"/>
       <c r="D161" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -27150,7 +26912,6 @@
           <t>Which ATP case is useful for validating CMG resilience?</t>
         </is>
       </c>
-      <c r="AH161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -27163,7 +26924,6 @@
           <t>Vaijinath Bhaskar Batule</t>
         </is>
       </c>
-      <c r="C162" t="inlineStr"/>
       <c r="D162" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -27314,7 +27074,6 @@
           <t>Why is CMG considered operationally flexible?</t>
         </is>
       </c>
-      <c r="AH162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -27327,7 +27086,6 @@
           <t>Kamal Kumar Ray</t>
         </is>
       </c>
-      <c r="C163" t="inlineStr"/>
       <c r="D163" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -27478,7 +27236,6 @@
           <t>Which CMM service hosts the MME functions?</t>
         </is>
       </c>
-      <c r="AH163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -27491,7 +27248,6 @@
           <t>Tanmoy Mojumder</t>
         </is>
       </c>
-      <c r="C164" t="inlineStr"/>
       <c r="D164" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -27642,7 +27398,6 @@
           <t>Which technology is highlighted in CMM for performance optimization on x86 platforms?</t>
         </is>
       </c>
-      <c r="AH164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -27655,7 +27410,6 @@
           <t>Shaikh Reshma</t>
         </is>
       </c>
-      <c r="C165" t="inlineStr"/>
       <c r="D165" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -27806,7 +27560,6 @@
           <t>Which CMM component is responsible for OAM functions and northbound interfaces?</t>
         </is>
       </c>
-      <c r="AH165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -27819,7 +27572,6 @@
           <t>Om Prakash Gautam</t>
         </is>
       </c>
-      <c r="C166" t="inlineStr"/>
       <c r="D166" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -27970,7 +27722,6 @@
           <t>What is the primary role of Nokia Cloud Mobile Gateway (CMG) in packet core?</t>
         </is>
       </c>
-      <c r="AH166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -27983,7 +27734,6 @@
           <t>Jaya Vohra</t>
         </is>
       </c>
-      <c r="C167" t="inlineStr"/>
       <c r="D167" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -28134,7 +27884,6 @@
           <t>CMG can support which access evolution model?</t>
         </is>
       </c>
-      <c r="AH167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -28147,7 +27896,6 @@
           <t>S Bijetananda Swain</t>
         </is>
       </c>
-      <c r="C168" t="inlineStr"/>
       <c r="D168" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -28298,7 +28046,6 @@
           <t>If attach succeeds but data service fails, which CMG area should be checked first?</t>
         </is>
       </c>
-      <c r="AH168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -28311,7 +28058,6 @@
           <t>Rohit Kumar</t>
         </is>
       </c>
-      <c r="C169" t="inlineStr"/>
       <c r="D169" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -28462,7 +28208,6 @@
           <t>Which is most likely to be verified in CMG acceptance for 4G?</t>
         </is>
       </c>
-      <c r="AH169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -28475,7 +28220,6 @@
           <t>Sujata Singh</t>
         </is>
       </c>
-      <c r="C170" t="inlineStr"/>
       <c r="D170" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -28626,7 +28370,6 @@
           <t>Why is CMG considered operationally flexible?</t>
         </is>
       </c>
-      <c r="AH170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -28639,7 +28382,6 @@
           <t>SUSHMA CHOLLETI</t>
         </is>
       </c>
-      <c r="C171" t="inlineStr"/>
       <c r="D171" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -28790,7 +28532,6 @@
           <t>Why is CMG considered operationally flexible?</t>
         </is>
       </c>
-      <c r="AH171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -28803,7 +28544,6 @@
           <t>Gaurav Verma</t>
         </is>
       </c>
-      <c r="C172" t="inlineStr"/>
       <c r="D172" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -28954,7 +28694,6 @@
           <t>CMG can support which access evolution model?</t>
         </is>
       </c>
-      <c r="AH172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -28967,7 +28706,6 @@
           <t>Kamna Peyal</t>
         </is>
       </c>
-      <c r="C173" t="inlineStr"/>
       <c r="D173" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -29118,7 +28856,6 @@
           <t>Key onboarding activity for CMM?</t>
         </is>
       </c>
-      <c r="AH173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -29131,7 +28868,6 @@
           <t>Damarasinghu Vinay Kumar</t>
         </is>
       </c>
-      <c r="C174" t="inlineStr"/>
       <c r="D174" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -29139,7 +28875,7 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>CMG</t>
+          <t>CMM</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
@@ -29159,130 +28895,129 @@
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>Which deployment characteristic is strongly associated with CMG?</t>
+          <t>What is critical to validate for mobility in ATP?</t>
         </is>
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>CMG can support which access evolution model?</t>
+          <t>Which CMM service handles 2G/3G mobility and session management?</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
         <is>
-          <t>In a CMG ATP plan, which test most directly verifies end-user data service?</t>
+          <t>Key onboarding activity for CMM?</t>
         </is>
       </c>
       <c r="L174" t="inlineStr">
         <is>
-          <t>Which scenario best tests CMG under mobility conditions?</t>
+          <t>Which CMM service is associated with user-plane packet processing and data forwarding?</t>
         </is>
       </c>
       <c r="M174" t="inlineStr">
         <is>
-          <t>In 4G EPC, CMG is most closely associated with which gateway role?</t>
+          <t>CMM supports which management interfaces for operations and troubleshooting?</t>
         </is>
       </c>
       <c r="N174" t="inlineStr">
         <is>
-          <t>In a 4G ATP scenario, what does successful bearer establishment mainly confirm?</t>
+          <t>Which CMM service hosts the MME functions?</t>
         </is>
       </c>
       <c r="O174" t="inlineStr">
         <is>
-          <t>Which is most likely to be verified in CMG acceptance for 4G?</t>
+          <t>First ATP validation step should be?</t>
         </is>
       </c>
       <c r="P174" t="inlineStr">
         <is>
-          <t>Why is CMG considered operationally flexible?</t>
+          <t>Attach fails after MME relocation. What is tested?</t>
         </is>
       </c>
       <c r="Q174" t="inlineStr">
         <is>
-          <t>If attach succeeds but data service fails, which CMG area should be checked first?</t>
+          <t>What is the primary role of Nokia Cloud Mobility Manager (CMM) in a 4G packet core?</t>
         </is>
       </c>
       <c r="R174" t="inlineStr">
         <is>
-          <t>CMG is part of which Nokia family?</t>
+          <t>Which CMM component provides logical interface termination for GTP and Diameter?</t>
         </is>
       </c>
       <c r="S174" t="inlineStr">
         <is>
-          <t>Which protocol family is most relevant to CMG integration with EPC nodes?</t>
+          <t>Attach fails for specific IMSI range. Cause?</t>
         </is>
       </c>
       <c r="T174" t="inlineStr">
         <is>
-          <t>Which symptom during ATP most likely indicates a control-plane integration problem?</t>
+          <t>Purpose of S1-AP on S1-MME?</t>
         </is>
       </c>
       <c r="U174" t="inlineStr">
         <is>
-          <t>Which aspect is most important during CMG onboarding?</t>
+          <t>Attach succeeds but bearer fails. Likely issue?</t>
         </is>
       </c>
       <c r="V174" t="inlineStr">
         <is>
-          <t>CMG supports evolution toward which major core direction?</t>
+          <t>Which CMM component is responsible for OAM functions and northbound interfaces?</t>
         </is>
       </c>
       <c r="W174" t="inlineStr">
         <is>
-          <t>In onboarding, which item is usually validated first?</t>
+          <t>Attach ok but PDN fails. Check?</t>
         </is>
       </c>
       <c r="X174" t="inlineStr">
         <is>
-          <t>What is a practical ATP objective for CMG interworking?</t>
+          <t>Which Nokia platform is commonly used for CMM management?</t>
         </is>
       </c>
       <c r="Y174" t="inlineStr">
         <is>
-          <t>Which is a common integration point for CMG in EPC?</t>
+          <t>In 4G LTE, CMM most commonly provides which network function?</t>
         </is>
       </c>
       <c r="Z174" t="inlineStr">
         <is>
-          <t>Which statement best reflects CMG architecture?</t>
+          <t>Which technology is highlighted in CMM for performance optimization on x86 platforms?</t>
         </is>
       </c>
       <c r="AA174" t="inlineStr">
         <is>
-          <t>Which ATP check best confirms attach-related functionality?</t>
+          <t>Which interface is key for LTE access during ATP?</t>
         </is>
       </c>
       <c r="AB174" t="inlineStr">
         <is>
-          <t>What is a major functional benefit of CMG in packet core?</t>
+          <t>What does NECC stand for in Nokia CMM architecture?</t>
         </is>
       </c>
       <c r="AC174" t="inlineStr">
         <is>
-          <t>CMG is best described as:</t>
+          <t>Best failover ATP test?</t>
         </is>
       </c>
       <c r="AD174" t="inlineStr">
         <is>
-          <t>What is the primary role of Nokia Cloud Mobile Gateway (CMG) in packet core?</t>
+          <t>Which protocols relate to CMM control plane?</t>
         </is>
       </c>
       <c r="AE174" t="inlineStr">
         <is>
-          <t>Which ATP case is useful for validating CMG resilience?</t>
+          <t>Successful ATP indication?</t>
         </is>
       </c>
       <c r="AF174" t="inlineStr">
         <is>
-          <t>What is the key purpose of ATP testing for CMG?</t>
+          <t>CMM is described by Nokia as having what kind of architecture?</t>
         </is>
       </c>
       <c r="AG174" t="inlineStr">
         <is>
-          <t>Which outcome indicates a successful CMG onboarding and integration cycle?</t>
-        </is>
-      </c>
-      <c r="AH174" t="inlineStr"/>
+          <t>What enables scaling in CMM?</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -29295,7 +29030,6 @@
           <t>Devarapalli Siva Naga Srivalli</t>
         </is>
       </c>
-      <c r="C175" t="inlineStr"/>
       <c r="D175" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -29446,7 +29180,6 @@
           <t>Which ATP case is useful for validating CMG resilience?</t>
         </is>
       </c>
-      <c r="AH175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -29459,7 +29192,6 @@
           <t>Etakaati Chandan Srinivas</t>
         </is>
       </c>
-      <c r="C176" t="inlineStr"/>
       <c r="D176" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -29610,7 +29342,6 @@
           <t>Which scenario best tests CMG under mobility conditions?</t>
         </is>
       </c>
-      <c r="AH176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -29623,7 +29354,6 @@
           <t>Guttula Vaishnavi</t>
         </is>
       </c>
-      <c r="C177" t="inlineStr"/>
       <c r="D177" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -29774,7 +29504,6 @@
           <t>Attach ok but PDN fails. Check?</t>
         </is>
       </c>
-      <c r="AH177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -29787,7 +29516,6 @@
           <t>Hamsa Yaswanth Paul</t>
         </is>
       </c>
-      <c r="C178" t="inlineStr"/>
       <c r="D178" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -29938,7 +29666,6 @@
           <t>In 4G LTE, CMM most commonly provides which network function?</t>
         </is>
       </c>
-      <c r="AH178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -29951,7 +29678,6 @@
           <t>Kasi Nandini</t>
         </is>
       </c>
-      <c r="C179" t="inlineStr"/>
       <c r="D179" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -30102,7 +29828,6 @@
           <t>Attach fails after MME relocation. What is tested?</t>
         </is>
       </c>
-      <c r="AH179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -30115,7 +29840,6 @@
           <t>Lavanya Seerapu</t>
         </is>
       </c>
-      <c r="C180" t="inlineStr"/>
       <c r="D180" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -30266,7 +29990,6 @@
           <t>What is the best description of a Network Function Instance in NRD/SBA context?</t>
         </is>
       </c>
-      <c r="AH180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -30279,7 +30002,6 @@
           <t>Pappala Sai Kishor</t>
         </is>
       </c>
-      <c r="C181" t="inlineStr"/>
       <c r="D181" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -30430,7 +30152,6 @@
           <t>In a CMG ATP plan, which test most directly verifies end-user data service?</t>
         </is>
       </c>
-      <c r="AH181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -30443,7 +30164,6 @@
           <t>Rachabathula Deepthisri</t>
         </is>
       </c>
-      <c r="C182" t="inlineStr"/>
       <c r="D182" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -30594,7 +30314,6 @@
           <t>CMG supports evolution toward which major core direction?</t>
         </is>
       </c>
-      <c r="AH182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -30607,7 +30326,6 @@
           <t>Srujan Palla</t>
         </is>
       </c>
-      <c r="C183" t="inlineStr"/>
       <c r="D183" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -30758,7 +30476,6 @@
           <t>In a 4G ATP scenario, what does successful bearer establishment mainly confirm?</t>
         </is>
       </c>
-      <c r="AH183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -30771,7 +30488,6 @@
           <t>Swetha Konchada</t>
         </is>
       </c>
-      <c r="C184" t="inlineStr"/>
       <c r="D184" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -30922,7 +30638,6 @@
           <t>CMG supports evolution toward which major core direction?</t>
         </is>
       </c>
-      <c r="AH184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -30935,7 +30650,6 @@
           <t>Vivek Singh</t>
         </is>
       </c>
-      <c r="C185" t="inlineStr"/>
       <c r="D185" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -31086,7 +30800,6 @@
           <t>Which is a common integration point for CMG in EPC?</t>
         </is>
       </c>
-      <c r="AH185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -31099,7 +30812,6 @@
           <t>Akshit Sahni</t>
         </is>
       </c>
-      <c r="C186" t="inlineStr"/>
       <c r="D186" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -31250,7 +30962,6 @@
           <t>Which aspect is most important during CMG onboarding?</t>
         </is>
       </c>
-      <c r="AH186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -31263,7 +30974,6 @@
           <t>Abhiram Jagarlamudi</t>
         </is>
       </c>
-      <c r="C187" t="inlineStr"/>
       <c r="D187" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -31414,7 +31124,6 @@
           <t>Why is CMG considered operationally flexible?</t>
         </is>
       </c>
-      <c r="AH187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -31427,7 +31136,6 @@
           <t>Debopriyo Halder</t>
         </is>
       </c>
-      <c r="C188" t="inlineStr"/>
       <c r="D188" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -31578,7 +31286,6 @@
           <t>Which CMM service is associated with user-plane packet processing and data forwarding?</t>
         </is>
       </c>
-      <c r="AH188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -31591,7 +31298,6 @@
           <t>Alok Kumar Nayak</t>
         </is>
       </c>
-      <c r="C189" t="inlineStr"/>
       <c r="D189" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -31742,7 +31448,6 @@
           <t>Which ATP case is useful for validating CMG resilience?</t>
         </is>
       </c>
-      <c r="AH189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -31755,7 +31460,6 @@
           <t>Archit Bagulia</t>
         </is>
       </c>
-      <c r="C190" t="inlineStr"/>
       <c r="D190" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -31906,7 +31610,6 @@
           <t>Which design goal is central to NRD’s cloud-native approach?</t>
         </is>
       </c>
-      <c r="AH190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -31919,7 +31622,6 @@
           <t>Arunkumar Balappa Pattadakall</t>
         </is>
       </c>
-      <c r="C191" t="inlineStr"/>
       <c r="D191" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -32070,7 +31772,6 @@
           <t>Successful ATP indication?</t>
         </is>
       </c>
-      <c r="AH191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -32083,7 +31784,6 @@
           <t>Dewashish Kumar</t>
         </is>
       </c>
-      <c r="C192" t="inlineStr"/>
       <c r="D192" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -32234,7 +31934,6 @@
           <t>Which design goal is central to NRD’s cloud-native approach?</t>
         </is>
       </c>
-      <c r="AH192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -32247,7 +31946,6 @@
           <t>Subhankar Hazra</t>
         </is>
       </c>
-      <c r="C193" t="inlineStr"/>
       <c r="D193" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -32398,7 +32096,6 @@
           <t>Attach fails after MME relocation. What is tested?</t>
         </is>
       </c>
-      <c r="AH193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -32411,7 +32108,6 @@
           <t>Ajay Kumar</t>
         </is>
       </c>
-      <c r="C194" t="inlineStr"/>
       <c r="D194" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -32562,7 +32258,6 @@
           <t>In a 4G ATP scenario, what does successful bearer establishment mainly confirm?</t>
         </is>
       </c>
-      <c r="AH194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -32575,7 +32270,6 @@
           <t>Altamash Ashfaq</t>
         </is>
       </c>
-      <c r="C195" t="inlineStr"/>
       <c r="D195" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -32726,7 +32420,6 @@
           <t>What is the best description of a Network Function Instance in NRD/SBA context?</t>
         </is>
       </c>
-      <c r="AH195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -32739,7 +32432,6 @@
           <t>Preetam Mehta</t>
         </is>
       </c>
-      <c r="C196" t="inlineStr"/>
       <c r="D196" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -32890,7 +32582,6 @@
           <t>Which protocol family is most relevant to CMG integration with EPC nodes?</t>
         </is>
       </c>
-      <c r="AH196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -32903,7 +32594,6 @@
           <t>Guru Prasad</t>
         </is>
       </c>
-      <c r="C197" t="inlineStr"/>
       <c r="D197" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -33054,7 +32744,6 @@
           <t>Which CMM service handles 2G/3G mobility and session management?</t>
         </is>
       </c>
-      <c r="AH197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -33067,7 +32756,6 @@
           <t>Raviraj Dhondiram Chalikwar</t>
         </is>
       </c>
-      <c r="C198" t="inlineStr"/>
       <c r="D198" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -33218,7 +32906,6 @@
           <t>Which protocol style is most aligned with NRD in an SBA environment?</t>
         </is>
       </c>
-      <c r="AH198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -33231,7 +32918,6 @@
           <t>Snehal Mavale</t>
         </is>
       </c>
-      <c r="C199" t="inlineStr"/>
       <c r="D199" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -33382,7 +33068,6 @@
           <t>Which lifecycle operations are associated with NRD CNF management?</t>
         </is>
       </c>
-      <c r="AH199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -33395,7 +33080,6 @@
           <t>Rakshitha K M</t>
         </is>
       </c>
-      <c r="C200" t="inlineStr"/>
       <c r="D200" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -33546,7 +33230,6 @@
           <t>Key onboarding activity for CMM?</t>
         </is>
       </c>
-      <c r="AH200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -33559,7 +33242,6 @@
           <t>Sakshi Srivastava</t>
         </is>
       </c>
-      <c r="C201" t="inlineStr"/>
       <c r="D201" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -33710,7 +33392,6 @@
           <t>Attach ok but PDN fails. Check?</t>
         </is>
       </c>
-      <c r="AH201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -33723,7 +33404,6 @@
           <t>Sukanya</t>
         </is>
       </c>
-      <c r="C202" t="inlineStr"/>
       <c r="D202" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -33874,7 +33554,6 @@
           <t>CMM is described by Nokia as having what kind of architecture?</t>
         </is>
       </c>
-      <c r="AH202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -33887,7 +33566,6 @@
           <t>Vijay Laxman Dhomase</t>
         </is>
       </c>
-      <c r="C203" t="inlineStr"/>
       <c r="D203" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -34038,7 +33716,6 @@
           <t>Which CMM service hosts the MME functions?</t>
         </is>
       </c>
-      <c r="AH203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -34051,7 +33728,6 @@
           <t>Angshuman Sarma</t>
         </is>
       </c>
-      <c r="C204" t="inlineStr"/>
       <c r="D204" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -34202,7 +33878,6 @@
           <t>What is the best description of a Network Function Instance in NRD/SBA context?</t>
         </is>
       </c>
-      <c r="AH204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -34215,7 +33890,6 @@
           <t>Nisha Kailas Mali</t>
         </is>
       </c>
-      <c r="C205" t="inlineStr"/>
       <c r="D205" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -34366,7 +34040,6 @@
           <t>Which is a common integration point for CMG in EPC?</t>
         </is>
       </c>
-      <c r="AH205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -34379,7 +34052,6 @@
           <t>Ravi Ranjan</t>
         </is>
       </c>
-      <c r="C206" t="inlineStr"/>
       <c r="D206" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -34530,7 +34202,6 @@
           <t>In 4G LTE, CMM most commonly provides which network function?</t>
         </is>
       </c>
-      <c r="AH206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -34543,7 +34214,6 @@
           <t>Sarjitkumar Rajyaguru</t>
         </is>
       </c>
-      <c r="C207" t="inlineStr"/>
       <c r="D207" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -34694,7 +34364,6 @@
           <t>Which symptom during ATP most likely indicates a control-plane integration problem?</t>
         </is>
       </c>
-      <c r="AH207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -34707,7 +34376,6 @@
           <t>Ajith V A</t>
         </is>
       </c>
-      <c r="C208" t="inlineStr"/>
       <c r="D208" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -34858,7 +34526,6 @@
           <t>Which CMM component provides logical interface termination for GTP and Diameter?</t>
         </is>
       </c>
-      <c r="AH208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -34871,7 +34538,6 @@
           <t>Sugat Bhalshankar</t>
         </is>
       </c>
-      <c r="C209" t="inlineStr"/>
       <c r="D209" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -35022,7 +34688,6 @@
           <t>Which is most likely to be verified in CMG acceptance for 4G?</t>
         </is>
       </c>
-      <c r="AH209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -35035,7 +34700,6 @@
           <t>Altaf Ahmad</t>
         </is>
       </c>
-      <c r="C210" t="inlineStr"/>
       <c r="D210" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -35186,7 +34850,6 @@
           <t>What is critical to validate for mobility in ATP?</t>
         </is>
       </c>
-      <c r="AH210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -35199,7 +34862,6 @@
           <t>Dhruv Kant Goyal</t>
         </is>
       </c>
-      <c r="C211" t="inlineStr"/>
       <c r="D211" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -35350,7 +35012,6 @@
           <t>Which design goal is central to NRD’s cloud-native approach?</t>
         </is>
       </c>
-      <c r="AH211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -35363,7 +35024,6 @@
           <t>Mohammad Ayyub</t>
         </is>
       </c>
-      <c r="C212" t="inlineStr"/>
       <c r="D212" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -35514,7 +35174,6 @@
           <t>What is the primary role of Nokia Cloud Mobile Gateway (CMG) in packet core?</t>
         </is>
       </c>
-      <c r="AH212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -35527,7 +35186,6 @@
           <t>Vivek Mishra</t>
         </is>
       </c>
-      <c r="C213" t="inlineStr"/>
       <c r="D213" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -35678,7 +35336,6 @@
           <t>Which statement best describes NRD deployment architecture?</t>
         </is>
       </c>
-      <c r="AH213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -35691,7 +35348,6 @@
           <t>Abhishek Kumar Patel</t>
         </is>
       </c>
-      <c r="C214" t="inlineStr"/>
       <c r="D214" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -35842,7 +35498,6 @@
           <t>Key onboarding activity for CMM?</t>
         </is>
       </c>
-      <c r="AH214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -35855,7 +35510,6 @@
           <t>Chandra Sen</t>
         </is>
       </c>
-      <c r="C215" t="inlineStr"/>
       <c r="D215" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -36006,7 +35660,6 @@
           <t>CMG is best described as:</t>
         </is>
       </c>
-      <c r="AH215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -36019,7 +35672,6 @@
           <t>Depankar Kumar</t>
         </is>
       </c>
-      <c r="C216" t="inlineStr"/>
       <c r="D216" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -36170,7 +35822,6 @@
           <t>Which protocol family is most relevant to CMG integration with EPC nodes?</t>
         </is>
       </c>
-      <c r="AH216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -36183,7 +35834,6 @@
           <t>Mohanram G</t>
         </is>
       </c>
-      <c r="C217" t="inlineStr"/>
       <c r="D217" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -36334,7 +35984,6 @@
           <t>Which statement best reflects CMG architecture?</t>
         </is>
       </c>
-      <c r="AH217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -36347,7 +35996,6 @@
           <t>Manpreet Kaur</t>
         </is>
       </c>
-      <c r="C218" t="inlineStr"/>
       <c r="D218" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -36498,7 +36146,6 @@
           <t>Attach succeeds but bearer fails. Likely issue?</t>
         </is>
       </c>
-      <c r="AH218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -36511,7 +36158,6 @@
           <t>R Timmappa</t>
         </is>
       </c>
-      <c r="C219" t="inlineStr"/>
       <c r="D219" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -36662,7 +36308,6 @@
           <t>Which Nokia platform is commonly used for CMM management?</t>
         </is>
       </c>
-      <c r="AH219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -36675,7 +36320,6 @@
           <t>Smruti Snigdha Sahoo</t>
         </is>
       </c>
-      <c r="C220" t="inlineStr"/>
       <c r="D220" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -36826,7 +36470,6 @@
           <t>In a CMG ATP plan, which test most directly verifies end-user data service?</t>
         </is>
       </c>
-      <c r="AH220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -36839,7 +36482,6 @@
           <t>Tejaswini Patel</t>
         </is>
       </c>
-      <c r="C221" t="inlineStr"/>
       <c r="D221" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -36990,7 +36632,6 @@
           <t>Which ATP case is useful for validating CMG resilience?</t>
         </is>
       </c>
-      <c r="AH221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -37003,7 +36644,6 @@
           <t>Amit Ravindra Ghadge</t>
         </is>
       </c>
-      <c r="C222" t="inlineStr"/>
       <c r="D222" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -37154,7 +36794,6 @@
           <t>Which scenario best tests CMG under mobility conditions?</t>
         </is>
       </c>
-      <c r="AH222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -37167,7 +36806,6 @@
           <t>Sayanth A V</t>
         </is>
       </c>
-      <c r="C223" t="inlineStr"/>
       <c r="D223" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -37318,7 +36956,6 @@
           <t>CMM supports which management interfaces for operations and troubleshooting?</t>
         </is>
       </c>
-      <c r="AH223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -37331,7 +36968,6 @@
           <t>Abhishek Kumar</t>
         </is>
       </c>
-      <c r="C224" t="inlineStr"/>
       <c r="D224" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -37482,7 +37118,6 @@
           <t>Which aspect is most important during CMG onboarding?</t>
         </is>
       </c>
-      <c r="AH224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -37495,7 +37130,6 @@
           <t>Avinash Yadav</t>
         </is>
       </c>
-      <c r="C225" t="inlineStr"/>
       <c r="D225" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -37646,7 +37280,6 @@
           <t>Attach ok but PDN fails. Check?</t>
         </is>
       </c>
-      <c r="AH225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -37659,7 +37292,6 @@
           <t>Mohammad Ali Ahmed Jameel</t>
         </is>
       </c>
-      <c r="C226" t="inlineStr"/>
       <c r="D226" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -37810,7 +37442,6 @@
           <t>CMG is best described as:</t>
         </is>
       </c>
-      <c r="AH226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -37823,7 +37454,6 @@
           <t>Mohammad Mohasin Khan</t>
         </is>
       </c>
-      <c r="C227" t="inlineStr"/>
       <c r="D227" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -37974,7 +37604,6 @@
           <t>Attach fails after MME relocation. What is tested?</t>
         </is>
       </c>
-      <c r="AH227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -37987,7 +37616,6 @@
           <t>Naredla Nirosha</t>
         </is>
       </c>
-      <c r="C228" t="inlineStr"/>
       <c r="D228" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -38138,7 +37766,6 @@
           <t>What is a major functional benefit of CMG in packet core?</t>
         </is>
       </c>
-      <c r="AH228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -38151,7 +37778,6 @@
           <t>Sachin P Gilbile</t>
         </is>
       </c>
-      <c r="C229" t="inlineStr"/>
       <c r="D229" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -38302,7 +37928,6 @@
           <t>CMG is best described as:</t>
         </is>
       </c>
-      <c r="AH229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -38315,7 +37940,6 @@
           <t>Liji Babu</t>
         </is>
       </c>
-      <c r="C230" t="inlineStr"/>
       <c r="D230" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -38466,7 +38090,6 @@
           <t>CMM supports which management interfaces for operations and troubleshooting?</t>
         </is>
       </c>
-      <c r="AH230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -38479,7 +38102,6 @@
           <t>Arvind Kumar Singh</t>
         </is>
       </c>
-      <c r="C231" t="inlineStr"/>
       <c r="D231" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -38630,7 +38252,6 @@
           <t>Successful ATP indication?</t>
         </is>
       </c>
-      <c r="AH231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -38643,7 +38264,6 @@
           <t>Aparajita Shankar</t>
         </is>
       </c>
-      <c r="C232" t="inlineStr"/>
       <c r="D232" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -38794,7 +38414,6 @@
           <t>What is the best description of a Network Function Instance in NRD/SBA context?</t>
         </is>
       </c>
-      <c r="AH232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -38807,7 +38426,6 @@
           <t>Phani Shree</t>
         </is>
       </c>
-      <c r="C233" t="inlineStr"/>
       <c r="D233" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -38958,7 +38576,6 @@
           <t>Attach fails for specific IMSI range. Cause?</t>
         </is>
       </c>
-      <c r="AH233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -38971,7 +38588,6 @@
           <t>S Mohankumar</t>
         </is>
       </c>
-      <c r="C234" t="inlineStr"/>
       <c r="D234" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -39122,7 +38738,6 @@
           <t>In onboarding, which item is usually validated first?</t>
         </is>
       </c>
-      <c r="AH234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -39135,7 +38750,6 @@
           <t>Manojkannan</t>
         </is>
       </c>
-      <c r="C235" t="inlineStr"/>
       <c r="D235" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -39286,7 +38900,6 @@
           <t>If attach succeeds but data service fails, which CMG area should be checked first?</t>
         </is>
       </c>
-      <c r="AH235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -39299,7 +38912,6 @@
           <t>Srivani Supraja</t>
         </is>
       </c>
-      <c r="C236" t="inlineStr"/>
       <c r="D236" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -39450,7 +39062,6 @@
           <t>CMM is described by Nokia as having what kind of architecture?</t>
         </is>
       </c>
-      <c r="AH236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -39463,7 +39074,6 @@
           <t>Nutan Rani</t>
         </is>
       </c>
-      <c r="C237" t="inlineStr"/>
       <c r="D237" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -39614,7 +39224,6 @@
           <t>First ATP validation step should be?</t>
         </is>
       </c>
-      <c r="AH237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -39627,7 +39236,6 @@
           <t>Prasanth S</t>
         </is>
       </c>
-      <c r="C238" t="inlineStr"/>
       <c r="D238" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -39778,7 +39386,6 @@
           <t>Which aspect is most important during CMG onboarding?</t>
         </is>
       </c>
-      <c r="AH238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -39791,7 +39398,6 @@
           <t>Pankaj Verma</t>
         </is>
       </c>
-      <c r="C239" t="inlineStr"/>
       <c r="D239" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -39942,7 +39548,6 @@
           <t>Which protocol family is most relevant to CMG integration with EPC nodes?</t>
         </is>
       </c>
-      <c r="AH239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -39955,7 +39560,6 @@
           <t>Madhura Atul Kulkarni</t>
         </is>
       </c>
-      <c r="C240" t="inlineStr"/>
       <c r="D240" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -40106,7 +39710,6 @@
           <t>Which interface is key for LTE access during ATP?</t>
         </is>
       </c>
-      <c r="AH240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -40119,7 +39722,6 @@
           <t>Sahil Mantrao</t>
         </is>
       </c>
-      <c r="C241" t="inlineStr"/>
       <c r="D241" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -40270,7 +39872,6 @@
           <t>What is the primary role of Nokia Cloud Mobility Manager (CMM) in a 4G packet core?</t>
         </is>
       </c>
-      <c r="AH241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -40283,7 +39884,6 @@
           <t>Satish Maurya</t>
         </is>
       </c>
-      <c r="C242" t="inlineStr"/>
       <c r="D242" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -40434,7 +40034,6 @@
           <t>If attach succeeds but data service fails, which CMG area should be checked first?</t>
         </is>
       </c>
-      <c r="AH242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -40447,7 +40046,6 @@
           <t>Janardan Singh</t>
         </is>
       </c>
-      <c r="C243" t="inlineStr"/>
       <c r="D243" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -40598,7 +40196,6 @@
           <t>CMM is described by Nokia as having what kind of architecture?</t>
         </is>
       </c>
-      <c r="AH243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -40611,7 +40208,6 @@
           <t>Kushagra Chaudhary</t>
         </is>
       </c>
-      <c r="C244" t="inlineStr"/>
       <c r="D244" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -40762,7 +40358,6 @@
           <t>Which ATP case is useful for validating CMG resilience?</t>
         </is>
       </c>
-      <c r="AH244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -40775,7 +40370,6 @@
           <t>Ayan Kumar Roy</t>
         </is>
       </c>
-      <c r="C245" t="inlineStr"/>
       <c r="D245" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -40926,7 +40520,6 @@
           <t>Which is a common integration point for CMG in EPC?</t>
         </is>
       </c>
-      <c r="AH245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -40939,7 +40532,6 @@
           <t>Yashi Gupta</t>
         </is>
       </c>
-      <c r="C246" t="inlineStr"/>
       <c r="D246" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -41090,7 +40682,6 @@
           <t>Best failover ATP test?</t>
         </is>
       </c>
-      <c r="AH246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -41103,7 +40694,6 @@
           <t>Anita KM</t>
         </is>
       </c>
-      <c r="C247" t="inlineStr"/>
       <c r="D247" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -41254,7 +40844,6 @@
           <t>Attach fails after MME relocation. What is tested?</t>
         </is>
       </c>
-      <c r="AH247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -41267,7 +40856,6 @@
           <t>Nitesh Kumar</t>
         </is>
       </c>
-      <c r="C248" t="inlineStr"/>
       <c r="D248" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -41418,7 +41006,6 @@
           <t>In 4G EPC, CMG is most closely associated with which gateway role?</t>
         </is>
       </c>
-      <c r="AH248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -41431,7 +41018,6 @@
           <t>Pratibha Singh</t>
         </is>
       </c>
-      <c r="C249" t="inlineStr"/>
       <c r="D249" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -41582,7 +41168,6 @@
           <t>Which ATP check best confirms attach-related functionality?</t>
         </is>
       </c>
-      <c r="AH249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -41595,7 +41180,6 @@
           <t>Neha Ojha</t>
         </is>
       </c>
-      <c r="C250" t="inlineStr"/>
       <c r="D250" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -41746,7 +41330,6 @@
           <t>If attach succeeds but data service fails, which CMG area should be checked first?</t>
         </is>
       </c>
-      <c r="AH250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -41759,7 +41342,6 @@
           <t>P Vishnu</t>
         </is>
       </c>
-      <c r="C251" t="inlineStr"/>
       <c r="D251" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -41910,7 +41492,6 @@
           <t>Which ATP outcome best confirms correct NRD functionality?</t>
         </is>
       </c>
-      <c r="AH251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -41923,7 +41504,6 @@
           <t>khusboo Mantoo</t>
         </is>
       </c>
-      <c r="C252" t="inlineStr"/>
       <c r="D252" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -42074,7 +41654,6 @@
           <t>In 4G EPC, CMG is most closely associated with which gateway role?</t>
         </is>
       </c>
-      <c r="AH252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -42087,7 +41666,6 @@
           <t>Shridhar Patange</t>
         </is>
       </c>
-      <c r="C253" t="inlineStr"/>
       <c r="D253" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -42238,7 +41816,6 @@
           <t>What is the primary role of Nokia Cloud Mobile Gateway (CMG) in packet core?</t>
         </is>
       </c>
-      <c r="AH253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -42251,7 +41828,6 @@
           <t>Vishal Chaudhary</t>
         </is>
       </c>
-      <c r="C254" t="inlineStr"/>
       <c r="D254" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -42402,7 +41978,6 @@
           <t>NRD implements which kind of services?</t>
         </is>
       </c>
-      <c r="AH254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -42415,7 +41990,6 @@
           <t>Niteesh Pandey</t>
         </is>
       </c>
-      <c r="C255" t="inlineStr"/>
       <c r="D255" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -42566,7 +42140,6 @@
           <t>Which outcome indicates a successful CMG onboarding and integration cycle?</t>
         </is>
       </c>
-      <c r="AH255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -42579,7 +42152,6 @@
           <t>Akanksha Haste</t>
         </is>
       </c>
-      <c r="C256" t="inlineStr"/>
       <c r="D256" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -42730,7 +42302,6 @@
           <t>In onboarding, which item is usually validated first?</t>
         </is>
       </c>
-      <c r="AH256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -42743,7 +42314,6 @@
           <t>Abdullah Ahmed</t>
         </is>
       </c>
-      <c r="C257" t="inlineStr"/>
       <c r="D257" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -42894,7 +42464,6 @@
           <t>In a 4G ATP scenario, what does successful bearer establishment mainly confirm?</t>
         </is>
       </c>
-      <c r="AH257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -42907,7 +42476,6 @@
           <t>Devendra Pratap Gupta</t>
         </is>
       </c>
-      <c r="C258" t="inlineStr"/>
       <c r="D258" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -43058,7 +42626,6 @@
           <t>Which aspect is most important during CMG onboarding?</t>
         </is>
       </c>
-      <c r="AH258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -43071,7 +42638,6 @@
           <t>Mukkollu Nagababu</t>
         </is>
       </c>
-      <c r="C259" t="inlineStr"/>
       <c r="D259" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -43222,7 +42788,6 @@
           <t>Which is a common integration point for CMG in EPC?</t>
         </is>
       </c>
-      <c r="AH259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -43235,7 +42800,6 @@
           <t>Divyanshu Vikram Bhadouria</t>
         </is>
       </c>
-      <c r="C260" t="inlineStr"/>
       <c r="D260" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -43386,7 +42950,6 @@
           <t>What is a practical ATP objective for CMG interworking?</t>
         </is>
       </c>
-      <c r="AH260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -43399,7 +42962,6 @@
           <t>Harshraj Sharma</t>
         </is>
       </c>
-      <c r="C261" t="inlineStr"/>
       <c r="D261" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -43550,7 +43112,6 @@
           <t>What is a practical ATP objective for CMG interworking?</t>
         </is>
       </c>
-      <c r="AH261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -43563,7 +43124,6 @@
           <t>Deepak Kumar Sharma</t>
         </is>
       </c>
-      <c r="C262" t="inlineStr"/>
       <c r="D262" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -43714,7 +43274,6 @@
           <t>In 4G EPC, CMG is most closely associated with which gateway role?</t>
         </is>
       </c>
-      <c r="AH262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -43727,7 +43286,6 @@
           <t>Anand Kumar</t>
         </is>
       </c>
-      <c r="C263" t="inlineStr"/>
       <c r="D263" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -43878,7 +43436,6 @@
           <t>Which is a common integration point for CMG in EPC?</t>
         </is>
       </c>
-      <c r="AH263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -43891,7 +43448,6 @@
           <t>Priya  M</t>
         </is>
       </c>
-      <c r="C264" t="inlineStr"/>
       <c r="D264" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -44042,7 +43598,6 @@
           <t>Which ATP check best confirms attach-related functionality?</t>
         </is>
       </c>
-      <c r="AH264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -44055,7 +43610,6 @@
           <t>Navyasri Neelapu</t>
         </is>
       </c>
-      <c r="C265" t="inlineStr"/>
       <c r="D265" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -44206,7 +43760,6 @@
           <t>CMG is best described as:</t>
         </is>
       </c>
-      <c r="AH265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -44219,7 +43772,6 @@
           <t>Deepika  S</t>
         </is>
       </c>
-      <c r="C266" t="inlineStr"/>
       <c r="D266" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -44370,7 +43922,6 @@
           <t>CMG can support which access evolution model?</t>
         </is>
       </c>
-      <c r="AH266" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>